<commit_message>
Actualizacion: monitoreo integrado en SPA, corregido loader turno, busqueda con acentos, reordenamiento de modulos y regeneracion de documentacion
</commit_message>
<xml_diff>
--- a/Horario/Horario 2026.xlsx
+++ b/Horario/Horario 2026.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Maria Alejandra\Downloads\Pagina Web de Riesgo VS\Horario\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{155C489B-A603-49D9-81E7-222D9BA7A249}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9D16BB9E-340D-4BDB-B5ED-422BF14398D6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{9AAEFA76-0198-46F6-BBF5-EADAB38A6758}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{9AAEFA76-0198-46F6-BBF5-EADAB38A6758}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="517" uniqueCount="26">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="605" uniqueCount="26">
   <si>
     <t>GESTOR</t>
   </si>
@@ -658,16 +658,16 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4B1D5CB7-A214-4F9F-A075-10C6E5CC7E55}">
-  <dimension ref="A1:O64"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <dimension ref="A1:O77"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="19.5546875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="19.5703125" bestFit="1" customWidth="1"/>
     <col min="2" max="6" width="12" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="17" bestFit="1" customWidth="1"/>
     <col min="8" max="15" width="12" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:15" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A1" s="11" t="s">
         <v>0</v>
       </c>
@@ -714,7 +714,7 @@
         <v>46138</v>
       </c>
     </row>
-    <row r="2" spans="1:15" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A2" s="12"/>
       <c r="B2" s="2" t="s">
         <v>1</v>
@@ -759,7 +759,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="3" spans="1:15" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
         <v>8</v>
       </c>
@@ -806,7 +806,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="4" spans="1:15" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A4" s="3" t="s">
         <v>12</v>
       </c>
@@ -853,7 +853,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="5" spans="1:15" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A5" s="3" t="s">
         <v>14</v>
       </c>
@@ -900,7 +900,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="6" spans="1:15" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A6" s="3" t="s">
         <v>15</v>
       </c>
@@ -947,7 +947,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="7" spans="1:15" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A7" s="3" t="s">
         <v>17</v>
       </c>
@@ -994,7 +994,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="8" spans="1:15" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A8" s="3" t="s">
         <v>18</v>
       </c>
@@ -1041,7 +1041,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="9" spans="1:15" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A9" s="3" t="s">
         <v>20</v>
       </c>
@@ -1088,7 +1088,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="10" spans="1:15" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A10" s="3" t="s">
         <v>21</v>
       </c>
@@ -1135,7 +1135,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="11" spans="1:15" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A11" s="3" t="s">
         <v>22</v>
       </c>
@@ -1182,7 +1182,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="12" spans="1:15" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A12" s="3" t="s">
         <v>23</v>
       </c>
@@ -1229,7 +1229,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="14" spans="1:15" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A14" s="11" t="s">
         <v>0</v>
       </c>
@@ -1255,7 +1255,7 @@
         <v>46145</v>
       </c>
     </row>
-    <row r="15" spans="1:15" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A15" s="12"/>
       <c r="B15" s="2" t="s">
         <v>1</v>
@@ -1279,7 +1279,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="16" spans="1:15" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A16" s="3" t="s">
         <v>17</v>
       </c>
@@ -1305,7 +1305,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="17" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A17" s="3" t="s">
         <v>8</v>
       </c>
@@ -1331,7 +1331,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="18" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A18" s="3" t="s">
         <v>12</v>
       </c>
@@ -1357,7 +1357,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="19" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A19" s="3" t="s">
         <v>15</v>
       </c>
@@ -1383,7 +1383,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="20" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A20" s="3" t="s">
         <v>18</v>
       </c>
@@ -1409,7 +1409,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="21" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A21" s="3" t="s">
         <v>23</v>
       </c>
@@ -1435,7 +1435,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="22" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A22" s="3" t="s">
         <v>21</v>
       </c>
@@ -1461,7 +1461,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="23" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A23" s="3" t="s">
         <v>22</v>
       </c>
@@ -1487,7 +1487,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="24" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A24" s="3" t="s">
         <v>14</v>
       </c>
@@ -1513,7 +1513,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="25" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A25" s="3" t="s">
         <v>20</v>
       </c>
@@ -1539,7 +1539,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="27" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A27" s="11" t="s">
         <v>0</v>
       </c>
@@ -1565,7 +1565,7 @@
         <v>46152</v>
       </c>
     </row>
-    <row r="28" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A28" s="12"/>
       <c r="B28" s="2" t="s">
         <v>1</v>
@@ -1589,7 +1589,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="29" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A29" s="3" t="s">
         <v>22</v>
       </c>
@@ -1615,7 +1615,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="30" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A30" s="3" t="s">
         <v>14</v>
       </c>
@@ -1641,7 +1641,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="31" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A31" s="3" t="s">
         <v>20</v>
       </c>
@@ -1667,7 +1667,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="32" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A32" s="3" t="s">
         <v>15</v>
       </c>
@@ -1693,7 +1693,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="33" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A33" s="3" t="s">
         <v>18</v>
       </c>
@@ -1719,7 +1719,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="34" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A34" s="3" t="s">
         <v>21</v>
       </c>
@@ -1745,7 +1745,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="35" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A35" s="3" t="s">
         <v>8</v>
       </c>
@@ -1771,7 +1771,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="36" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A36" s="3" t="s">
         <v>12</v>
       </c>
@@ -1797,7 +1797,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="37" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A37" s="3" t="s">
         <v>23</v>
       </c>
@@ -1823,7 +1823,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="38" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A38" s="3" t="s">
         <v>17</v>
       </c>
@@ -1849,7 +1849,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="40" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A40" s="13" t="s">
         <v>0</v>
       </c>
@@ -1875,7 +1875,7 @@
         <v>46159</v>
       </c>
     </row>
-    <row r="41" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A41" s="13"/>
       <c r="B41" s="2" t="s">
         <v>1</v>
@@ -1899,7 +1899,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="42" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A42" s="3" t="s">
         <v>22</v>
       </c>
@@ -1925,7 +1925,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="43" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A43" s="3" t="s">
         <v>12</v>
       </c>
@@ -1951,7 +1951,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="44" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A44" s="3" t="s">
         <v>18</v>
       </c>
@@ -1977,7 +1977,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="45" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A45" s="3" t="s">
         <v>23</v>
       </c>
@@ -2003,7 +2003,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="46" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A46" s="3" t="s">
         <v>15</v>
       </c>
@@ -2029,7 +2029,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="47" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A47" s="3" t="s">
         <v>24</v>
       </c>
@@ -2055,7 +2055,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="48" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A48" s="3" t="s">
         <v>14</v>
       </c>
@@ -2081,7 +2081,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="49" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A49" s="3" t="s">
         <v>21</v>
       </c>
@@ -2107,7 +2107,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="50" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="50" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A50" s="3" t="s">
         <v>20</v>
       </c>
@@ -2133,7 +2133,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="51" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="51" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A51" s="3" t="s">
         <v>8</v>
       </c>
@@ -2159,7 +2159,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="53" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="53" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A53" s="13" t="s">
         <v>0</v>
       </c>
@@ -2185,7 +2185,7 @@
         <v>46166</v>
       </c>
     </row>
-    <row r="54" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="54" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A54" s="13"/>
       <c r="B54" s="2" t="s">
         <v>1</v>
@@ -2209,7 +2209,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="55" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="55" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A55" s="3" t="s">
         <v>22</v>
       </c>
@@ -2235,7 +2235,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="56" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="56" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A56" s="3" t="s">
         <v>14</v>
       </c>
@@ -2261,7 +2261,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="57" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="57" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A57" s="3" t="s">
         <v>17</v>
       </c>
@@ -2287,7 +2287,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="58" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="58" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A58" s="3" t="s">
         <v>18</v>
       </c>
@@ -2313,7 +2313,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="59" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="59" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A59" s="3" t="s">
         <v>23</v>
       </c>
@@ -2339,7 +2339,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="60" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="60" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A60" s="3" t="s">
         <v>21</v>
       </c>
@@ -2365,7 +2365,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="61" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="61" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A61" s="3" t="s">
         <v>8</v>
       </c>
@@ -2391,7 +2391,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="62" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="62" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A62" s="3" t="s">
         <v>12</v>
       </c>
@@ -2417,7 +2417,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="63" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="63" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A63" s="3" t="s">
         <v>20</v>
       </c>
@@ -2443,7 +2443,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="64" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="64" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A64" s="3" t="s">
         <v>15</v>
       </c>
@@ -2469,8 +2469,319 @@
         <v>19</v>
       </c>
     </row>
+    <row r="66" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A66" s="13" t="s">
+        <v>0</v>
+      </c>
+      <c r="B66" s="1">
+        <v>46167</v>
+      </c>
+      <c r="C66" s="1">
+        <v>46168</v>
+      </c>
+      <c r="D66" s="1">
+        <v>46169</v>
+      </c>
+      <c r="E66" s="1">
+        <v>46170</v>
+      </c>
+      <c r="F66" s="1">
+        <v>46171</v>
+      </c>
+      <c r="G66" s="1">
+        <v>46172</v>
+      </c>
+      <c r="H66" s="1">
+        <v>46173</v>
+      </c>
+    </row>
+    <row r="67" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A67" s="13"/>
+      <c r="B67" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C67" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="D67" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="E67" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="F67" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="G67" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="H67" s="2" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="68" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A68" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="B68" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C68" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="D68" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="E68" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="F68" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="G68" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="H68" s="4" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="69" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A69" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="B69" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C69" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="D69" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="E69" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="F69" s="10" t="s">
+        <v>25</v>
+      </c>
+      <c r="G69" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="H69" s="5" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="70" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A70" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="B70" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C70" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="D70" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="E70" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="F70" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="G70" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="H70" s="5" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="71" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A71" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="B71" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C71" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="D71" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="E71" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="F71" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="G71" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="H71" s="5" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="72" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A72" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="B72" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C72" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="D72" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="E72" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="F72" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="G72" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="H72" s="4" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="73" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A73" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="B73" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C73" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="D73" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="E73" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="F73" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="G73" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="H73" s="5" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="74" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A74" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="B74" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="C74" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="D74" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="E74" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="F74" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="G74" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="H74" s="4" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="75" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A75" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="B75" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="C75" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="D75" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="E75" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="F75" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="G75" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="H75" s="4" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="76" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A76" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="B76" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="C76" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="D76" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="E76" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="F76" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="G76" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="H76" s="4" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="77" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A77" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="B77" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="C77" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="D77" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="E77" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="F77" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="G77" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="H77" s="5" t="s">
+        <v>10</v>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="5">
+  <mergeCells count="6">
+    <mergeCell ref="A66:A67"/>
     <mergeCell ref="A1:A2"/>
     <mergeCell ref="A14:A15"/>
     <mergeCell ref="A27:A28"/>
@@ -2483,17 +2794,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="9d4e7416-6feb-444a-9f0d-6e119e2a4ded">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="ab20b492-db1c-4b70-84db-283da62d5dcb" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100A49D20B196870C459C080BD3A88F41F5" ma:contentTypeVersion="12" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="c891d3af3c5d8789d4a1386f5525110a">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="9d4e7416-6feb-444a-9f0d-6e119e2a4ded" xmlns:ns3="ab20b492-db1c-4b70-84db-283da62d5dcb" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="a2d778173b158e0f4887e6c1a7be78b9" ns2:_="" ns3:_="">
     <xsd:import namespace="9d4e7416-6feb-444a-9f0d-6e119e2a4ded"/>
@@ -2694,6 +2994,17 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="9d4e7416-6feb-444a-9f0d-6e119e2a4ded">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="ab20b492-db1c-4b70-84db-283da62d5dcb" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
 <FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
@@ -2704,17 +3015,6 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{3E7BE3CC-8834-4B2B-B0A5-EDC239DF005F}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="9d4e7416-6feb-444a-9f0d-6e119e2a4ded"/>
-    <ds:schemaRef ds:uri="ab20b492-db1c-4b70-84db-283da62d5dcb"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9D90F563-717D-4F15-9FD2-892B1218D415}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -2733,6 +3033,17 @@
 </ds:datastoreItem>
 </file>
 
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{3E7BE3CC-8834-4B2B-B0A5-EDC239DF005F}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="9d4e7416-6feb-444a-9f0d-6e119e2a4ded"/>
+    <ds:schemaRef ds:uri="ab20b492-db1c-4b70-84db-283da62d5dcb"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{3E90FB8C-E259-434B-8A97-2530AD5FA4BD}">
   <ds:schemaRefs>

</xml_diff>

<commit_message>
Actualizacion automatica de datos - mar 02/06/2026  8:30:44,03
</commit_message>
<xml_diff>
--- a/Horario/Horario 2026.xlsx
+++ b/Horario/Horario 2026.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Maria Alejandra\Downloads\Pagina Web de Riesgo VS\Horario\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://virtualsoftserv-my.sharepoint.com/personal/maria_sanchez_virtualsoft_tech/Documents/Indicadores y Pagina WEB/Horario/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9D16BB9E-340D-4BDB-B5ED-422BF14398D6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="1" documentId="13_ncr:1_{9D16BB9E-340D-4BDB-B5ED-422BF14398D6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{E724598E-DA6A-46A9-9494-576E9250E565}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{9AAEFA76-0198-46F6-BBF5-EADAB38A6758}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="605" uniqueCount="26">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="691" uniqueCount="26">
   <si>
     <t>GESTOR</t>
   </si>
@@ -186,7 +186,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="9">
+  <fills count="10">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -235,8 +235,14 @@
         <bgColor rgb="FF000000"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="2" tint="-9.9978637043366805E-2"/>
+        <bgColor rgb="FF000000"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="4">
+  <borders count="6">
     <border>
       <left/>
       <right/>
@@ -285,12 +291,38 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="16" fontId="2" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -314,14 +346,20 @@
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="4" fillId="9" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="9" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -658,7 +696,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4B1D5CB7-A214-4F9F-A075-10C6E5CC7E55}">
-  <dimension ref="A1:O77"/>
+  <dimension ref="A1:O90"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="19.5703125" bestFit="1" customWidth="1"/>
@@ -668,7 +706,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A1" s="11" t="s">
+      <c r="A1" s="12" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="1">
@@ -715,7 +753,7 @@
       </c>
     </row>
     <row r="2" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A2" s="12"/>
+      <c r="A2" s="13"/>
       <c r="B2" s="2" t="s">
         <v>1</v>
       </c>
@@ -1230,7 +1268,7 @@
       </c>
     </row>
     <row r="14" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A14" s="11" t="s">
+      <c r="A14" s="12" t="s">
         <v>0</v>
       </c>
       <c r="B14" s="1">
@@ -1256,7 +1294,7 @@
       </c>
     </row>
     <row r="15" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A15" s="12"/>
+      <c r="A15" s="13"/>
       <c r="B15" s="2" t="s">
         <v>1</v>
       </c>
@@ -1540,7 +1578,7 @@
       </c>
     </row>
     <row r="27" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A27" s="11" t="s">
+      <c r="A27" s="12" t="s">
         <v>0</v>
       </c>
       <c r="B27" s="1">
@@ -1566,7 +1604,7 @@
       </c>
     </row>
     <row r="28" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A28" s="12"/>
+      <c r="A28" s="13"/>
       <c r="B28" s="2" t="s">
         <v>1</v>
       </c>
@@ -1850,7 +1888,7 @@
       </c>
     </row>
     <row r="40" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A40" s="13" t="s">
+      <c r="A40" s="11" t="s">
         <v>0</v>
       </c>
       <c r="B40" s="1">
@@ -1876,7 +1914,7 @@
       </c>
     </row>
     <row r="41" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A41" s="13"/>
+      <c r="A41" s="11"/>
       <c r="B41" s="2" t="s">
         <v>1</v>
       </c>
@@ -2160,7 +2198,7 @@
       </c>
     </row>
     <row r="53" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A53" s="13" t="s">
+      <c r="A53" s="11" t="s">
         <v>0</v>
       </c>
       <c r="B53" s="1">
@@ -2186,7 +2224,7 @@
       </c>
     </row>
     <row r="54" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A54" s="13"/>
+      <c r="A54" s="11"/>
       <c r="B54" s="2" t="s">
         <v>1</v>
       </c>
@@ -2470,7 +2508,7 @@
       </c>
     </row>
     <row r="66" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A66" s="13" t="s">
+      <c r="A66" s="11" t="s">
         <v>0</v>
       </c>
       <c r="B66" s="1">
@@ -2496,7 +2534,7 @@
       </c>
     </row>
     <row r="67" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A67" s="13"/>
+      <c r="A67" s="11"/>
       <c r="B67" s="2" t="s">
         <v>1</v>
       </c>
@@ -2779,8 +2817,316 @@
         <v>10</v>
       </c>
     </row>
+    <row r="79" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A79" s="11" t="s">
+        <v>0</v>
+      </c>
+      <c r="B79" s="1">
+        <v>46174</v>
+      </c>
+      <c r="C79" s="1">
+        <v>46175</v>
+      </c>
+      <c r="D79" s="1">
+        <v>46176</v>
+      </c>
+      <c r="E79" s="1">
+        <v>46177</v>
+      </c>
+      <c r="F79" s="1">
+        <v>46178</v>
+      </c>
+      <c r="G79" s="1">
+        <v>46179</v>
+      </c>
+      <c r="H79" s="1">
+        <v>46180</v>
+      </c>
+    </row>
+    <row r="80" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A80" s="11"/>
+      <c r="B80" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C80" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="D80" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="E80" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="F80" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="G80" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="H80" s="2" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="81" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A81" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="B81" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C81" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="D81" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="E81" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="F81" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="G81" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="H81" s="4" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="82" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A82" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="B82" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C82" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="D82" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="E82" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="F82" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="G82" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="H82" s="5" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="83" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A83" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="B83" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C83" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="D83" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="E83" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="F83" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="G83" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="H83" s="4" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="84" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A84" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="B84" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C84" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="D84" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="E84" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="F84" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="G84" s="14"/>
+      <c r="H84" s="15"/>
+    </row>
+    <row r="85" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A85" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="B85" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C85" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="D85" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="E85" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="F85" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="G85" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="H85" s="4" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="86" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A86" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="B86" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C86" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="D86" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="E86" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="F86" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="G86" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="H86" s="4" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="87" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A87" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="B87" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="C87" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="D87" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="E87" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="F87" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="G87" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="H87" s="5" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="88" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A88" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="B88" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="C88" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="D88" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="E88" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="F88" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="G88" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="H88" s="5" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="89" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A89" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="B89" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="C89" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="D89" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="E89" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="F89" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="G89" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="H89" s="5" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="90" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A90" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="B90" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="C90" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="D90" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="E90" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="F90" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="G90" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="H90" s="5" t="s">
+        <v>10</v>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="6">
+  <mergeCells count="8">
+    <mergeCell ref="A79:A80"/>
+    <mergeCell ref="G84:H84"/>
     <mergeCell ref="A66:A67"/>
     <mergeCell ref="A1:A2"/>
     <mergeCell ref="A14:A15"/>
@@ -2794,6 +3140,26 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="9d4e7416-6feb-444a-9f0d-6e119e2a4ded">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="ab20b492-db1c-4b70-84db-283da62d5dcb" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100A49D20B196870C459C080BD3A88F41F5" ma:contentTypeVersion="12" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="c891d3af3c5d8789d4a1386f5525110a">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="9d4e7416-6feb-444a-9f0d-6e119e2a4ded" xmlns:ns3="ab20b492-db1c-4b70-84db-283da62d5dcb" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="a2d778173b158e0f4887e6c1a7be78b9" ns2:_="" ns3:_="">
     <xsd:import namespace="9d4e7416-6feb-444a-9f0d-6e119e2a4ded"/>
@@ -2994,27 +3360,26 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="9d4e7416-6feb-444a-9f0d-6e119e2a4ded">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="ab20b492-db1c-4b70-84db-283da62d5dcb" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{3E90FB8C-E259-434B-8A97-2530AD5FA4BD}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{3E7BE3CC-8834-4B2B-B0A5-EDC239DF005F}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="9d4e7416-6feb-444a-9f0d-6e119e2a4ded"/>
+    <ds:schemaRef ds:uri="ab20b492-db1c-4b70-84db-283da62d5dcb"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9D90F563-717D-4F15-9FD2-892B1218D415}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -3031,23 +3396,4 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{3E7BE3CC-8834-4B2B-B0A5-EDC239DF005F}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="9d4e7416-6feb-444a-9f0d-6e119e2a4ded"/>
-    <ds:schemaRef ds:uri="ab20b492-db1c-4b70-84db-283da62d5dcb"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{3E90FB8C-E259-434B-8A97-2530AD5FA4BD}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
Actualizacion automatica de datos - jue 04/06/2026  8:28:07,87
</commit_message>
<xml_diff>
--- a/Horario/Horario 2026.xlsx
+++ b/Horario/Horario 2026.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://virtualsoftserv-my.sharepoint.com/personal/maria_sanchez_virtualsoft_tech/Documents/Indicadores y Pagina WEB/Horario/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="1" documentId="13_ncr:1_{9D16BB9E-340D-4BDB-B5ED-422BF14398D6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{E724598E-DA6A-46A9-9494-576E9250E565}"/>
+  <xr:revisionPtr revIDLastSave="2" documentId="13_ncr:1_{9D16BB9E-340D-4BDB-B5ED-422BF14398D6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{705138F6-F38D-4977-96B2-2ADFBE7B6659}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{9AAEFA76-0198-46F6-BBF5-EADAB38A6758}"/>
+    <workbookView xWindow="1920" yWindow="1920" windowWidth="17280" windowHeight="8880" xr2:uid="{9AAEFA76-0198-46F6-BBF5-EADAB38A6758}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
@@ -349,17 +349,17 @@
     <xf numFmtId="0" fontId="2" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="9" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="9" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="9" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="9" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -697,16 +697,16 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4B1D5CB7-A214-4F9F-A075-10C6E5CC7E55}">
   <dimension ref="A1:O90"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="19.5703125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="19.5546875" bestFit="1" customWidth="1"/>
     <col min="2" max="6" width="12" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="17" bestFit="1" customWidth="1"/>
     <col min="8" max="15" width="12" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A1" s="12" t="s">
+    <row r="1" spans="1:15" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A1" s="14" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="1">
@@ -752,8 +752,8 @@
         <v>46138</v>
       </c>
     </row>
-    <row r="2" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A2" s="13"/>
+    <row r="2" spans="1:15" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A2" s="15"/>
       <c r="B2" s="2" t="s">
         <v>1</v>
       </c>
@@ -797,7 +797,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="3" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:15" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A3" s="3" t="s">
         <v>8</v>
       </c>
@@ -844,7 +844,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="4" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:15" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A4" s="3" t="s">
         <v>12</v>
       </c>
@@ -891,7 +891,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="5" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:15" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A5" s="3" t="s">
         <v>14</v>
       </c>
@@ -938,7 +938,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="6" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:15" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A6" s="3" t="s">
         <v>15</v>
       </c>
@@ -985,7 +985,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="7" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:15" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A7" s="3" t="s">
         <v>17</v>
       </c>
@@ -1032,7 +1032,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="8" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:15" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A8" s="3" t="s">
         <v>18</v>
       </c>
@@ -1079,7 +1079,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="9" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:15" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A9" s="3" t="s">
         <v>20</v>
       </c>
@@ -1126,7 +1126,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="10" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:15" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A10" s="3" t="s">
         <v>21</v>
       </c>
@@ -1173,7 +1173,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="11" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:15" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A11" s="3" t="s">
         <v>22</v>
       </c>
@@ -1220,7 +1220,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="12" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:15" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A12" s="3" t="s">
         <v>23</v>
       </c>
@@ -1267,8 +1267,8 @@
         <v>9</v>
       </c>
     </row>
-    <row r="14" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A14" s="12" t="s">
+    <row r="14" spans="1:15" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A14" s="14" t="s">
         <v>0</v>
       </c>
       <c r="B14" s="1">
@@ -1293,8 +1293,8 @@
         <v>46145</v>
       </c>
     </row>
-    <row r="15" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A15" s="13"/>
+    <row r="15" spans="1:15" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A15" s="15"/>
       <c r="B15" s="2" t="s">
         <v>1</v>
       </c>
@@ -1317,7 +1317,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="16" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:15" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A16" s="3" t="s">
         <v>17</v>
       </c>
@@ -1343,7 +1343,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="17" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A17" s="3" t="s">
         <v>8</v>
       </c>
@@ -1369,7 +1369,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="18" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A18" s="3" t="s">
         <v>12</v>
       </c>
@@ -1395,7 +1395,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="19" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A19" s="3" t="s">
         <v>15</v>
       </c>
@@ -1421,7 +1421,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="20" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A20" s="3" t="s">
         <v>18</v>
       </c>
@@ -1447,7 +1447,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="21" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A21" s="3" t="s">
         <v>23</v>
       </c>
@@ -1473,7 +1473,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="22" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A22" s="3" t="s">
         <v>21</v>
       </c>
@@ -1499,7 +1499,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="23" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A23" s="3" t="s">
         <v>22</v>
       </c>
@@ -1525,7 +1525,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="24" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A24" s="3" t="s">
         <v>14</v>
       </c>
@@ -1551,7 +1551,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="25" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A25" s="3" t="s">
         <v>20</v>
       </c>
@@ -1577,8 +1577,8 @@
         <v>10</v>
       </c>
     </row>
-    <row r="27" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A27" s="12" t="s">
+    <row r="27" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A27" s="14" t="s">
         <v>0</v>
       </c>
       <c r="B27" s="1">
@@ -1603,8 +1603,8 @@
         <v>46152</v>
       </c>
     </row>
-    <row r="28" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A28" s="13"/>
+    <row r="28" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A28" s="15"/>
       <c r="B28" s="2" t="s">
         <v>1</v>
       </c>
@@ -1627,7 +1627,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="29" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A29" s="3" t="s">
         <v>22</v>
       </c>
@@ -1653,7 +1653,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="30" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A30" s="3" t="s">
         <v>14</v>
       </c>
@@ -1679,7 +1679,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="31" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A31" s="3" t="s">
         <v>20</v>
       </c>
@@ -1705,7 +1705,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="32" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A32" s="3" t="s">
         <v>15</v>
       </c>
@@ -1731,7 +1731,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="33" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A33" s="3" t="s">
         <v>18</v>
       </c>
@@ -1757,7 +1757,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="34" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A34" s="3" t="s">
         <v>21</v>
       </c>
@@ -1783,7 +1783,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="35" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A35" s="3" t="s">
         <v>8</v>
       </c>
@@ -1809,7 +1809,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="36" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A36" s="3" t="s">
         <v>12</v>
       </c>
@@ -1835,7 +1835,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="37" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A37" s="3" t="s">
         <v>23</v>
       </c>
@@ -1861,7 +1861,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="38" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A38" s="3" t="s">
         <v>17</v>
       </c>
@@ -1887,7 +1887,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="40" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A40" s="11" t="s">
         <v>0</v>
       </c>
@@ -1913,7 +1913,7 @@
         <v>46159</v>
       </c>
     </row>
-    <row r="41" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A41" s="11"/>
       <c r="B41" s="2" t="s">
         <v>1</v>
@@ -1937,7 +1937,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="42" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A42" s="3" t="s">
         <v>22</v>
       </c>
@@ -1963,7 +1963,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="43" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A43" s="3" t="s">
         <v>12</v>
       </c>
@@ -1989,7 +1989,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="44" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A44" s="3" t="s">
         <v>18</v>
       </c>
@@ -2015,7 +2015,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="45" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A45" s="3" t="s">
         <v>23</v>
       </c>
@@ -2041,7 +2041,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="46" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A46" s="3" t="s">
         <v>15</v>
       </c>
@@ -2067,7 +2067,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="47" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A47" s="3" t="s">
         <v>24</v>
       </c>
@@ -2093,7 +2093,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="48" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A48" s="3" t="s">
         <v>14</v>
       </c>
@@ -2119,7 +2119,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="49" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A49" s="3" t="s">
         <v>21</v>
       </c>
@@ -2145,7 +2145,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="50" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A50" s="3" t="s">
         <v>20</v>
       </c>
@@ -2171,7 +2171,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="51" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A51" s="3" t="s">
         <v>8</v>
       </c>
@@ -2197,7 +2197,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="53" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A53" s="11" t="s">
         <v>0</v>
       </c>
@@ -2223,7 +2223,7 @@
         <v>46166</v>
       </c>
     </row>
-    <row r="54" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A54" s="11"/>
       <c r="B54" s="2" t="s">
         <v>1</v>
@@ -2247,7 +2247,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="55" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A55" s="3" t="s">
         <v>22</v>
       </c>
@@ -2273,7 +2273,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="56" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A56" s="3" t="s">
         <v>14</v>
       </c>
@@ -2299,7 +2299,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="57" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A57" s="3" t="s">
         <v>17</v>
       </c>
@@ -2325,7 +2325,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="58" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A58" s="3" t="s">
         <v>18</v>
       </c>
@@ -2351,7 +2351,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="59" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A59" s="3" t="s">
         <v>23</v>
       </c>
@@ -2377,7 +2377,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="60" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A60" s="3" t="s">
         <v>21</v>
       </c>
@@ -2403,7 +2403,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="61" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A61" s="3" t="s">
         <v>8</v>
       </c>
@@ -2429,7 +2429,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="62" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A62" s="3" t="s">
         <v>12</v>
       </c>
@@ -2455,7 +2455,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="63" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A63" s="3" t="s">
         <v>20</v>
       </c>
@@ -2481,7 +2481,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="64" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A64" s="3" t="s">
         <v>15</v>
       </c>
@@ -2507,7 +2507,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="66" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A66" s="11" t="s">
         <v>0</v>
       </c>
@@ -2533,7 +2533,7 @@
         <v>46173</v>
       </c>
     </row>
-    <row r="67" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A67" s="11"/>
       <c r="B67" s="2" t="s">
         <v>1</v>
@@ -2557,7 +2557,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="68" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A68" s="3" t="s">
         <v>22</v>
       </c>
@@ -2583,7 +2583,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="69" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A69" s="3" t="s">
         <v>21</v>
       </c>
@@ -2609,7 +2609,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="70" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A70" s="3" t="s">
         <v>8</v>
       </c>
@@ -2635,7 +2635,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="71" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A71" s="3" t="s">
         <v>18</v>
       </c>
@@ -2661,7 +2661,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="72" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A72" s="3" t="s">
         <v>20</v>
       </c>
@@ -2687,7 +2687,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="73" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="73" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A73" s="3" t="s">
         <v>15</v>
       </c>
@@ -2713,7 +2713,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="74" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="74" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A74" s="3" t="s">
         <v>14</v>
       </c>
@@ -2739,7 +2739,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="75" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="75" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A75" s="3" t="s">
         <v>17</v>
       </c>
@@ -2765,7 +2765,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="76" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="76" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A76" s="3" t="s">
         <v>23</v>
       </c>
@@ -2791,7 +2791,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="77" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="77" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A77" s="3" t="s">
         <v>12</v>
       </c>
@@ -2817,7 +2817,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="79" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="79" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A79" s="11" t="s">
         <v>0</v>
       </c>
@@ -2843,7 +2843,7 @@
         <v>46180</v>
       </c>
     </row>
-    <row r="80" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="80" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A80" s="11"/>
       <c r="B80" s="2" t="s">
         <v>1</v>
@@ -2867,7 +2867,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="81" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="81" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A81" s="3" t="s">
         <v>22</v>
       </c>
@@ -2893,7 +2893,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="82" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="82" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A82" s="3" t="s">
         <v>14</v>
       </c>
@@ -2919,7 +2919,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="83" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="83" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A83" s="3" t="s">
         <v>12</v>
       </c>
@@ -2935,8 +2935,8 @@
       <c r="E83" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="F83" s="4" t="s">
-        <v>9</v>
+      <c r="F83" s="10" t="s">
+        <v>25</v>
       </c>
       <c r="G83" s="5" t="s">
         <v>10</v>
@@ -2945,7 +2945,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="84" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="84" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A84" s="3" t="s">
         <v>15</v>
       </c>
@@ -2964,10 +2964,10 @@
       <c r="F84" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="G84" s="14"/>
-      <c r="H84" s="15"/>
-    </row>
-    <row r="85" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="G84" s="12"/>
+      <c r="H84" s="13"/>
+    </row>
+    <row r="85" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A85" s="3" t="s">
         <v>17</v>
       </c>
@@ -2993,7 +2993,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="86" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="86" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A86" s="3" t="s">
         <v>18</v>
       </c>
@@ -3019,7 +3019,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="87" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="87" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A87" s="3" t="s">
         <v>21</v>
       </c>
@@ -3045,7 +3045,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="88" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="88" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A88" s="3" t="s">
         <v>8</v>
       </c>
@@ -3071,7 +3071,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="89" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="89" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A89" s="3" t="s">
         <v>20</v>
       </c>
@@ -3097,7 +3097,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="90" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="90" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A90" s="3" t="s">
         <v>23</v>
       </c>
@@ -3140,15 +3140,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
     <lcf76f155ced4ddcb4097134ff3c332f xmlns="9d4e7416-6feb-444a-9f0d-6e119e2a4ded">
@@ -3157,6 +3148,15 @@
     <TaxCatchAll xmlns="ab20b492-db1c-4b70-84db-283da62d5dcb" xsi:nil="true"/>
   </documentManagement>
 </p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
@@ -3361,20 +3361,20 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{3E90FB8C-E259-434B-8A97-2530AD5FA4BD}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{3E7BE3CC-8834-4B2B-B0A5-EDC239DF005F}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
     <ds:schemaRef ds:uri="9d4e7416-6feb-444a-9f0d-6e119e2a4ded"/>
     <ds:schemaRef ds:uri="ab20b492-db1c-4b70-84db-283da62d5dcb"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{3E90FB8C-E259-434B-8A97-2530AD5FA4BD}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>

</xml_diff>

<commit_message>
Actualizacion automatica de datos - vie 12/06/2026 12:47:31,82
</commit_message>
<xml_diff>
--- a/Horario/Horario 2026.xlsx
+++ b/Horario/Horario 2026.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://virtualsoftserv-my.sharepoint.com/personal/maria_sanchez_virtualsoft_tech/Documents/Indicadores y Pagina WEB/Horario/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="3" documentId="13_ncr:1_{9D16BB9E-340D-4BDB-B5ED-422BF14398D6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{BAD4FFD9-4F4D-41E9-894C-DCFE18A56FA3}"/>
+  <xr:revisionPtr revIDLastSave="4" documentId="13_ncr:1_{9D16BB9E-340D-4BDB-B5ED-422BF14398D6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{BDBDBEEF-DC36-48C1-B3C7-7D4C7FB3AC40}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{9AAEFA76-0198-46F6-BBF5-EADAB38A6758}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{9AAEFA76-0198-46F6-BBF5-EADAB38A6758}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="771" uniqueCount="26">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="851" uniqueCount="26">
   <si>
     <t>GESTOR</t>
   </si>
@@ -696,16 +696,16 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4B1D5CB7-A214-4F9F-A075-10C6E5CC7E55}">
-  <dimension ref="A1:O102"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <dimension ref="A1:O114"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="19.5546875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="19.5703125" bestFit="1" customWidth="1"/>
     <col min="2" max="6" width="12" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="17" bestFit="1" customWidth="1"/>
     <col min="8" max="15" width="12" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:15" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A1" s="14" t="s">
         <v>0</v>
       </c>
@@ -752,7 +752,7 @@
         <v>46138</v>
       </c>
     </row>
-    <row r="2" spans="1:15" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A2" s="15"/>
       <c r="B2" s="2" t="s">
         <v>1</v>
@@ -797,7 +797,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="3" spans="1:15" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
         <v>8</v>
       </c>
@@ -844,7 +844,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="4" spans="1:15" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A4" s="3" t="s">
         <v>12</v>
       </c>
@@ -891,7 +891,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="5" spans="1:15" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A5" s="3" t="s">
         <v>14</v>
       </c>
@@ -938,7 +938,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="6" spans="1:15" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A6" s="3" t="s">
         <v>15</v>
       </c>
@@ -985,7 +985,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="7" spans="1:15" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A7" s="3" t="s">
         <v>17</v>
       </c>
@@ -1032,7 +1032,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="8" spans="1:15" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A8" s="3" t="s">
         <v>18</v>
       </c>
@@ -1079,7 +1079,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="9" spans="1:15" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A9" s="3" t="s">
         <v>20</v>
       </c>
@@ -1126,7 +1126,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="10" spans="1:15" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A10" s="3" t="s">
         <v>21</v>
       </c>
@@ -1173,7 +1173,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="11" spans="1:15" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A11" s="3" t="s">
         <v>22</v>
       </c>
@@ -1220,7 +1220,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="12" spans="1:15" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A12" s="3" t="s">
         <v>23</v>
       </c>
@@ -1267,7 +1267,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="14" spans="1:15" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A14" s="14" t="s">
         <v>0</v>
       </c>
@@ -1293,7 +1293,7 @@
         <v>46145</v>
       </c>
     </row>
-    <row r="15" spans="1:15" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A15" s="15"/>
       <c r="B15" s="2" t="s">
         <v>1</v>
@@ -1317,7 +1317,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="16" spans="1:15" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A16" s="3" t="s">
         <v>17</v>
       </c>
@@ -1343,7 +1343,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="17" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A17" s="3" t="s">
         <v>8</v>
       </c>
@@ -1369,7 +1369,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="18" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A18" s="3" t="s">
         <v>12</v>
       </c>
@@ -1395,7 +1395,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="19" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A19" s="3" t="s">
         <v>15</v>
       </c>
@@ -1421,7 +1421,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="20" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A20" s="3" t="s">
         <v>18</v>
       </c>
@@ -1447,7 +1447,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="21" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A21" s="3" t="s">
         <v>23</v>
       </c>
@@ -1473,7 +1473,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="22" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A22" s="3" t="s">
         <v>21</v>
       </c>
@@ -1499,7 +1499,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="23" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A23" s="3" t="s">
         <v>22</v>
       </c>
@@ -1525,7 +1525,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="24" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A24" s="3" t="s">
         <v>14</v>
       </c>
@@ -1551,7 +1551,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="25" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A25" s="3" t="s">
         <v>20</v>
       </c>
@@ -1577,7 +1577,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="27" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A27" s="14" t="s">
         <v>0</v>
       </c>
@@ -1603,7 +1603,7 @@
         <v>46152</v>
       </c>
     </row>
-    <row r="28" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A28" s="15"/>
       <c r="B28" s="2" t="s">
         <v>1</v>
@@ -1627,7 +1627,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="29" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A29" s="3" t="s">
         <v>22</v>
       </c>
@@ -1653,7 +1653,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="30" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A30" s="3" t="s">
         <v>14</v>
       </c>
@@ -1679,7 +1679,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="31" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A31" s="3" t="s">
         <v>20</v>
       </c>
@@ -1705,7 +1705,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="32" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A32" s="3" t="s">
         <v>15</v>
       </c>
@@ -1731,7 +1731,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="33" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A33" s="3" t="s">
         <v>18</v>
       </c>
@@ -1757,7 +1757,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="34" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A34" s="3" t="s">
         <v>21</v>
       </c>
@@ -1783,7 +1783,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="35" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A35" s="3" t="s">
         <v>8</v>
       </c>
@@ -1809,7 +1809,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="36" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A36" s="3" t="s">
         <v>12</v>
       </c>
@@ -1835,7 +1835,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="37" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A37" s="3" t="s">
         <v>23</v>
       </c>
@@ -1861,7 +1861,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="38" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A38" s="3" t="s">
         <v>17</v>
       </c>
@@ -1887,7 +1887,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="40" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A40" s="11" t="s">
         <v>0</v>
       </c>
@@ -1913,7 +1913,7 @@
         <v>46159</v>
       </c>
     </row>
-    <row r="41" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A41" s="11"/>
       <c r="B41" s="2" t="s">
         <v>1</v>
@@ -1937,7 +1937,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="42" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A42" s="3" t="s">
         <v>22</v>
       </c>
@@ -1963,7 +1963,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="43" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A43" s="3" t="s">
         <v>12</v>
       </c>
@@ -1989,7 +1989,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="44" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A44" s="3" t="s">
         <v>18</v>
       </c>
@@ -2015,7 +2015,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="45" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A45" s="3" t="s">
         <v>23</v>
       </c>
@@ -2041,7 +2041,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="46" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A46" s="3" t="s">
         <v>15</v>
       </c>
@@ -2067,7 +2067,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="47" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A47" s="3" t="s">
         <v>24</v>
       </c>
@@ -2093,7 +2093,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="48" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A48" s="3" t="s">
         <v>14</v>
       </c>
@@ -2119,7 +2119,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="49" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A49" s="3" t="s">
         <v>21</v>
       </c>
@@ -2145,7 +2145,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="50" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="50" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A50" s="3" t="s">
         <v>20</v>
       </c>
@@ -2171,7 +2171,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="51" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="51" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A51" s="3" t="s">
         <v>8</v>
       </c>
@@ -2197,7 +2197,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="53" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="53" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A53" s="11" t="s">
         <v>0</v>
       </c>
@@ -2223,7 +2223,7 @@
         <v>46166</v>
       </c>
     </row>
-    <row r="54" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="54" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A54" s="11"/>
       <c r="B54" s="2" t="s">
         <v>1</v>
@@ -2247,7 +2247,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="55" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="55" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A55" s="3" t="s">
         <v>22</v>
       </c>
@@ -2273,7 +2273,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="56" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="56" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A56" s="3" t="s">
         <v>14</v>
       </c>
@@ -2299,7 +2299,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="57" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="57" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A57" s="3" t="s">
         <v>17</v>
       </c>
@@ -2325,7 +2325,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="58" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="58" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A58" s="3" t="s">
         <v>18</v>
       </c>
@@ -2351,7 +2351,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="59" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="59" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A59" s="3" t="s">
         <v>23</v>
       </c>
@@ -2377,7 +2377,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="60" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="60" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A60" s="3" t="s">
         <v>21</v>
       </c>
@@ -2403,7 +2403,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="61" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="61" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A61" s="3" t="s">
         <v>8</v>
       </c>
@@ -2429,7 +2429,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="62" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="62" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A62" s="3" t="s">
         <v>12</v>
       </c>
@@ -2455,7 +2455,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="63" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="63" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A63" s="3" t="s">
         <v>20</v>
       </c>
@@ -2481,7 +2481,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="64" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="64" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A64" s="3" t="s">
         <v>15</v>
       </c>
@@ -2507,7 +2507,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="66" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="66" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A66" s="11" t="s">
         <v>0</v>
       </c>
@@ -2533,7 +2533,7 @@
         <v>46173</v>
       </c>
     </row>
-    <row r="67" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="67" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A67" s="11"/>
       <c r="B67" s="2" t="s">
         <v>1</v>
@@ -2557,7 +2557,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="68" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="68" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A68" s="3" t="s">
         <v>22</v>
       </c>
@@ -2583,7 +2583,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="69" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="69" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A69" s="3" t="s">
         <v>21</v>
       </c>
@@ -2609,7 +2609,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="70" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="70" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A70" s="3" t="s">
         <v>8</v>
       </c>
@@ -2635,7 +2635,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="71" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="71" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A71" s="3" t="s">
         <v>18</v>
       </c>
@@ -2661,7 +2661,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="72" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="72" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A72" s="3" t="s">
         <v>20</v>
       </c>
@@ -2687,7 +2687,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="73" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="73" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A73" s="3" t="s">
         <v>15</v>
       </c>
@@ -2713,7 +2713,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="74" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="74" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A74" s="3" t="s">
         <v>14</v>
       </c>
@@ -2739,7 +2739,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="75" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="75" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A75" s="3" t="s">
         <v>17</v>
       </c>
@@ -2765,7 +2765,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="76" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="76" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A76" s="3" t="s">
         <v>23</v>
       </c>
@@ -2791,7 +2791,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="77" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="77" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A77" s="3" t="s">
         <v>12</v>
       </c>
@@ -2817,7 +2817,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="79" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="79" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A79" s="11" t="s">
         <v>0</v>
       </c>
@@ -2843,7 +2843,7 @@
         <v>46180</v>
       </c>
     </row>
-    <row r="80" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="80" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A80" s="11"/>
       <c r="B80" s="2" t="s">
         <v>1</v>
@@ -2867,7 +2867,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="81" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="81" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A81" s="3" t="s">
         <v>22</v>
       </c>
@@ -2893,7 +2893,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="82" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="82" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A82" s="3" t="s">
         <v>14</v>
       </c>
@@ -2919,7 +2919,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="83" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="83" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A83" s="3" t="s">
         <v>12</v>
       </c>
@@ -2945,7 +2945,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="84" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="84" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A84" s="3" t="s">
         <v>15</v>
       </c>
@@ -2967,7 +2967,7 @@
       <c r="G84" s="12"/>
       <c r="H84" s="13"/>
     </row>
-    <row r="85" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="85" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A85" s="3" t="s">
         <v>17</v>
       </c>
@@ -2993,7 +2993,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="86" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="86" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A86" s="3" t="s">
         <v>18</v>
       </c>
@@ -3019,7 +3019,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="87" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="87" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A87" s="3" t="s">
         <v>21</v>
       </c>
@@ -3045,7 +3045,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="88" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="88" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A88" s="3" t="s">
         <v>8</v>
       </c>
@@ -3071,7 +3071,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="89" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="89" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A89" s="3" t="s">
         <v>20</v>
       </c>
@@ -3097,7 +3097,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="90" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="90" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A90" s="3" t="s">
         <v>23</v>
       </c>
@@ -3123,7 +3123,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="92" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="92" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A92" s="11" t="s">
         <v>0</v>
       </c>
@@ -3149,7 +3149,7 @@
         <v>46187</v>
       </c>
     </row>
-    <row r="93" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="93" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A93" s="11"/>
       <c r="B93" s="2" t="s">
         <v>1</v>
@@ -3173,7 +3173,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="94" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="94" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A94" s="3" t="s">
         <v>22</v>
       </c>
@@ -3199,7 +3199,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="95" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="95" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A95" s="3" t="s">
         <v>21</v>
       </c>
@@ -3225,7 +3225,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="96" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="96" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A96" s="3" t="s">
         <v>8</v>
       </c>
@@ -3251,7 +3251,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="97" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="97" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A97" s="3" t="s">
         <v>23</v>
       </c>
@@ -3277,7 +3277,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="98" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="98" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A98" s="3" t="s">
         <v>18</v>
       </c>
@@ -3303,7 +3303,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="99" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="99" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A99" s="3" t="s">
         <v>14</v>
       </c>
@@ -3329,7 +3329,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="100" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="100" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A100" s="3" t="s">
         <v>12</v>
       </c>
@@ -3355,7 +3355,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="101" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="101" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A101" s="3" t="s">
         <v>20</v>
       </c>
@@ -3381,7 +3381,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="102" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="102" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A102" s="3" t="s">
         <v>17</v>
       </c>
@@ -3407,8 +3407,293 @@
         <v>10</v>
       </c>
     </row>
+    <row r="104" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A104" s="11" t="s">
+        <v>0</v>
+      </c>
+      <c r="B104" s="1">
+        <v>46188</v>
+      </c>
+      <c r="C104" s="1">
+        <v>46189</v>
+      </c>
+      <c r="D104" s="1">
+        <v>46190</v>
+      </c>
+      <c r="E104" s="1">
+        <v>46191</v>
+      </c>
+      <c r="F104" s="1">
+        <v>46192</v>
+      </c>
+      <c r="G104" s="1">
+        <v>46193</v>
+      </c>
+      <c r="H104" s="1">
+        <v>46194</v>
+      </c>
+    </row>
+    <row r="105" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A105" s="11"/>
+      <c r="B105" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C105" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="D105" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="E105" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="F105" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="G105" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="H105" s="2" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="106" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A106" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="B106" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C106" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="D106" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="E106" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="F106" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="G106" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="H106" s="4" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="107" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A107" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="B107" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C107" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="D107" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="E107" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="F107" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="G107" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="H107" s="4" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="108" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A108" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="B108" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C108" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="D108" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="E108" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="F108" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="G108" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="H108" s="5" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="109" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A109" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="B109" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C109" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="D109" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="E109" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="F109" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="G109" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="H109" s="5" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="110" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A110" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="B110" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="C110" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="D110" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="E110" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="F110" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="G110" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="H110" s="5" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="111" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A111" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="B111" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="C111" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="D111" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="E111" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="F111" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="G111" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="H111" s="5" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="112" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A112" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="B112" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="C112" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="D112" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="E112" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="F112" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="G112" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="H112" s="4" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="113" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A113" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="B113" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="C113" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="D113" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="E113" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="F113" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="G113" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="H113" s="4" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="114" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A114" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="B114" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="C114" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="D114" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="E114" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="F114" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="G114" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="H114" s="5" t="s">
+        <v>10</v>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="9">
+  <mergeCells count="10">
+    <mergeCell ref="A104:A105"/>
     <mergeCell ref="A92:A93"/>
     <mergeCell ref="A79:A80"/>
     <mergeCell ref="G84:H84"/>
@@ -3425,6 +3710,26 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="9d4e7416-6feb-444a-9f0d-6e119e2a4ded">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="ab20b492-db1c-4b70-84db-283da62d5dcb" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100A49D20B196870C459C080BD3A88F41F5" ma:contentTypeVersion="12" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="c891d3af3c5d8789d4a1386f5525110a">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="9d4e7416-6feb-444a-9f0d-6e119e2a4ded" xmlns:ns3="ab20b492-db1c-4b70-84db-283da62d5dcb" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="a2d778173b158e0f4887e6c1a7be78b9" ns2:_="" ns3:_="">
     <xsd:import namespace="9d4e7416-6feb-444a-9f0d-6e119e2a4ded"/>
@@ -3625,27 +3930,26 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{3E7BE3CC-8834-4B2B-B0A5-EDC239DF005F}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="9d4e7416-6feb-444a-9f0d-6e119e2a4ded"/>
+    <ds:schemaRef ds:uri="ab20b492-db1c-4b70-84db-283da62d5dcb"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="9d4e7416-6feb-444a-9f0d-6e119e2a4ded">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="ab20b492-db1c-4b70-84db-283da62d5dcb" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{3E90FB8C-E259-434B-8A97-2530AD5FA4BD}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9D90F563-717D-4F15-9FD2-892B1218D415}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -3662,23 +3966,4 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{3E90FB8C-E259-434B-8A97-2530AD5FA4BD}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{3E7BE3CC-8834-4B2B-B0A5-EDC239DF005F}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="9d4e7416-6feb-444a-9f0d-6e119e2a4ded"/>
-    <ds:schemaRef ds:uri="ab20b492-db1c-4b70-84db-283da62d5dcb"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
Actualizar horario y cronograma a Julio
</commit_message>
<xml_diff>
--- a/Horario/Horario 2026.xlsx
+++ b/Horario/Horario 2026.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://virtualsoftserv-my.sharepoint.com/personal/maria_sanchez_virtualsoft_tech/Documents/Indicadores y Pagina WEB/Horario/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="13" documentId="13_ncr:1_{9D16BB9E-340D-4BDB-B5ED-422BF14398D6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{052E6E8A-249E-4FB9-A97F-4A15CCC6428E}"/>
+  <xr:revisionPtr revIDLastSave="21" documentId="13_ncr:1_{9D16BB9E-340D-4BDB-B5ED-422BF14398D6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{FEBE6699-5698-4B61-85A0-119C70C71826}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="5280" windowWidth="23280" windowHeight="12480" xr2:uid="{9AAEFA76-0198-46F6-BBF5-EADAB38A6758}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{9AAEFA76-0198-46F6-BBF5-EADAB38A6758}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1051" uniqueCount="30">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1155" uniqueCount="30">
   <si>
     <t>GESTOR</t>
   </si>
@@ -711,7 +711,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4B1D5CB7-A214-4F9F-A075-10C6E5CC7E55}">
-  <dimension ref="A1:O143"/>
+  <dimension ref="A1:O158"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="19.5703125" bestFit="1" customWidth="1"/>
@@ -4404,8 +4404,371 @@
         <v>10</v>
       </c>
     </row>
+    <row r="145" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A145" s="14" t="s">
+        <v>0</v>
+      </c>
+      <c r="B145" s="1">
+        <v>46209</v>
+      </c>
+      <c r="C145" s="1">
+        <v>46210</v>
+      </c>
+      <c r="D145" s="1">
+        <v>46211</v>
+      </c>
+      <c r="E145" s="1">
+        <v>46212</v>
+      </c>
+      <c r="F145" s="1">
+        <v>46213</v>
+      </c>
+      <c r="G145" s="1">
+        <v>46214</v>
+      </c>
+      <c r="H145" s="1">
+        <v>46215</v>
+      </c>
+    </row>
+    <row r="146" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A146" s="14"/>
+      <c r="B146" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C146" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="D146" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="E146" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="F146" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="G146" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="H146" s="2" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="147" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A147" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="B147" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C147" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="D147" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="E147" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="F147" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="G147" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="H147" s="5" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="148" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A148" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="B148" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C148" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="D148" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="E148" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="F148" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="G148" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="H148" s="5" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="149" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A149" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="B149" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C149" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="D149" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="E149" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="F149" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="G149" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="H149" s="5" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="150" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A150" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="B150" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C150" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="D150" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="E150" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="F150" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="G150" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="H150" s="4" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="151" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A151" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="B151" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C151" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="D151" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="E151" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="F151" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="G151" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="H151" s="4" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="152" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A152" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="B152" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C152" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="D152" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="E152" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="F152" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="G152" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="H152" s="4" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="153" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A153" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="B153" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="C153" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="D153" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="E153" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="F153" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="G153" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="H153" s="4" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="154" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A154" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="B154" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="C154" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="D154" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="E154" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="F154" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="G154" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="H154" s="4" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="155" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A155" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="B155" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="C155" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="D155" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="E155" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="F155" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="G155" s="8" t="s">
+        <v>11</v>
+      </c>
+      <c r="H155" s="5" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="156" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A156" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="B156" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="C156" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="D156" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="E156" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="F156" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="G156" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="H156" s="5" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="157" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A157" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="B157" s="8" t="s">
+        <v>11</v>
+      </c>
+      <c r="C157" s="8" t="s">
+        <v>11</v>
+      </c>
+      <c r="D157" s="8" t="s">
+        <v>11</v>
+      </c>
+      <c r="E157" s="8" t="s">
+        <v>11</v>
+      </c>
+      <c r="F157" s="8" t="s">
+        <v>11</v>
+      </c>
+      <c r="G157" s="8" t="s">
+        <v>11</v>
+      </c>
+      <c r="H157" s="5" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="158" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A158" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="B158" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C158" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="D158" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="E158" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="F158" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="G158" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="H158" s="8" t="s">
+        <v>11</v>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="11">
+  <mergeCells count="12">
+    <mergeCell ref="A145:A146"/>
     <mergeCell ref="G84:H84"/>
     <mergeCell ref="A66:A67"/>
     <mergeCell ref="A116:A117"/>
@@ -4424,15 +4787,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
     <lcf76f155ced4ddcb4097134ff3c332f xmlns="9d4e7416-6feb-444a-9f0d-6e119e2a4ded">
@@ -4441,6 +4795,15 @@
     <TaxCatchAll xmlns="ab20b492-db1c-4b70-84db-283da62d5dcb" xsi:nil="true"/>
   </documentManagement>
 </p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
@@ -4645,20 +5008,20 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{3E90FB8C-E259-434B-8A97-2530AD5FA4BD}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{3E7BE3CC-8834-4B2B-B0A5-EDC239DF005F}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
     <ds:schemaRef ds:uri="9d4e7416-6feb-444a-9f0d-6e119e2a4ded"/>
     <ds:schemaRef ds:uri="ab20b492-db1c-4b70-84db-283da62d5dcb"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{3E90FB8C-E259-434B-8A97-2530AD5FA4BD}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>

</xml_diff>

<commit_message>
Cargar archivo de Horario 2026 actualizado
</commit_message>
<xml_diff>
--- a/Horario/Horario 2026.xlsx
+++ b/Horario/Horario 2026.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://virtualsoftserv-my.sharepoint.com/personal/maria_sanchez_virtualsoft_tech/Documents/Indicadores y Pagina WEB/Horario/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="23" documentId="13_ncr:1_{9D16BB9E-340D-4BDB-B5ED-422BF14398D6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{1AA4026B-ECF4-42D8-9DFD-53DCFCBA9E3E}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="14_{F0C57C6A-092A-43C3-B98A-364FA8EFBE8C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{9AAEFA76-0198-46F6-BBF5-EADAB38A6758}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{9AAEFA76-0198-46F6-BBF5-EADAB38A6758}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1363" uniqueCount="35">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1467" uniqueCount="36">
   <si>
     <t>GESTOR</t>
   </si>
@@ -145,12 +145,15 @@
   <si>
     <t>Disponible</t>
   </si>
+  <si>
+    <t>Dia de Votación</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="9" x14ac:knownFonts="1">
+  <fonts count="13" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -212,8 +215,31 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="12"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="12"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+    </font>
   </fonts>
-  <fills count="11">
+  <fills count="12">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -271,6 +297,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="8" tint="0.59999389629810485"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="2" tint="-9.9978637043366805E-2"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -355,7 +387,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="27">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="16" fontId="2" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -382,7 +414,14 @@
     <xf numFmtId="0" fontId="2" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="10" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="9" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -391,13 +430,23 @@
     <xf numFmtId="0" fontId="4" fillId="9" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="10" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="10" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="11" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="11" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="12" fillId="10" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="20% - Énfasis4" xfId="1" builtinId="42"/>
@@ -414,6 +463,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -733,17 +786,18 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4B1D5CB7-A214-4F9F-A075-10C6E5CC7E55}">
-  <dimension ref="A1:O188"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <dimension ref="A1:O203"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="19.5546875" bestFit="1" customWidth="1"/>
-    <col min="2" max="6" width="12" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="19.5703125" bestFit="1" customWidth="1"/>
+    <col min="2" max="4" width="12" bestFit="1" customWidth="1"/>
+    <col min="5" max="6" width="16.5703125" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="17" bestFit="1" customWidth="1"/>
     <col min="8" max="15" width="12" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:15" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A1" s="15" t="s">
+    <row r="1" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A1" s="14" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="1">
@@ -789,8 +843,8 @@
         <v>46138</v>
       </c>
     </row>
-    <row r="2" spans="1:15" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A2" s="16"/>
+    <row r="2" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A2" s="15"/>
       <c r="B2" s="2" t="s">
         <v>1</v>
       </c>
@@ -834,7 +888,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="3" spans="1:15" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
         <v>8</v>
       </c>
@@ -881,7 +935,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="4" spans="1:15" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A4" s="3" t="s">
         <v>12</v>
       </c>
@@ -928,7 +982,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="5" spans="1:15" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A5" s="3" t="s">
         <v>14</v>
       </c>
@@ -975,7 +1029,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="6" spans="1:15" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A6" s="3" t="s">
         <v>15</v>
       </c>
@@ -1022,7 +1076,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="7" spans="1:15" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A7" s="3" t="s">
         <v>17</v>
       </c>
@@ -1069,7 +1123,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="8" spans="1:15" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A8" s="3" t="s">
         <v>18</v>
       </c>
@@ -1116,7 +1170,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="9" spans="1:15" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A9" s="3" t="s">
         <v>20</v>
       </c>
@@ -1163,7 +1217,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="10" spans="1:15" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A10" s="3" t="s">
         <v>21</v>
       </c>
@@ -1210,7 +1264,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="11" spans="1:15" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A11" s="3" t="s">
         <v>22</v>
       </c>
@@ -1257,7 +1311,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="12" spans="1:15" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A12" s="3" t="s">
         <v>23</v>
       </c>
@@ -1304,8 +1358,8 @@
         <v>9</v>
       </c>
     </row>
-    <row r="14" spans="1:15" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A14" s="15" t="s">
+    <row r="14" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A14" s="14" t="s">
         <v>0</v>
       </c>
       <c r="B14" s="1">
@@ -1330,8 +1384,8 @@
         <v>46145</v>
       </c>
     </row>
-    <row r="15" spans="1:15" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A15" s="16"/>
+    <row r="15" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A15" s="15"/>
       <c r="B15" s="2" t="s">
         <v>1</v>
       </c>
@@ -1354,7 +1408,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="16" spans="1:15" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A16" s="3" t="s">
         <v>17</v>
       </c>
@@ -1380,7 +1434,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="17" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A17" s="3" t="s">
         <v>8</v>
       </c>
@@ -1406,7 +1460,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="18" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A18" s="3" t="s">
         <v>12</v>
       </c>
@@ -1432,7 +1486,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="19" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A19" s="3" t="s">
         <v>15</v>
       </c>
@@ -1458,7 +1512,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="20" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A20" s="3" t="s">
         <v>18</v>
       </c>
@@ -1484,7 +1538,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="21" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A21" s="3" t="s">
         <v>23</v>
       </c>
@@ -1510,7 +1564,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="22" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A22" s="3" t="s">
         <v>21</v>
       </c>
@@ -1536,7 +1590,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="23" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A23" s="3" t="s">
         <v>22</v>
       </c>
@@ -1562,7 +1616,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="24" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A24" s="3" t="s">
         <v>14</v>
       </c>
@@ -1588,7 +1642,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="25" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A25" s="3" t="s">
         <v>20</v>
       </c>
@@ -1614,8 +1668,8 @@
         <v>10</v>
       </c>
     </row>
-    <row r="27" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A27" s="15" t="s">
+    <row r="27" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A27" s="14" t="s">
         <v>0</v>
       </c>
       <c r="B27" s="1">
@@ -1640,8 +1694,8 @@
         <v>46152</v>
       </c>
     </row>
-    <row r="28" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A28" s="16"/>
+    <row r="28" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A28" s="15"/>
       <c r="B28" s="2" t="s">
         <v>1</v>
       </c>
@@ -1664,7 +1718,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="29" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A29" s="3" t="s">
         <v>22</v>
       </c>
@@ -1690,7 +1744,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="30" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A30" s="3" t="s">
         <v>14</v>
       </c>
@@ -1716,7 +1770,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="31" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A31" s="3" t="s">
         <v>20</v>
       </c>
@@ -1742,7 +1796,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="32" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A32" s="3" t="s">
         <v>15</v>
       </c>
@@ -1768,7 +1822,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="33" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A33" s="3" t="s">
         <v>18</v>
       </c>
@@ -1794,7 +1848,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="34" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A34" s="3" t="s">
         <v>21</v>
       </c>
@@ -1820,7 +1874,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="35" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A35" s="3" t="s">
         <v>8</v>
       </c>
@@ -1846,7 +1900,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="36" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A36" s="3" t="s">
         <v>12</v>
       </c>
@@ -1872,7 +1926,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="37" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A37" s="3" t="s">
         <v>23</v>
       </c>
@@ -1898,7 +1952,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="38" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A38" s="3" t="s">
         <v>17</v>
       </c>
@@ -1924,8 +1978,8 @@
         <v>10</v>
       </c>
     </row>
-    <row r="40" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A40" s="12" t="s">
+    <row r="40" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A40" s="13" t="s">
         <v>0</v>
       </c>
       <c r="B40" s="1">
@@ -1950,8 +2004,8 @@
         <v>46159</v>
       </c>
     </row>
-    <row r="41" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A41" s="12"/>
+    <row r="41" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A41" s="13"/>
       <c r="B41" s="2" t="s">
         <v>1</v>
       </c>
@@ -1974,7 +2028,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="42" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A42" s="3" t="s">
         <v>22</v>
       </c>
@@ -2000,7 +2054,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="43" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A43" s="3" t="s">
         <v>12</v>
       </c>
@@ -2026,7 +2080,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="44" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A44" s="3" t="s">
         <v>18</v>
       </c>
@@ -2052,7 +2106,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="45" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A45" s="3" t="s">
         <v>23</v>
       </c>
@@ -2078,7 +2132,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="46" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A46" s="3" t="s">
         <v>15</v>
       </c>
@@ -2104,7 +2158,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="47" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A47" s="3" t="s">
         <v>24</v>
       </c>
@@ -2130,7 +2184,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="48" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A48" s="3" t="s">
         <v>14</v>
       </c>
@@ -2156,7 +2210,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="49" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A49" s="3" t="s">
         <v>21</v>
       </c>
@@ -2182,7 +2236,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="50" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="50" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A50" s="3" t="s">
         <v>20</v>
       </c>
@@ -2208,7 +2262,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="51" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="51" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A51" s="3" t="s">
         <v>8</v>
       </c>
@@ -2234,8 +2288,8 @@
         <v>9</v>
       </c>
     </row>
-    <row r="53" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A53" s="12" t="s">
+    <row r="53" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A53" s="13" t="s">
         <v>0</v>
       </c>
       <c r="B53" s="1">
@@ -2260,8 +2314,8 @@
         <v>46166</v>
       </c>
     </row>
-    <row r="54" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A54" s="12"/>
+    <row r="54" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A54" s="13"/>
       <c r="B54" s="2" t="s">
         <v>1</v>
       </c>
@@ -2284,7 +2338,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="55" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="55" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A55" s="3" t="s">
         <v>22</v>
       </c>
@@ -2310,7 +2364,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="56" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="56" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A56" s="3" t="s">
         <v>14</v>
       </c>
@@ -2336,7 +2390,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="57" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="57" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A57" s="3" t="s">
         <v>17</v>
       </c>
@@ -2362,7 +2416,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="58" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="58" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A58" s="3" t="s">
         <v>18</v>
       </c>
@@ -2388,7 +2442,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="59" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="59" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A59" s="3" t="s">
         <v>23</v>
       </c>
@@ -2414,7 +2468,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="60" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="60" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A60" s="3" t="s">
         <v>21</v>
       </c>
@@ -2440,7 +2494,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="61" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="61" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A61" s="3" t="s">
         <v>8</v>
       </c>
@@ -2466,7 +2520,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="62" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="62" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A62" s="3" t="s">
         <v>12</v>
       </c>
@@ -2492,7 +2546,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="63" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="63" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A63" s="3" t="s">
         <v>20</v>
       </c>
@@ -2518,7 +2572,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="64" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="64" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A64" s="3" t="s">
         <v>15</v>
       </c>
@@ -2544,8 +2598,8 @@
         <v>19</v>
       </c>
     </row>
-    <row r="66" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A66" s="12" t="s">
+    <row r="66" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A66" s="13" t="s">
         <v>0</v>
       </c>
       <c r="B66" s="1">
@@ -2570,8 +2624,8 @@
         <v>46173</v>
       </c>
     </row>
-    <row r="67" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A67" s="12"/>
+    <row r="67" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A67" s="13"/>
       <c r="B67" s="2" t="s">
         <v>1</v>
       </c>
@@ -2594,7 +2648,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="68" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="68" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A68" s="3" t="s">
         <v>22</v>
       </c>
@@ -2620,7 +2674,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="69" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="69" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A69" s="3" t="s">
         <v>21</v>
       </c>
@@ -2646,7 +2700,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="70" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="70" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A70" s="3" t="s">
         <v>8</v>
       </c>
@@ -2672,7 +2726,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="71" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="71" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A71" s="3" t="s">
         <v>18</v>
       </c>
@@ -2698,7 +2752,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="72" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="72" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A72" s="3" t="s">
         <v>20</v>
       </c>
@@ -2724,7 +2778,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="73" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="73" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A73" s="3" t="s">
         <v>15</v>
       </c>
@@ -2750,7 +2804,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="74" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="74" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A74" s="3" t="s">
         <v>14</v>
       </c>
@@ -2776,7 +2830,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="75" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="75" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A75" s="3" t="s">
         <v>17</v>
       </c>
@@ -2802,7 +2856,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="76" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="76" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A76" s="3" t="s">
         <v>23</v>
       </c>
@@ -2828,7 +2882,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="77" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="77" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A77" s="3" t="s">
         <v>12</v>
       </c>
@@ -2854,8 +2908,8 @@
         <v>10</v>
       </c>
     </row>
-    <row r="79" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A79" s="12" t="s">
+    <row r="79" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A79" s="13" t="s">
         <v>0</v>
       </c>
       <c r="B79" s="1">
@@ -2880,8 +2934,8 @@
         <v>46180</v>
       </c>
     </row>
-    <row r="80" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A80" s="12"/>
+    <row r="80" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A80" s="13"/>
       <c r="B80" s="2" t="s">
         <v>1</v>
       </c>
@@ -2904,7 +2958,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="81" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="81" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A81" s="3" t="s">
         <v>22</v>
       </c>
@@ -2930,7 +2984,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="82" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="82" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A82" s="3" t="s">
         <v>14</v>
       </c>
@@ -2956,7 +3010,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="83" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="83" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A83" s="3" t="s">
         <v>12</v>
       </c>
@@ -2982,7 +3036,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="84" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="84" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A84" s="3" t="s">
         <v>15</v>
       </c>
@@ -3001,10 +3055,10 @@
       <c r="F84" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="G84" s="13"/>
-      <c r="H84" s="14"/>
-    </row>
-    <row r="85" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="G84" s="16"/>
+      <c r="H84" s="17"/>
+    </row>
+    <row r="85" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A85" s="3" t="s">
         <v>17</v>
       </c>
@@ -3030,7 +3084,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="86" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="86" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A86" s="3" t="s">
         <v>18</v>
       </c>
@@ -3056,7 +3110,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="87" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="87" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A87" s="3" t="s">
         <v>21</v>
       </c>
@@ -3082,7 +3136,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="88" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="88" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A88" s="3" t="s">
         <v>8</v>
       </c>
@@ -3108,7 +3162,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="89" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="89" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A89" s="3" t="s">
         <v>20</v>
       </c>
@@ -3134,7 +3188,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="90" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="90" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A90" s="3" t="s">
         <v>23</v>
       </c>
@@ -3160,8 +3214,8 @@
         <v>10</v>
       </c>
     </row>
-    <row r="92" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A92" s="12" t="s">
+    <row r="92" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A92" s="13" t="s">
         <v>0</v>
       </c>
       <c r="B92" s="1">
@@ -3186,8 +3240,8 @@
         <v>46187</v>
       </c>
     </row>
-    <row r="93" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A93" s="12"/>
+    <row r="93" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A93" s="13"/>
       <c r="B93" s="2" t="s">
         <v>1</v>
       </c>
@@ -3210,7 +3264,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="94" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="94" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A94" s="3" t="s">
         <v>22</v>
       </c>
@@ -3236,7 +3290,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="95" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="95" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A95" s="3" t="s">
         <v>21</v>
       </c>
@@ -3262,7 +3316,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="96" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="96" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A96" s="3" t="s">
         <v>8</v>
       </c>
@@ -3288,7 +3342,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="97" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="97" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A97" s="3" t="s">
         <v>23</v>
       </c>
@@ -3314,7 +3368,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="98" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="98" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A98" s="3" t="s">
         <v>18</v>
       </c>
@@ -3340,7 +3394,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="99" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="99" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A99" s="3" t="s">
         <v>14</v>
       </c>
@@ -3366,7 +3420,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="100" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="100" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A100" s="3" t="s">
         <v>12</v>
       </c>
@@ -3392,7 +3446,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="101" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="101" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A101" s="3" t="s">
         <v>20</v>
       </c>
@@ -3418,7 +3472,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="102" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="102" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A102" s="3" t="s">
         <v>17</v>
       </c>
@@ -3444,8 +3498,8 @@
         <v>10</v>
       </c>
     </row>
-    <row r="104" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A104" s="12" t="s">
+    <row r="104" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A104" s="13" t="s">
         <v>0</v>
       </c>
       <c r="B104" s="1">
@@ -3470,8 +3524,8 @@
         <v>46194</v>
       </c>
     </row>
-    <row r="105" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A105" s="12"/>
+    <row r="105" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A105" s="13"/>
       <c r="B105" s="2" t="s">
         <v>1</v>
       </c>
@@ -3494,7 +3548,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="106" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="106" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A106" s="3" t="s">
         <v>22</v>
       </c>
@@ -3520,7 +3574,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="107" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="107" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A107" s="3" t="s">
         <v>12</v>
       </c>
@@ -3546,7 +3600,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="108" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="108" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A108" s="3" t="s">
         <v>17</v>
       </c>
@@ -3572,7 +3626,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="109" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="109" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A109" s="3" t="s">
         <v>20</v>
       </c>
@@ -3598,7 +3652,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="110" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="110" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A110" s="3" t="s">
         <v>23</v>
       </c>
@@ -3624,7 +3678,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="111" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="111" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A111" s="3" t="s">
         <v>18</v>
       </c>
@@ -3650,7 +3704,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="112" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="112" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A112" s="3" t="s">
         <v>14</v>
       </c>
@@ -3676,7 +3730,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="113" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="113" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A113" s="3" t="s">
         <v>8</v>
       </c>
@@ -3702,7 +3756,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="114" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="114" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A114" s="3" t="s">
         <v>21</v>
       </c>
@@ -3728,8 +3782,8 @@
         <v>10</v>
       </c>
     </row>
-    <row r="116" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A116" s="12" t="s">
+    <row r="116" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A116" s="13" t="s">
         <v>0</v>
       </c>
       <c r="B116" s="1">
@@ -3754,8 +3808,8 @@
         <v>46201</v>
       </c>
     </row>
-    <row r="117" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A117" s="12"/>
+    <row r="117" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A117" s="13"/>
       <c r="B117" s="2" t="s">
         <v>1</v>
       </c>
@@ -3778,7 +3832,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="118" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="118" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A118" s="3" t="s">
         <v>8</v>
       </c>
@@ -3804,7 +3858,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="119" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="119" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A119" s="3" t="s">
         <v>22</v>
       </c>
@@ -3830,7 +3884,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="120" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="120" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A120" s="3" t="s">
         <v>18</v>
       </c>
@@ -3856,7 +3910,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="121" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="121" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A121" s="3" t="s">
         <v>23</v>
       </c>
@@ -3882,7 +3936,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="122" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="122" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A122" s="3" t="s">
         <v>21</v>
       </c>
@@ -3908,7 +3962,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="123" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="123" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A123" s="3" t="s">
         <v>12</v>
       </c>
@@ -3934,7 +3988,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="124" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="124" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A124" s="3" t="s">
         <v>17</v>
       </c>
@@ -3960,7 +4014,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="125" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="125" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A125" s="3" t="s">
         <v>20</v>
       </c>
@@ -3986,7 +4040,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="126" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="126" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A126" s="3" t="s">
         <v>14</v>
       </c>
@@ -4012,7 +4066,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="127" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="127" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A127" s="3" t="s">
         <v>27</v>
       </c>
@@ -4038,7 +4092,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="128" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="128" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A128" s="3" t="s">
         <v>28</v>
       </c>
@@ -4064,7 +4118,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="130" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="130" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A130" s="11" t="s">
         <v>0</v>
       </c>
@@ -4090,7 +4144,7 @@
         <v>46208</v>
       </c>
     </row>
-    <row r="131" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="131" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A131" s="11"/>
       <c r="B131" s="2" t="s">
         <v>1</v>
@@ -4114,7 +4168,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="132" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="132" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A132" s="3" t="s">
         <v>22</v>
       </c>
@@ -4140,7 +4194,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="133" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="133" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A133" s="3" t="s">
         <v>29</v>
       </c>
@@ -4166,7 +4220,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="134" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="134" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A134" s="3" t="s">
         <v>12</v>
       </c>
@@ -4192,7 +4246,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="135" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="135" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A135" s="3" t="s">
         <v>17</v>
       </c>
@@ -4218,7 +4272,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="136" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="136" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A136" s="3" t="s">
         <v>20</v>
       </c>
@@ -4244,7 +4298,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="137" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="137" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A137" s="3" t="s">
         <v>14</v>
       </c>
@@ -4270,7 +4324,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="138" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="138" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A138" s="3" t="s">
         <v>18</v>
       </c>
@@ -4296,7 +4350,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="139" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="139" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A139" s="3" t="s">
         <v>23</v>
       </c>
@@ -4322,7 +4376,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="140" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="140" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A140" s="3" t="s">
         <v>21</v>
       </c>
@@ -4348,7 +4402,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="141" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="141" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A141" s="3" t="s">
         <v>8</v>
       </c>
@@ -4374,7 +4428,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="142" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="142" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A142" s="3" t="s">
         <v>27</v>
       </c>
@@ -4400,7 +4454,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="143" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="143" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A143" s="3" t="s">
         <v>28</v>
       </c>
@@ -4426,8 +4480,8 @@
         <v>10</v>
       </c>
     </row>
-    <row r="145" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A145" s="12" t="s">
+    <row r="145" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A145" s="13" t="s">
         <v>0</v>
       </c>
       <c r="B145" s="1">
@@ -4452,8 +4506,8 @@
         <v>46215</v>
       </c>
     </row>
-    <row r="146" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A146" s="12"/>
+    <row r="146" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A146" s="13"/>
       <c r="B146" s="2" t="s">
         <v>1</v>
       </c>
@@ -4476,7 +4530,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="147" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="147" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A147" s="3" t="s">
         <v>22</v>
       </c>
@@ -4502,7 +4556,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="148" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="148" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A148" s="3" t="s">
         <v>29</v>
       </c>
@@ -4528,7 +4582,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="149" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="149" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A149" s="3" t="s">
         <v>14</v>
       </c>
@@ -4554,7 +4608,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="150" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="150" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A150" s="3" t="s">
         <v>18</v>
       </c>
@@ -4580,7 +4634,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="151" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="151" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A151" s="3" t="s">
         <v>20</v>
       </c>
@@ -4606,7 +4660,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="152" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="152" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A152" s="3" t="s">
         <v>21</v>
       </c>
@@ -4632,7 +4686,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="153" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="153" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A153" s="3" t="s">
         <v>12</v>
       </c>
@@ -4658,7 +4712,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="154" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="154" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A154" s="3" t="s">
         <v>8</v>
       </c>
@@ -4684,7 +4738,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="155" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="155" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A155" s="3" t="s">
         <v>17</v>
       </c>
@@ -4710,7 +4764,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="156" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="156" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A156" s="3" t="s">
         <v>23</v>
       </c>
@@ -4736,7 +4790,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="157" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="157" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A157" s="3" t="s">
         <v>27</v>
       </c>
@@ -4762,7 +4816,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="158" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="158" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A158" s="3" t="s">
         <v>28</v>
       </c>
@@ -4788,8 +4842,8 @@
         <v>11</v>
       </c>
     </row>
-    <row r="160" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A160" s="12" t="s">
+    <row r="160" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A160" s="13" t="s">
         <v>0</v>
       </c>
       <c r="B160" s="1">
@@ -4814,8 +4868,8 @@
         <v>46222</v>
       </c>
     </row>
-    <row r="161" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A161" s="12"/>
+    <row r="161" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A161" s="13"/>
       <c r="B161" s="2" t="s">
         <v>1</v>
       </c>
@@ -4838,7 +4892,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="162" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="162" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A162" s="3" t="s">
         <v>22</v>
       </c>
@@ -4864,7 +4918,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="163" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="163" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A163" s="3" t="s">
         <v>29</v>
       </c>
@@ -4890,7 +4944,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="164" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="164" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A164" s="3" t="s">
         <v>8</v>
       </c>
@@ -4916,7 +4970,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="165" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="165" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A165" s="3" t="s">
         <v>17</v>
       </c>
@@ -4942,7 +4996,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="166" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="166" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A166" s="3" t="s">
         <v>21</v>
       </c>
@@ -4968,7 +5022,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="167" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="167" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A167" s="3" t="s">
         <v>14</v>
       </c>
@@ -4994,7 +5048,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="168" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="168" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A168" s="3" t="s">
         <v>23</v>
       </c>
@@ -5020,7 +5074,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="169" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="169" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A169" s="3" t="s">
         <v>18</v>
       </c>
@@ -5046,7 +5100,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="170" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="170" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A170" s="3" t="s">
         <v>20</v>
       </c>
@@ -5072,7 +5126,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="171" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="171" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A171" s="3" t="s">
         <v>12</v>
       </c>
@@ -5098,7 +5152,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="172" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="172" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A172" s="3" t="s">
         <v>27</v>
       </c>
@@ -5124,7 +5178,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="173" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="173" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A173" s="3" t="s">
         <v>28</v>
       </c>
@@ -5150,8 +5204,8 @@
         <v>10</v>
       </c>
     </row>
-    <row r="175" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A175" s="12" t="s">
+    <row r="175" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A175" s="13" t="s">
         <v>0</v>
       </c>
       <c r="B175" s="1">
@@ -5176,8 +5230,8 @@
         <v>46229</v>
       </c>
     </row>
-    <row r="176" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A176" s="12"/>
+    <row r="176" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A176" s="13"/>
       <c r="B176" s="2" t="s">
         <v>1</v>
       </c>
@@ -5200,7 +5254,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="177" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="177" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A177" s="3" t="s">
         <v>22</v>
       </c>
@@ -5226,7 +5280,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="178" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="178" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A178" s="3" t="s">
         <v>29</v>
       </c>
@@ -5252,7 +5306,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="179" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="179" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A179" s="3" t="s">
         <v>12</v>
       </c>
@@ -5278,7 +5332,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="180" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="180" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A180" s="3" t="s">
         <v>21</v>
       </c>
@@ -5304,7 +5358,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="181" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="181" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A181" s="3" t="s">
         <v>23</v>
       </c>
@@ -5330,7 +5384,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="182" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="182" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A182" s="3" t="s">
         <v>18</v>
       </c>
@@ -5356,7 +5410,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="183" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="183" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A183" s="3" t="s">
         <v>17</v>
       </c>
@@ -5382,7 +5436,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="184" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="184" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A184" s="3" t="s">
         <v>14</v>
       </c>
@@ -5408,7 +5462,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="185" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="185" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A185" s="3" t="s">
         <v>8</v>
       </c>
@@ -5434,7 +5488,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="186" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="186" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A186" s="3" t="s">
         <v>20</v>
       </c>
@@ -5460,11 +5514,11 @@
         <v>10</v>
       </c>
     </row>
-    <row r="187" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="187" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A187" s="3" t="s">
         <v>28</v>
       </c>
-      <c r="B187" s="17" t="s">
+      <c r="B187" s="12" t="s">
         <v>30</v>
       </c>
       <c r="C187" s="4" t="s">
@@ -5486,11 +5540,11 @@
         <v>10</v>
       </c>
     </row>
-    <row r="188" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="188" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A188" s="3" t="s">
         <v>27</v>
       </c>
-      <c r="B188" s="17" t="s">
+      <c r="B188" s="12" t="s">
         <v>32</v>
       </c>
       <c r="C188" s="4" t="s">
@@ -5505,15 +5559,384 @@
       <c r="F188" s="4" t="s">
         <v>33</v>
       </c>
-      <c r="G188" s="17" t="s">
+      <c r="G188" s="12" t="s">
         <v>34</v>
       </c>
-      <c r="H188" s="17" t="s">
+      <c r="H188" s="12" t="s">
         <v>34</v>
       </c>
     </row>
+    <row r="190" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A190" s="13" t="s">
+        <v>0</v>
+      </c>
+      <c r="B190" s="1">
+        <v>46230</v>
+      </c>
+      <c r="C190" s="1">
+        <v>46231</v>
+      </c>
+      <c r="D190" s="1">
+        <v>46232</v>
+      </c>
+      <c r="E190" s="1">
+        <v>46233</v>
+      </c>
+      <c r="F190" s="1">
+        <v>46234</v>
+      </c>
+      <c r="G190" s="1">
+        <v>46235</v>
+      </c>
+      <c r="H190" s="1">
+        <v>46236</v>
+      </c>
+    </row>
+    <row r="191" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A191" s="13"/>
+      <c r="B191" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C191" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="D191" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="E191" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="F191" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="G191" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="H191" s="2" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="192" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A192" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="B192" s="18" t="s">
+        <v>9</v>
+      </c>
+      <c r="C192" s="18" t="s">
+        <v>9</v>
+      </c>
+      <c r="D192" s="18" t="s">
+        <v>9</v>
+      </c>
+      <c r="E192" s="18" t="s">
+        <v>9</v>
+      </c>
+      <c r="F192" s="18" t="s">
+        <v>9</v>
+      </c>
+      <c r="G192" s="19" t="s">
+        <v>9</v>
+      </c>
+      <c r="H192" s="20" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="193" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A193" s="21" t="s">
+        <v>29</v>
+      </c>
+      <c r="B193" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C193" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="D193" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="E193" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="F193" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="G193" s="20" t="s">
+        <v>10</v>
+      </c>
+      <c r="H193" s="19" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="194" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A194" s="21" t="s">
+        <v>14</v>
+      </c>
+      <c r="B194" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C194" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="D194" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="E194" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="F194" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="G194" s="20" t="s">
+        <v>10</v>
+      </c>
+      <c r="H194" s="4" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="195" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A195" s="21" t="s">
+        <v>8</v>
+      </c>
+      <c r="B195" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C195" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="D195" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="E195" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="F195" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="G195" s="19" t="s">
+        <v>9</v>
+      </c>
+      <c r="H195" s="20" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="196" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A196" s="22" t="s">
+        <v>20</v>
+      </c>
+      <c r="B196" s="19" t="s">
+        <v>9</v>
+      </c>
+      <c r="C196" s="19" t="s">
+        <v>9</v>
+      </c>
+      <c r="D196" s="19" t="s">
+        <v>9</v>
+      </c>
+      <c r="E196" s="19" t="s">
+        <v>9</v>
+      </c>
+      <c r="F196" s="19" t="s">
+        <v>9</v>
+      </c>
+      <c r="G196" s="20" t="s">
+        <v>10</v>
+      </c>
+      <c r="H196" s="19" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="197" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A197" s="23" t="s">
+        <v>23</v>
+      </c>
+      <c r="B197" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C197" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="D197" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="E197" s="24" t="s">
+        <v>35</v>
+      </c>
+      <c r="F197" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="G197" s="20" t="s">
+        <v>10</v>
+      </c>
+      <c r="H197" s="19" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="198" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A198" s="22" t="s">
+        <v>12</v>
+      </c>
+      <c r="B198" s="19" t="s">
+        <v>11</v>
+      </c>
+      <c r="C198" s="19" t="s">
+        <v>11</v>
+      </c>
+      <c r="D198" s="19" t="s">
+        <v>11</v>
+      </c>
+      <c r="E198" s="19" t="s">
+        <v>11</v>
+      </c>
+      <c r="F198" s="19" t="s">
+        <v>11</v>
+      </c>
+      <c r="G198" s="19" t="s">
+        <v>11</v>
+      </c>
+      <c r="H198" s="20" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="199" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A199" s="21" t="s">
+        <v>21</v>
+      </c>
+      <c r="B199" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="C199" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="D199" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="E199" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="F199" s="24" t="s">
+        <v>35</v>
+      </c>
+      <c r="G199" s="20" t="s">
+        <v>10</v>
+      </c>
+      <c r="H199" s="19" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="200" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A200" s="21" t="s">
+        <v>18</v>
+      </c>
+      <c r="B200" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="C200" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="D200" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="E200" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="F200" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="G200" s="19" t="s">
+        <v>11</v>
+      </c>
+      <c r="H200" s="20" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="201" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A201" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="B201" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="C201" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="D201" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="E201" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="F201" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="G201" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="H201" s="20" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="202" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A202" s="21" t="s">
+        <v>27</v>
+      </c>
+      <c r="B202" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="C202" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="D202" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="E202" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="F202" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="G202" s="20" t="s">
+        <v>10</v>
+      </c>
+      <c r="H202" s="20" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="203" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A203" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="B203" s="25" t="s">
+        <v>33</v>
+      </c>
+      <c r="C203" s="25" t="s">
+        <v>33</v>
+      </c>
+      <c r="D203" s="25" t="s">
+        <v>33</v>
+      </c>
+      <c r="E203" s="25" t="s">
+        <v>33</v>
+      </c>
+      <c r="F203" s="25" t="s">
+        <v>33</v>
+      </c>
+      <c r="G203" s="26" t="s">
+        <v>34</v>
+      </c>
+      <c r="H203" s="26" t="s">
+        <v>34</v>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="14">
+  <mergeCells count="15">
+    <mergeCell ref="A190:A191"/>
+    <mergeCell ref="G84:H84"/>
+    <mergeCell ref="A66:A67"/>
+    <mergeCell ref="A116:A117"/>
+    <mergeCell ref="A104:A105"/>
+    <mergeCell ref="A92:A93"/>
+    <mergeCell ref="A79:A80"/>
     <mergeCell ref="A175:A176"/>
     <mergeCell ref="A1:A2"/>
     <mergeCell ref="A14:A15"/>
@@ -5522,12 +5945,6 @@
     <mergeCell ref="A53:A54"/>
     <mergeCell ref="A160:A161"/>
     <mergeCell ref="A145:A146"/>
-    <mergeCell ref="G84:H84"/>
-    <mergeCell ref="A66:A67"/>
-    <mergeCell ref="A116:A117"/>
-    <mergeCell ref="A104:A105"/>
-    <mergeCell ref="A92:A93"/>
-    <mergeCell ref="A79:A80"/>
   </mergeCells>
   <phoneticPr fontId="7" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -5535,15 +5952,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100A49D20B196870C459C080BD3A88F41F5" ma:contentTypeVersion="12" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="c891d3af3c5d8789d4a1386f5525110a">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="9d4e7416-6feb-444a-9f0d-6e119e2a4ded" xmlns:ns3="ab20b492-db1c-4b70-84db-283da62d5dcb" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="a2d778173b158e0f4887e6c1a7be78b9" ns2:_="" ns3:_="">
     <xsd:import namespace="9d4e7416-6feb-444a-9f0d-6e119e2a4ded"/>
@@ -5744,6 +6152,15 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
@@ -5756,14 +6173,6 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{3E90FB8C-E259-434B-8A97-2530AD5FA4BD}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9D90F563-717D-4F15-9FD2-892B1218D415}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -5782,6 +6191,14 @@
 </ds:datastoreItem>
 </file>
 
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{3E90FB8C-E259-434B-8A97-2530AD5FA4BD}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{3E7BE3CC-8834-4B2B-B0A5-EDC239DF005F}">
   <ds:schemaRefs>

</xml_diff>

<commit_message>
Actualizacion de horario y configuracion de exclusiones de archivos pesados
</commit_message>
<xml_diff>
--- a/Horario/Horario 2026.xlsx
+++ b/Horario/Horario 2026.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://virtualsoftserv-my.sharepoint.com/personal/maria_sanchez_virtualsoft_tech/Documents/Indicadores y Pagina WEB/Horario/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="14_{F0C57C6A-092A-43C3-B98A-364FA8EFBE8C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="6_{6E17BD36-3E42-42F2-8AFD-92DB165A9BC2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{9AAEFA76-0198-46F6-BBF5-EADAB38A6758}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{9AAEFA76-0198-46F6-BBF5-EADAB38A6758}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
@@ -219,24 +219,28 @@
       <sz val="12"/>
       <color theme="1"/>
       <name val="Calibri"/>
+      <family val="2"/>
     </font>
     <font>
       <b/>
       <sz val="12"/>
       <color rgb="FF000000"/>
       <name val="Calibri"/>
+      <family val="2"/>
     </font>
     <font>
       <b/>
       <sz val="12"/>
       <color rgb="FFFFFFFF"/>
       <name val="Calibri"/>
+      <family val="2"/>
     </font>
     <font>
       <b/>
       <sz val="12"/>
       <color theme="1"/>
       <name val="Calibri"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="12">
@@ -415,21 +419,6 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="10" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="9" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="9" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="10" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -447,6 +436,21 @@
     <xf numFmtId="0" fontId="5" fillId="11" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="12" fillId="10" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="9" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="9" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="20% - Énfasis4" xfId="1" builtinId="42"/>
@@ -465,8 +469,57 @@
 </styleSheet>
 </file>
 
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>194</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>304800</xdr:colOff>
+      <xdr:row>195</xdr:row>
+      <xdr:rowOff>106680</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="1025" name="AutoShape 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{0D4ADAC6-934E-F14F-7EBC-3B184D690824}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr>
+          <a:spLocks noChangeAspect="1" noChangeArrowheads="1"/>
+        </xdr:cNvSpPr>
+      </xdr:nvSpPr>
+      <xdr:spPr bwMode="auto">
+        <a:xfrm>
+          <a:off x="6080760" y="38221920"/>
+          <a:ext cx="304800" cy="304800"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:extLst>
+          <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
+            <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+              <a:solidFill>
+                <a:srgbClr val="FFFFFF"/>
+              </a:solidFill>
+            </a14:hiddenFill>
+          </a:ext>
+        </a:extLst>
+      </xdr:spPr>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -787,17 +840,17 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4B1D5CB7-A214-4F9F-A075-10C6E5CC7E55}">
   <dimension ref="A1:O203"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="19.5703125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="19.5546875" bestFit="1" customWidth="1"/>
     <col min="2" max="4" width="12" bestFit="1" customWidth="1"/>
-    <col min="5" max="6" width="16.5703125" bestFit="1" customWidth="1"/>
+    <col min="5" max="6" width="16.5546875" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="17" bestFit="1" customWidth="1"/>
     <col min="8" max="15" width="12" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A1" s="14" t="s">
+    <row r="1" spans="1:15" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A1" s="25" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="1">
@@ -843,8 +896,8 @@
         <v>46138</v>
       </c>
     </row>
-    <row r="2" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A2" s="15"/>
+    <row r="2" spans="1:15" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A2" s="26"/>
       <c r="B2" s="2" t="s">
         <v>1</v>
       </c>
@@ -888,7 +941,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="3" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:15" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A3" s="3" t="s">
         <v>8</v>
       </c>
@@ -935,7 +988,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="4" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:15" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A4" s="3" t="s">
         <v>12</v>
       </c>
@@ -982,7 +1035,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="5" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:15" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A5" s="3" t="s">
         <v>14</v>
       </c>
@@ -1029,7 +1082,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="6" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:15" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A6" s="3" t="s">
         <v>15</v>
       </c>
@@ -1076,7 +1129,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="7" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:15" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A7" s="3" t="s">
         <v>17</v>
       </c>
@@ -1123,7 +1176,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="8" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:15" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A8" s="3" t="s">
         <v>18</v>
       </c>
@@ -1170,7 +1223,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="9" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:15" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A9" s="3" t="s">
         <v>20</v>
       </c>
@@ -1217,7 +1270,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="10" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:15" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A10" s="3" t="s">
         <v>21</v>
       </c>
@@ -1264,7 +1317,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="11" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:15" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A11" s="3" t="s">
         <v>22</v>
       </c>
@@ -1311,7 +1364,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="12" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:15" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A12" s="3" t="s">
         <v>23</v>
       </c>
@@ -1358,8 +1411,8 @@
         <v>9</v>
       </c>
     </row>
-    <row r="14" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A14" s="14" t="s">
+    <row r="14" spans="1:15" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A14" s="25" t="s">
         <v>0</v>
       </c>
       <c r="B14" s="1">
@@ -1384,8 +1437,8 @@
         <v>46145</v>
       </c>
     </row>
-    <row r="15" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A15" s="15"/>
+    <row r="15" spans="1:15" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A15" s="26"/>
       <c r="B15" s="2" t="s">
         <v>1</v>
       </c>
@@ -1408,7 +1461,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="16" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:15" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A16" s="3" t="s">
         <v>17</v>
       </c>
@@ -1434,7 +1487,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="17" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A17" s="3" t="s">
         <v>8</v>
       </c>
@@ -1460,7 +1513,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="18" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A18" s="3" t="s">
         <v>12</v>
       </c>
@@ -1486,7 +1539,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="19" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A19" s="3" t="s">
         <v>15</v>
       </c>
@@ -1512,7 +1565,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="20" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A20" s="3" t="s">
         <v>18</v>
       </c>
@@ -1538,7 +1591,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="21" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A21" s="3" t="s">
         <v>23</v>
       </c>
@@ -1564,7 +1617,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="22" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A22" s="3" t="s">
         <v>21</v>
       </c>
@@ -1590,7 +1643,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="23" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A23" s="3" t="s">
         <v>22</v>
       </c>
@@ -1616,7 +1669,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="24" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A24" s="3" t="s">
         <v>14</v>
       </c>
@@ -1642,7 +1695,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="25" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A25" s="3" t="s">
         <v>20</v>
       </c>
@@ -1668,8 +1721,8 @@
         <v>10</v>
       </c>
     </row>
-    <row r="27" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A27" s="14" t="s">
+    <row r="27" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A27" s="25" t="s">
         <v>0</v>
       </c>
       <c r="B27" s="1">
@@ -1694,8 +1747,8 @@
         <v>46152</v>
       </c>
     </row>
-    <row r="28" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A28" s="15"/>
+    <row r="28" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A28" s="26"/>
       <c r="B28" s="2" t="s">
         <v>1</v>
       </c>
@@ -1718,7 +1771,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="29" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A29" s="3" t="s">
         <v>22</v>
       </c>
@@ -1744,7 +1797,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="30" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A30" s="3" t="s">
         <v>14</v>
       </c>
@@ -1770,7 +1823,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="31" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A31" s="3" t="s">
         <v>20</v>
       </c>
@@ -1796,7 +1849,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="32" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A32" s="3" t="s">
         <v>15</v>
       </c>
@@ -1822,7 +1875,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="33" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A33" s="3" t="s">
         <v>18</v>
       </c>
@@ -1848,7 +1901,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="34" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A34" s="3" t="s">
         <v>21</v>
       </c>
@@ -1874,7 +1927,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="35" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A35" s="3" t="s">
         <v>8</v>
       </c>
@@ -1900,7 +1953,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="36" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A36" s="3" t="s">
         <v>12</v>
       </c>
@@ -1926,7 +1979,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="37" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A37" s="3" t="s">
         <v>23</v>
       </c>
@@ -1952,7 +2005,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="38" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A38" s="3" t="s">
         <v>17</v>
       </c>
@@ -1978,8 +2031,8 @@
         <v>10</v>
       </c>
     </row>
-    <row r="40" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A40" s="13" t="s">
+    <row r="40" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A40" s="22" t="s">
         <v>0</v>
       </c>
       <c r="B40" s="1">
@@ -2004,8 +2057,8 @@
         <v>46159</v>
       </c>
     </row>
-    <row r="41" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A41" s="13"/>
+    <row r="41" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A41" s="22"/>
       <c r="B41" s="2" t="s">
         <v>1</v>
       </c>
@@ -2028,7 +2081,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="42" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A42" s="3" t="s">
         <v>22</v>
       </c>
@@ -2054,7 +2107,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="43" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A43" s="3" t="s">
         <v>12</v>
       </c>
@@ -2080,7 +2133,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="44" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A44" s="3" t="s">
         <v>18</v>
       </c>
@@ -2106,7 +2159,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="45" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A45" s="3" t="s">
         <v>23</v>
       </c>
@@ -2132,7 +2185,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="46" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A46" s="3" t="s">
         <v>15</v>
       </c>
@@ -2158,7 +2211,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="47" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A47" s="3" t="s">
         <v>24</v>
       </c>
@@ -2184,7 +2237,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="48" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A48" s="3" t="s">
         <v>14</v>
       </c>
@@ -2210,7 +2263,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="49" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A49" s="3" t="s">
         <v>21</v>
       </c>
@@ -2236,7 +2289,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="50" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A50" s="3" t="s">
         <v>20</v>
       </c>
@@ -2262,7 +2315,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="51" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A51" s="3" t="s">
         <v>8</v>
       </c>
@@ -2288,8 +2341,8 @@
         <v>9</v>
       </c>
     </row>
-    <row r="53" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A53" s="13" t="s">
+    <row r="53" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A53" s="22" t="s">
         <v>0</v>
       </c>
       <c r="B53" s="1">
@@ -2314,8 +2367,8 @@
         <v>46166</v>
       </c>
     </row>
-    <row r="54" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A54" s="13"/>
+    <row r="54" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A54" s="22"/>
       <c r="B54" s="2" t="s">
         <v>1</v>
       </c>
@@ -2338,7 +2391,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="55" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A55" s="3" t="s">
         <v>22</v>
       </c>
@@ -2364,7 +2417,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="56" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A56" s="3" t="s">
         <v>14</v>
       </c>
@@ -2390,7 +2443,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="57" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A57" s="3" t="s">
         <v>17</v>
       </c>
@@ -2416,7 +2469,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="58" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A58" s="3" t="s">
         <v>18</v>
       </c>
@@ -2442,7 +2495,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="59" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A59" s="3" t="s">
         <v>23</v>
       </c>
@@ -2468,7 +2521,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="60" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A60" s="3" t="s">
         <v>21</v>
       </c>
@@ -2494,7 +2547,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="61" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A61" s="3" t="s">
         <v>8</v>
       </c>
@@ -2520,7 +2573,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="62" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A62" s="3" t="s">
         <v>12</v>
       </c>
@@ -2546,7 +2599,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="63" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A63" s="3" t="s">
         <v>20</v>
       </c>
@@ -2572,7 +2625,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="64" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A64" s="3" t="s">
         <v>15</v>
       </c>
@@ -2598,8 +2651,8 @@
         <v>19</v>
       </c>
     </row>
-    <row r="66" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A66" s="13" t="s">
+    <row r="66" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A66" s="22" t="s">
         <v>0</v>
       </c>
       <c r="B66" s="1">
@@ -2624,8 +2677,8 @@
         <v>46173</v>
       </c>
     </row>
-    <row r="67" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A67" s="13"/>
+    <row r="67" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A67" s="22"/>
       <c r="B67" s="2" t="s">
         <v>1</v>
       </c>
@@ -2648,7 +2701,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="68" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A68" s="3" t="s">
         <v>22</v>
       </c>
@@ -2674,7 +2727,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="69" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A69" s="3" t="s">
         <v>21</v>
       </c>
@@ -2700,7 +2753,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="70" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A70" s="3" t="s">
         <v>8</v>
       </c>
@@ -2726,7 +2779,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="71" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A71" s="3" t="s">
         <v>18</v>
       </c>
@@ -2752,7 +2805,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="72" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A72" s="3" t="s">
         <v>20</v>
       </c>
@@ -2778,7 +2831,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="73" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="73" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A73" s="3" t="s">
         <v>15</v>
       </c>
@@ -2804,7 +2857,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="74" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="74" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A74" s="3" t="s">
         <v>14</v>
       </c>
@@ -2830,7 +2883,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="75" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="75" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A75" s="3" t="s">
         <v>17</v>
       </c>
@@ -2856,7 +2909,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="76" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="76" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A76" s="3" t="s">
         <v>23</v>
       </c>
@@ -2882,7 +2935,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="77" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="77" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A77" s="3" t="s">
         <v>12</v>
       </c>
@@ -2908,8 +2961,8 @@
         <v>10</v>
       </c>
     </row>
-    <row r="79" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A79" s="13" t="s">
+    <row r="79" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A79" s="22" t="s">
         <v>0</v>
       </c>
       <c r="B79" s="1">
@@ -2934,8 +2987,8 @@
         <v>46180</v>
       </c>
     </row>
-    <row r="80" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A80" s="13"/>
+    <row r="80" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A80" s="22"/>
       <c r="B80" s="2" t="s">
         <v>1</v>
       </c>
@@ -2958,7 +3011,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="81" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="81" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A81" s="3" t="s">
         <v>22</v>
       </c>
@@ -2984,7 +3037,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="82" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="82" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A82" s="3" t="s">
         <v>14</v>
       </c>
@@ -3010,7 +3063,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="83" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="83" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A83" s="3" t="s">
         <v>12</v>
       </c>
@@ -3036,7 +3089,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="84" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="84" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A84" s="3" t="s">
         <v>15</v>
       </c>
@@ -3055,10 +3108,10 @@
       <c r="F84" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="G84" s="16"/>
-      <c r="H84" s="17"/>
-    </row>
-    <row r="85" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="G84" s="23"/>
+      <c r="H84" s="24"/>
+    </row>
+    <row r="85" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A85" s="3" t="s">
         <v>17</v>
       </c>
@@ -3084,7 +3137,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="86" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="86" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A86" s="3" t="s">
         <v>18</v>
       </c>
@@ -3110,7 +3163,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="87" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="87" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A87" s="3" t="s">
         <v>21</v>
       </c>
@@ -3136,7 +3189,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="88" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="88" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A88" s="3" t="s">
         <v>8</v>
       </c>
@@ -3162,7 +3215,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="89" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="89" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A89" s="3" t="s">
         <v>20</v>
       </c>
@@ -3188,7 +3241,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="90" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="90" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A90" s="3" t="s">
         <v>23</v>
       </c>
@@ -3214,8 +3267,8 @@
         <v>10</v>
       </c>
     </row>
-    <row r="92" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A92" s="13" t="s">
+    <row r="92" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A92" s="22" t="s">
         <v>0</v>
       </c>
       <c r="B92" s="1">
@@ -3240,8 +3293,8 @@
         <v>46187</v>
       </c>
     </row>
-    <row r="93" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A93" s="13"/>
+    <row r="93" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A93" s="22"/>
       <c r="B93" s="2" t="s">
         <v>1</v>
       </c>
@@ -3264,7 +3317,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="94" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="94" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A94" s="3" t="s">
         <v>22</v>
       </c>
@@ -3290,7 +3343,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="95" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="95" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A95" s="3" t="s">
         <v>21</v>
       </c>
@@ -3316,7 +3369,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="96" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="96" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A96" s="3" t="s">
         <v>8</v>
       </c>
@@ -3342,7 +3395,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="97" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="97" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A97" s="3" t="s">
         <v>23</v>
       </c>
@@ -3368,7 +3421,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="98" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="98" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A98" s="3" t="s">
         <v>18</v>
       </c>
@@ -3394,7 +3447,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="99" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="99" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A99" s="3" t="s">
         <v>14</v>
       </c>
@@ -3420,7 +3473,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="100" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="100" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A100" s="3" t="s">
         <v>12</v>
       </c>
@@ -3446,7 +3499,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="101" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="101" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A101" s="3" t="s">
         <v>20</v>
       </c>
@@ -3472,7 +3525,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="102" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="102" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A102" s="3" t="s">
         <v>17</v>
       </c>
@@ -3498,8 +3551,8 @@
         <v>10</v>
       </c>
     </row>
-    <row r="104" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A104" s="13" t="s">
+    <row r="104" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A104" s="22" t="s">
         <v>0</v>
       </c>
       <c r="B104" s="1">
@@ -3524,8 +3577,8 @@
         <v>46194</v>
       </c>
     </row>
-    <row r="105" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A105" s="13"/>
+    <row r="105" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A105" s="22"/>
       <c r="B105" s="2" t="s">
         <v>1</v>
       </c>
@@ -3548,7 +3601,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="106" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="106" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A106" s="3" t="s">
         <v>22</v>
       </c>
@@ -3574,7 +3627,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="107" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="107" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A107" s="3" t="s">
         <v>12</v>
       </c>
@@ -3600,7 +3653,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="108" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="108" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A108" s="3" t="s">
         <v>17</v>
       </c>
@@ -3626,7 +3679,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="109" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="109" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A109" s="3" t="s">
         <v>20</v>
       </c>
@@ -3652,7 +3705,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="110" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="110" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A110" s="3" t="s">
         <v>23</v>
       </c>
@@ -3678,7 +3731,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="111" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="111" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A111" s="3" t="s">
         <v>18</v>
       </c>
@@ -3704,7 +3757,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="112" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="112" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A112" s="3" t="s">
         <v>14</v>
       </c>
@@ -3730,7 +3783,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="113" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="113" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A113" s="3" t="s">
         <v>8</v>
       </c>
@@ -3756,7 +3809,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="114" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="114" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A114" s="3" t="s">
         <v>21</v>
       </c>
@@ -3782,8 +3835,8 @@
         <v>10</v>
       </c>
     </row>
-    <row r="116" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A116" s="13" t="s">
+    <row r="116" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A116" s="22" t="s">
         <v>0</v>
       </c>
       <c r="B116" s="1">
@@ -3808,8 +3861,8 @@
         <v>46201</v>
       </c>
     </row>
-    <row r="117" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A117" s="13"/>
+    <row r="117" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A117" s="22"/>
       <c r="B117" s="2" t="s">
         <v>1</v>
       </c>
@@ -3832,7 +3885,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="118" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="118" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A118" s="3" t="s">
         <v>8</v>
       </c>
@@ -3858,7 +3911,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="119" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="119" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A119" s="3" t="s">
         <v>22</v>
       </c>
@@ -3884,7 +3937,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="120" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="120" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A120" s="3" t="s">
         <v>18</v>
       </c>
@@ -3910,7 +3963,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="121" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="121" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A121" s="3" t="s">
         <v>23</v>
       </c>
@@ -3936,7 +3989,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="122" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="122" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A122" s="3" t="s">
         <v>21</v>
       </c>
@@ -3962,7 +4015,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="123" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="123" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A123" s="3" t="s">
         <v>12</v>
       </c>
@@ -3988,7 +4041,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="124" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="124" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A124" s="3" t="s">
         <v>17</v>
       </c>
@@ -4014,7 +4067,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="125" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="125" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A125" s="3" t="s">
         <v>20</v>
       </c>
@@ -4040,7 +4093,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="126" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="126" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A126" s="3" t="s">
         <v>14</v>
       </c>
@@ -4066,7 +4119,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="127" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="127" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A127" s="3" t="s">
         <v>27</v>
       </c>
@@ -4092,7 +4145,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="128" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="128" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A128" s="3" t="s">
         <v>28</v>
       </c>
@@ -4118,7 +4171,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="130" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="130" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A130" s="11" t="s">
         <v>0</v>
       </c>
@@ -4144,7 +4197,7 @@
         <v>46208</v>
       </c>
     </row>
-    <row r="131" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="131" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A131" s="11"/>
       <c r="B131" s="2" t="s">
         <v>1</v>
@@ -4168,7 +4221,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="132" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="132" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A132" s="3" t="s">
         <v>22</v>
       </c>
@@ -4194,7 +4247,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="133" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="133" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A133" s="3" t="s">
         <v>29</v>
       </c>
@@ -4220,7 +4273,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="134" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="134" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A134" s="3" t="s">
         <v>12</v>
       </c>
@@ -4246,7 +4299,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="135" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="135" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A135" s="3" t="s">
         <v>17</v>
       </c>
@@ -4272,7 +4325,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="136" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="136" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A136" s="3" t="s">
         <v>20</v>
       </c>
@@ -4298,7 +4351,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="137" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="137" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A137" s="3" t="s">
         <v>14</v>
       </c>
@@ -4324,7 +4377,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="138" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="138" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A138" s="3" t="s">
         <v>18</v>
       </c>
@@ -4350,7 +4403,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="139" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="139" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A139" s="3" t="s">
         <v>23</v>
       </c>
@@ -4376,7 +4429,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="140" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="140" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A140" s="3" t="s">
         <v>21</v>
       </c>
@@ -4402,7 +4455,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="141" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="141" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A141" s="3" t="s">
         <v>8</v>
       </c>
@@ -4428,7 +4481,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="142" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="142" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A142" s="3" t="s">
         <v>27</v>
       </c>
@@ -4454,7 +4507,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="143" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="143" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A143" s="3" t="s">
         <v>28</v>
       </c>
@@ -4480,8 +4533,8 @@
         <v>10</v>
       </c>
     </row>
-    <row r="145" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A145" s="13" t="s">
+    <row r="145" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A145" s="22" t="s">
         <v>0</v>
       </c>
       <c r="B145" s="1">
@@ -4506,8 +4559,8 @@
         <v>46215</v>
       </c>
     </row>
-    <row r="146" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A146" s="13"/>
+    <row r="146" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A146" s="22"/>
       <c r="B146" s="2" t="s">
         <v>1</v>
       </c>
@@ -4530,7 +4583,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="147" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="147" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A147" s="3" t="s">
         <v>22</v>
       </c>
@@ -4556,7 +4609,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="148" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="148" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A148" s="3" t="s">
         <v>29</v>
       </c>
@@ -4582,7 +4635,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="149" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="149" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A149" s="3" t="s">
         <v>14</v>
       </c>
@@ -4608,7 +4661,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="150" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="150" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A150" s="3" t="s">
         <v>18</v>
       </c>
@@ -4634,7 +4687,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="151" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="151" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A151" s="3" t="s">
         <v>20</v>
       </c>
@@ -4660,7 +4713,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="152" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="152" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A152" s="3" t="s">
         <v>21</v>
       </c>
@@ -4686,7 +4739,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="153" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="153" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A153" s="3" t="s">
         <v>12</v>
       </c>
@@ -4712,7 +4765,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="154" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="154" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A154" s="3" t="s">
         <v>8</v>
       </c>
@@ -4738,7 +4791,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="155" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="155" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A155" s="3" t="s">
         <v>17</v>
       </c>
@@ -4764,7 +4817,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="156" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="156" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A156" s="3" t="s">
         <v>23</v>
       </c>
@@ -4790,7 +4843,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="157" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="157" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A157" s="3" t="s">
         <v>27</v>
       </c>
@@ -4816,7 +4869,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="158" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="158" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A158" s="3" t="s">
         <v>28</v>
       </c>
@@ -4842,8 +4895,8 @@
         <v>11</v>
       </c>
     </row>
-    <row r="160" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A160" s="13" t="s">
+    <row r="160" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A160" s="22" t="s">
         <v>0</v>
       </c>
       <c r="B160" s="1">
@@ -4868,8 +4921,8 @@
         <v>46222</v>
       </c>
     </row>
-    <row r="161" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A161" s="13"/>
+    <row r="161" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A161" s="22"/>
       <c r="B161" s="2" t="s">
         <v>1</v>
       </c>
@@ -4892,7 +4945,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="162" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="162" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A162" s="3" t="s">
         <v>22</v>
       </c>
@@ -4918,7 +4971,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="163" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="163" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A163" s="3" t="s">
         <v>29</v>
       </c>
@@ -4944,7 +4997,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="164" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="164" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A164" s="3" t="s">
         <v>8</v>
       </c>
@@ -4970,7 +5023,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="165" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="165" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A165" s="3" t="s">
         <v>17</v>
       </c>
@@ -4996,7 +5049,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="166" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="166" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A166" s="3" t="s">
         <v>21</v>
       </c>
@@ -5022,7 +5075,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="167" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="167" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A167" s="3" t="s">
         <v>14</v>
       </c>
@@ -5048,7 +5101,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="168" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="168" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A168" s="3" t="s">
         <v>23</v>
       </c>
@@ -5074,7 +5127,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="169" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="169" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A169" s="3" t="s">
         <v>18</v>
       </c>
@@ -5100,7 +5153,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="170" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="170" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A170" s="3" t="s">
         <v>20</v>
       </c>
@@ -5126,7 +5179,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="171" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="171" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A171" s="3" t="s">
         <v>12</v>
       </c>
@@ -5152,7 +5205,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="172" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="172" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A172" s="3" t="s">
         <v>27</v>
       </c>
@@ -5178,7 +5231,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="173" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="173" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A173" s="3" t="s">
         <v>28</v>
       </c>
@@ -5204,8 +5257,8 @@
         <v>10</v>
       </c>
     </row>
-    <row r="175" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A175" s="13" t="s">
+    <row r="175" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A175" s="22" t="s">
         <v>0</v>
       </c>
       <c r="B175" s="1">
@@ -5230,8 +5283,8 @@
         <v>46229</v>
       </c>
     </row>
-    <row r="176" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A176" s="13"/>
+    <row r="176" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A176" s="22"/>
       <c r="B176" s="2" t="s">
         <v>1</v>
       </c>
@@ -5254,7 +5307,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="177" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="177" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A177" s="3" t="s">
         <v>22</v>
       </c>
@@ -5280,7 +5333,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="178" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="178" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A178" s="3" t="s">
         <v>29</v>
       </c>
@@ -5306,7 +5359,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="179" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="179" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A179" s="3" t="s">
         <v>12</v>
       </c>
@@ -5332,7 +5385,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="180" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="180" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A180" s="3" t="s">
         <v>21</v>
       </c>
@@ -5358,7 +5411,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="181" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="181" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A181" s="3" t="s">
         <v>23</v>
       </c>
@@ -5384,7 +5437,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="182" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="182" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A182" s="3" t="s">
         <v>18</v>
       </c>
@@ -5410,7 +5463,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="183" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="183" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A183" s="3" t="s">
         <v>17</v>
       </c>
@@ -5436,7 +5489,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="184" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="184" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A184" s="3" t="s">
         <v>14</v>
       </c>
@@ -5462,7 +5515,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="185" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="185" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A185" s="3" t="s">
         <v>8</v>
       </c>
@@ -5488,7 +5541,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="186" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="186" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A186" s="3" t="s">
         <v>20</v>
       </c>
@@ -5514,7 +5567,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="187" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="187" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A187" s="3" t="s">
         <v>28</v>
       </c>
@@ -5540,7 +5593,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="188" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="188" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A188" s="3" t="s">
         <v>27</v>
       </c>
@@ -5566,8 +5619,8 @@
         <v>34</v>
       </c>
     </row>
-    <row r="190" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A190" s="13" t="s">
+    <row r="190" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A190" s="22" t="s">
         <v>0</v>
       </c>
       <c r="B190" s="1">
@@ -5592,8 +5645,8 @@
         <v>46236</v>
       </c>
     </row>
-    <row r="191" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A191" s="13"/>
+    <row r="191" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A191" s="22"/>
       <c r="B191" s="2" t="s">
         <v>1</v>
       </c>
@@ -5616,34 +5669,34 @@
         <v>7</v>
       </c>
     </row>
-    <row r="192" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="192" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A192" s="3" t="s">
         <v>22</v>
       </c>
-      <c r="B192" s="18" t="s">
-        <v>9</v>
-      </c>
-      <c r="C192" s="18" t="s">
-        <v>9</v>
-      </c>
-      <c r="D192" s="18" t="s">
-        <v>9</v>
-      </c>
-      <c r="E192" s="18" t="s">
-        <v>9</v>
-      </c>
-      <c r="F192" s="18" t="s">
-        <v>9</v>
-      </c>
-      <c r="G192" s="19" t="s">
-        <v>9</v>
-      </c>
-      <c r="H192" s="20" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="193" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A193" s="21" t="s">
+      <c r="B192" s="13" t="s">
+        <v>9</v>
+      </c>
+      <c r="C192" s="13" t="s">
+        <v>9</v>
+      </c>
+      <c r="D192" s="13" t="s">
+        <v>9</v>
+      </c>
+      <c r="E192" s="13" t="s">
+        <v>9</v>
+      </c>
+      <c r="F192" s="13" t="s">
+        <v>9</v>
+      </c>
+      <c r="G192" s="14" t="s">
+        <v>9</v>
+      </c>
+      <c r="H192" s="15" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="193" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A193" s="16" t="s">
         <v>29</v>
       </c>
       <c r="B193" s="4" t="s">
@@ -5661,15 +5714,15 @@
       <c r="F193" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="G193" s="20" t="s">
-        <v>10</v>
-      </c>
-      <c r="H193" s="19" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="194" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A194" s="21" t="s">
+      <c r="G193" s="15" t="s">
+        <v>10</v>
+      </c>
+      <c r="H193" s="14" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="194" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A194" s="16" t="s">
         <v>14</v>
       </c>
       <c r="B194" s="4" t="s">
@@ -5687,15 +5740,15 @@
       <c r="F194" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="G194" s="20" t="s">
+      <c r="G194" s="15" t="s">
         <v>10</v>
       </c>
       <c r="H194" s="4" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="195" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A195" s="21" t="s">
+    <row r="195" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A195" s="16" t="s">
         <v>8</v>
       </c>
       <c r="B195" s="4" t="s">
@@ -5713,41 +5766,41 @@
       <c r="F195" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="G195" s="19" t="s">
-        <v>9</v>
-      </c>
-      <c r="H195" s="20" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="196" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A196" s="22" t="s">
+      <c r="G195" s="15" t="s">
+        <v>10</v>
+      </c>
+      <c r="H195" s="14" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="196" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A196" s="17" t="s">
         <v>20</v>
       </c>
-      <c r="B196" s="19" t="s">
-        <v>9</v>
-      </c>
-      <c r="C196" s="19" t="s">
-        <v>9</v>
-      </c>
-      <c r="D196" s="19" t="s">
-        <v>9</v>
-      </c>
-      <c r="E196" s="19" t="s">
-        <v>9</v>
-      </c>
-      <c r="F196" s="19" t="s">
-        <v>9</v>
-      </c>
-      <c r="G196" s="20" t="s">
-        <v>10</v>
-      </c>
-      <c r="H196" s="19" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="197" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A197" s="23" t="s">
+      <c r="B196" s="14" t="s">
+        <v>9</v>
+      </c>
+      <c r="C196" s="14" t="s">
+        <v>9</v>
+      </c>
+      <c r="D196" s="14" t="s">
+        <v>9</v>
+      </c>
+      <c r="E196" s="14" t="s">
+        <v>9</v>
+      </c>
+      <c r="F196" s="14" t="s">
+        <v>9</v>
+      </c>
+      <c r="G196" s="15" t="s">
+        <v>10</v>
+      </c>
+      <c r="H196" s="14" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="197" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A197" s="18" t="s">
         <v>23</v>
       </c>
       <c r="B197" s="4" t="s">
@@ -5759,47 +5812,47 @@
       <c r="D197" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="E197" s="24" t="s">
+      <c r="E197" s="19" t="s">
         <v>35</v>
       </c>
       <c r="F197" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="G197" s="20" t="s">
-        <v>10</v>
-      </c>
-      <c r="H197" s="19" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="198" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A198" s="22" t="s">
+      <c r="G197" s="14" t="s">
+        <v>9</v>
+      </c>
+      <c r="H197" s="15" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="198" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A198" s="17" t="s">
         <v>12</v>
       </c>
-      <c r="B198" s="19" t="s">
-        <v>11</v>
-      </c>
-      <c r="C198" s="19" t="s">
-        <v>11</v>
-      </c>
-      <c r="D198" s="19" t="s">
-        <v>11</v>
-      </c>
-      <c r="E198" s="19" t="s">
-        <v>11</v>
-      </c>
-      <c r="F198" s="19" t="s">
-        <v>11</v>
-      </c>
-      <c r="G198" s="19" t="s">
-        <v>11</v>
-      </c>
-      <c r="H198" s="20" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="199" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A199" s="21" t="s">
+      <c r="B198" s="14" t="s">
+        <v>11</v>
+      </c>
+      <c r="C198" s="14" t="s">
+        <v>11</v>
+      </c>
+      <c r="D198" s="14" t="s">
+        <v>11</v>
+      </c>
+      <c r="E198" s="14" t="s">
+        <v>11</v>
+      </c>
+      <c r="F198" s="14" t="s">
+        <v>11</v>
+      </c>
+      <c r="G198" s="14" t="s">
+        <v>11</v>
+      </c>
+      <c r="H198" s="15" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="199" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A199" s="16" t="s">
         <v>21</v>
       </c>
       <c r="B199" s="4" t="s">
@@ -5814,18 +5867,18 @@
       <c r="E199" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="F199" s="24" t="s">
+      <c r="F199" s="19" t="s">
         <v>35</v>
       </c>
-      <c r="G199" s="20" t="s">
-        <v>10</v>
-      </c>
-      <c r="H199" s="19" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="200" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A200" s="21" t="s">
+      <c r="G199" s="15" t="s">
+        <v>10</v>
+      </c>
+      <c r="H199" s="14" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="200" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A200" s="16" t="s">
         <v>18</v>
       </c>
       <c r="B200" s="4" t="s">
@@ -5843,14 +5896,14 @@
       <c r="F200" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="G200" s="19" t="s">
-        <v>11</v>
-      </c>
-      <c r="H200" s="20" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="201" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="G200" s="14" t="s">
+        <v>11</v>
+      </c>
+      <c r="H200" s="15" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="201" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A201" s="3" t="s">
         <v>17</v>
       </c>
@@ -5872,12 +5925,12 @@
       <c r="G201" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="H201" s="20" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="202" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A202" s="21" t="s">
+      <c r="H201" s="15" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="202" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A202" s="16" t="s">
         <v>27</v>
       </c>
       <c r="B202" s="4" t="s">
@@ -5895,41 +5948,46 @@
       <c r="F202" s="4" t="s">
         <v>31</v>
       </c>
-      <c r="G202" s="20" t="s">
-        <v>10</v>
-      </c>
-      <c r="H202" s="20" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="203" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="G202" s="15" t="s">
+        <v>10</v>
+      </c>
+      <c r="H202" s="15" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="203" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A203" s="3" t="s">
         <v>28</v>
       </c>
-      <c r="B203" s="25" t="s">
+      <c r="B203" s="20" t="s">
         <v>33</v>
       </c>
-      <c r="C203" s="25" t="s">
+      <c r="C203" s="20" t="s">
         <v>33</v>
       </c>
-      <c r="D203" s="25" t="s">
+      <c r="D203" s="20" t="s">
         <v>33</v>
       </c>
-      <c r="E203" s="25" t="s">
+      <c r="E203" s="20" t="s">
         <v>33</v>
       </c>
-      <c r="F203" s="25" t="s">
+      <c r="F203" s="20" t="s">
         <v>33</v>
       </c>
-      <c r="G203" s="26" t="s">
+      <c r="G203" s="21" t="s">
         <v>34</v>
       </c>
-      <c r="H203" s="26" t="s">
+      <c r="H203" s="21" t="s">
         <v>34</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="15">
+    <mergeCell ref="A1:A2"/>
+    <mergeCell ref="A14:A15"/>
+    <mergeCell ref="A27:A28"/>
+    <mergeCell ref="A40:A41"/>
+    <mergeCell ref="A53:A54"/>
     <mergeCell ref="A190:A191"/>
     <mergeCell ref="G84:H84"/>
     <mergeCell ref="A66:A67"/>
@@ -5938,20 +5996,36 @@
     <mergeCell ref="A92:A93"/>
     <mergeCell ref="A79:A80"/>
     <mergeCell ref="A175:A176"/>
-    <mergeCell ref="A1:A2"/>
-    <mergeCell ref="A14:A15"/>
-    <mergeCell ref="A27:A28"/>
-    <mergeCell ref="A40:A41"/>
-    <mergeCell ref="A53:A54"/>
     <mergeCell ref="A160:A161"/>
     <mergeCell ref="A145:A146"/>
   </mergeCells>
   <phoneticPr fontId="7" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId1"/>
 </worksheet>
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="9d4e7416-6feb-444a-9f0d-6e119e2a4ded">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="ab20b492-db1c-4b70-84db-283da62d5dcb" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100A49D20B196870C459C080BD3A88F41F5" ma:contentTypeVersion="12" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="c891d3af3c5d8789d4a1386f5525110a">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="9d4e7416-6feb-444a-9f0d-6e119e2a4ded" xmlns:ns3="ab20b492-db1c-4b70-84db-283da62d5dcb" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="a2d778173b158e0f4887e6c1a7be78b9" ns2:_="" ns3:_="">
     <xsd:import namespace="9d4e7416-6feb-444a-9f0d-6e119e2a4ded"/>
@@ -6152,27 +6226,26 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{3E7BE3CC-8834-4B2B-B0A5-EDC239DF005F}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="9d4e7416-6feb-444a-9f0d-6e119e2a4ded"/>
+    <ds:schemaRef ds:uri="ab20b492-db1c-4b70-84db-283da62d5dcb"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="9d4e7416-6feb-444a-9f0d-6e119e2a4ded">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="ab20b492-db1c-4b70-84db-283da62d5dcb" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{3E90FB8C-E259-434B-8A97-2530AD5FA4BD}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9D90F563-717D-4F15-9FD2-892B1218D415}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -6189,23 +6262,4 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{3E90FB8C-E259-434B-8A97-2530AD5FA4BD}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{3E7BE3CC-8834-4B2B-B0A5-EDC239DF005F}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="9d4e7416-6feb-444a-9f0d-6e119e2a4ded"/>
-    <ds:schemaRef ds:uri="ab20b492-db1c-4b70-84db-283da62d5dcb"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
Actualizacion automatica de datos - vie 31/07/2026 16:32:02,54
</commit_message>
<xml_diff>
--- a/Horario/Horario 2026.xlsx
+++ b/Horario/Horario 2026.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://virtualsoftserv-my.sharepoint.com/personal/maria_sanchez_virtualsoft_tech/Documents/Indicadores y Pagina WEB/Horario/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="6_{6E17BD36-3E42-42F2-8AFD-92DB165A9BC2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="6" documentId="6_{6E17BD36-3E42-42F2-8AFD-92DB165A9BC2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{8BA25835-168D-4574-A6FF-3D390CF48E67}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{9AAEFA76-0198-46F6-BBF5-EADAB38A6758}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{9AAEFA76-0198-46F6-BBF5-EADAB38A6758}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1467" uniqueCount="36">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1659" uniqueCount="43">
   <si>
     <t>GESTOR</t>
   </si>
@@ -148,6 +148,27 @@
   <si>
     <t>Dia de Votación</t>
   </si>
+  <si>
+    <t>6am - 12pm / 4:30pm - 5:30pm</t>
+  </si>
+  <si>
+    <t>7am - 3pm</t>
+  </si>
+  <si>
+    <t>6am - 11am / 7pm - 9pm</t>
+  </si>
+  <si>
+    <t>1pm - 6pm / 9pm - 11pm</t>
+  </si>
+  <si>
+    <t>Incapacidad</t>
+  </si>
+  <si>
+    <t>11am - 7pm</t>
+  </si>
+  <si>
+    <t>1pm - 9pm</t>
+  </si>
 </sst>
 </file>
 
@@ -243,7 +264,7 @@
       <family val="2"/>
     </font>
   </fonts>
-  <fills count="12">
+  <fills count="13">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -307,6 +328,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="2" tint="-9.9978637043366805E-2"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.79998168889431442"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -391,7 +418,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="27">
+  <cellXfs count="40">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="16" fontId="2" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -436,6 +463,45 @@
     <xf numFmtId="0" fontId="5" fillId="11" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="12" fillId="10" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="16" fontId="2" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="7" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="10" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="12" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -839,18 +905,19 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4B1D5CB7-A214-4F9F-A075-10C6E5CC7E55}">
-  <dimension ref="A1:O203"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <dimension ref="A1:O232"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="19.5546875" bestFit="1" customWidth="1"/>
-    <col min="2" max="4" width="12" bestFit="1" customWidth="1"/>
-    <col min="5" max="6" width="16.5546875" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="17" bestFit="1" customWidth="1"/>
-    <col min="8" max="15" width="12" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="20.140625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="17" bestFit="1" customWidth="1"/>
+    <col min="3" max="4" width="12.42578125" bestFit="1" customWidth="1"/>
+    <col min="5" max="7" width="17" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="15.5703125" bestFit="1" customWidth="1"/>
+    <col min="9" max="15" width="12.42578125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:15" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A1" s="25" t="s">
+    <row r="1" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A1" s="38" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="1">
@@ -896,8 +963,8 @@
         <v>46138</v>
       </c>
     </row>
-    <row r="2" spans="1:15" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A2" s="26"/>
+    <row r="2" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A2" s="39"/>
       <c r="B2" s="2" t="s">
         <v>1</v>
       </c>
@@ -941,7 +1008,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="3" spans="1:15" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
         <v>8</v>
       </c>
@@ -988,7 +1055,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="4" spans="1:15" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A4" s="3" t="s">
         <v>12</v>
       </c>
@@ -1035,7 +1102,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="5" spans="1:15" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A5" s="3" t="s">
         <v>14</v>
       </c>
@@ -1082,7 +1149,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="6" spans="1:15" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A6" s="3" t="s">
         <v>15</v>
       </c>
@@ -1129,7 +1196,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="7" spans="1:15" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A7" s="3" t="s">
         <v>17</v>
       </c>
@@ -1176,7 +1243,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="8" spans="1:15" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A8" s="3" t="s">
         <v>18</v>
       </c>
@@ -1223,7 +1290,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="9" spans="1:15" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A9" s="3" t="s">
         <v>20</v>
       </c>
@@ -1270,7 +1337,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="10" spans="1:15" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A10" s="3" t="s">
         <v>21</v>
       </c>
@@ -1317,7 +1384,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="11" spans="1:15" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A11" s="3" t="s">
         <v>22</v>
       </c>
@@ -1364,7 +1431,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="12" spans="1:15" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A12" s="3" t="s">
         <v>23</v>
       </c>
@@ -1411,8 +1478,8 @@
         <v>9</v>
       </c>
     </row>
-    <row r="14" spans="1:15" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A14" s="25" t="s">
+    <row r="14" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A14" s="38" t="s">
         <v>0</v>
       </c>
       <c r="B14" s="1">
@@ -1437,8 +1504,8 @@
         <v>46145</v>
       </c>
     </row>
-    <row r="15" spans="1:15" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A15" s="26"/>
+    <row r="15" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A15" s="39"/>
       <c r="B15" s="2" t="s">
         <v>1</v>
       </c>
@@ -1461,7 +1528,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="16" spans="1:15" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A16" s="3" t="s">
         <v>17</v>
       </c>
@@ -1487,7 +1554,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="17" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A17" s="3" t="s">
         <v>8</v>
       </c>
@@ -1513,7 +1580,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="18" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A18" s="3" t="s">
         <v>12</v>
       </c>
@@ -1539,7 +1606,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="19" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A19" s="3" t="s">
         <v>15</v>
       </c>
@@ -1565,7 +1632,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="20" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A20" s="3" t="s">
         <v>18</v>
       </c>
@@ -1591,7 +1658,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="21" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A21" s="3" t="s">
         <v>23</v>
       </c>
@@ -1617,7 +1684,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="22" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A22" s="3" t="s">
         <v>21</v>
       </c>
@@ -1643,7 +1710,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="23" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A23" s="3" t="s">
         <v>22</v>
       </c>
@@ -1669,7 +1736,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="24" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A24" s="3" t="s">
         <v>14</v>
       </c>
@@ -1695,7 +1762,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="25" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A25" s="3" t="s">
         <v>20</v>
       </c>
@@ -1721,8 +1788,8 @@
         <v>10</v>
       </c>
     </row>
-    <row r="27" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A27" s="25" t="s">
+    <row r="27" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A27" s="38" t="s">
         <v>0</v>
       </c>
       <c r="B27" s="1">
@@ -1747,8 +1814,8 @@
         <v>46152</v>
       </c>
     </row>
-    <row r="28" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A28" s="26"/>
+    <row r="28" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A28" s="39"/>
       <c r="B28" s="2" t="s">
         <v>1</v>
       </c>
@@ -1771,7 +1838,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="29" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A29" s="3" t="s">
         <v>22</v>
       </c>
@@ -1797,7 +1864,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="30" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A30" s="3" t="s">
         <v>14</v>
       </c>
@@ -1823,7 +1890,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="31" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A31" s="3" t="s">
         <v>20</v>
       </c>
@@ -1849,7 +1916,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="32" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A32" s="3" t="s">
         <v>15</v>
       </c>
@@ -1875,7 +1942,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="33" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A33" s="3" t="s">
         <v>18</v>
       </c>
@@ -1901,7 +1968,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="34" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A34" s="3" t="s">
         <v>21</v>
       </c>
@@ -1927,7 +1994,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="35" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A35" s="3" t="s">
         <v>8</v>
       </c>
@@ -1953,7 +2020,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="36" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A36" s="3" t="s">
         <v>12</v>
       </c>
@@ -1979,7 +2046,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="37" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A37" s="3" t="s">
         <v>23</v>
       </c>
@@ -2005,7 +2072,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="38" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A38" s="3" t="s">
         <v>17</v>
       </c>
@@ -2031,8 +2098,8 @@
         <v>10</v>
       </c>
     </row>
-    <row r="40" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A40" s="22" t="s">
+    <row r="40" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A40" s="35" t="s">
         <v>0</v>
       </c>
       <c r="B40" s="1">
@@ -2057,8 +2124,8 @@
         <v>46159</v>
       </c>
     </row>
-    <row r="41" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A41" s="22"/>
+    <row r="41" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A41" s="35"/>
       <c r="B41" s="2" t="s">
         <v>1</v>
       </c>
@@ -2081,7 +2148,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="42" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A42" s="3" t="s">
         <v>22</v>
       </c>
@@ -2107,7 +2174,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="43" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A43" s="3" t="s">
         <v>12</v>
       </c>
@@ -2133,7 +2200,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="44" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A44" s="3" t="s">
         <v>18</v>
       </c>
@@ -2159,7 +2226,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="45" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A45" s="3" t="s">
         <v>23</v>
       </c>
@@ -2185,7 +2252,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="46" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A46" s="3" t="s">
         <v>15</v>
       </c>
@@ -2211,7 +2278,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="47" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A47" s="3" t="s">
         <v>24</v>
       </c>
@@ -2237,7 +2304,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="48" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A48" s="3" t="s">
         <v>14</v>
       </c>
@@ -2263,7 +2330,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="49" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A49" s="3" t="s">
         <v>21</v>
       </c>
@@ -2289,7 +2356,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="50" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="50" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A50" s="3" t="s">
         <v>20</v>
       </c>
@@ -2315,7 +2382,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="51" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="51" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A51" s="3" t="s">
         <v>8</v>
       </c>
@@ -2341,8 +2408,8 @@
         <v>9</v>
       </c>
     </row>
-    <row r="53" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A53" s="22" t="s">
+    <row r="53" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A53" s="35" t="s">
         <v>0</v>
       </c>
       <c r="B53" s="1">
@@ -2367,8 +2434,8 @@
         <v>46166</v>
       </c>
     </row>
-    <row r="54" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A54" s="22"/>
+    <row r="54" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A54" s="35"/>
       <c r="B54" s="2" t="s">
         <v>1</v>
       </c>
@@ -2391,7 +2458,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="55" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="55" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A55" s="3" t="s">
         <v>22</v>
       </c>
@@ -2417,7 +2484,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="56" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="56" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A56" s="3" t="s">
         <v>14</v>
       </c>
@@ -2443,7 +2510,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="57" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="57" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A57" s="3" t="s">
         <v>17</v>
       </c>
@@ -2469,7 +2536,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="58" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="58" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A58" s="3" t="s">
         <v>18</v>
       </c>
@@ -2495,7 +2562,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="59" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="59" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A59" s="3" t="s">
         <v>23</v>
       </c>
@@ -2521,7 +2588,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="60" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="60" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A60" s="3" t="s">
         <v>21</v>
       </c>
@@ -2547,7 +2614,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="61" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="61" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A61" s="3" t="s">
         <v>8</v>
       </c>
@@ -2573,7 +2640,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="62" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="62" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A62" s="3" t="s">
         <v>12</v>
       </c>
@@ -2599,7 +2666,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="63" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="63" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A63" s="3" t="s">
         <v>20</v>
       </c>
@@ -2625,7 +2692,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="64" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="64" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A64" s="3" t="s">
         <v>15</v>
       </c>
@@ -2651,8 +2718,8 @@
         <v>19</v>
       </c>
     </row>
-    <row r="66" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A66" s="22" t="s">
+    <row r="66" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A66" s="35" t="s">
         <v>0</v>
       </c>
       <c r="B66" s="1">
@@ -2677,8 +2744,8 @@
         <v>46173</v>
       </c>
     </row>
-    <row r="67" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A67" s="22"/>
+    <row r="67" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A67" s="35"/>
       <c r="B67" s="2" t="s">
         <v>1</v>
       </c>
@@ -2701,7 +2768,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="68" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="68" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A68" s="3" t="s">
         <v>22</v>
       </c>
@@ -2727,7 +2794,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="69" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="69" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A69" s="3" t="s">
         <v>21</v>
       </c>
@@ -2753,7 +2820,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="70" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="70" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A70" s="3" t="s">
         <v>8</v>
       </c>
@@ -2779,7 +2846,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="71" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="71" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A71" s="3" t="s">
         <v>18</v>
       </c>
@@ -2805,7 +2872,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="72" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="72" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A72" s="3" t="s">
         <v>20</v>
       </c>
@@ -2831,7 +2898,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="73" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="73" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A73" s="3" t="s">
         <v>15</v>
       </c>
@@ -2857,7 +2924,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="74" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="74" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A74" s="3" t="s">
         <v>14</v>
       </c>
@@ -2883,7 +2950,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="75" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="75" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A75" s="3" t="s">
         <v>17</v>
       </c>
@@ -2909,7 +2976,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="76" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="76" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A76" s="3" t="s">
         <v>23</v>
       </c>
@@ -2935,7 +3002,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="77" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="77" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A77" s="3" t="s">
         <v>12</v>
       </c>
@@ -2961,8 +3028,8 @@
         <v>10</v>
       </c>
     </row>
-    <row r="79" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A79" s="22" t="s">
+    <row r="79" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A79" s="35" t="s">
         <v>0</v>
       </c>
       <c r="B79" s="1">
@@ -2987,8 +3054,8 @@
         <v>46180</v>
       </c>
     </row>
-    <row r="80" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A80" s="22"/>
+    <row r="80" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A80" s="35"/>
       <c r="B80" s="2" t="s">
         <v>1</v>
       </c>
@@ -3011,7 +3078,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="81" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="81" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A81" s="3" t="s">
         <v>22</v>
       </c>
@@ -3037,7 +3104,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="82" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="82" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A82" s="3" t="s">
         <v>14</v>
       </c>
@@ -3063,7 +3130,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="83" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="83" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A83" s="3" t="s">
         <v>12</v>
       </c>
@@ -3089,7 +3156,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="84" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="84" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A84" s="3" t="s">
         <v>15</v>
       </c>
@@ -3108,10 +3175,10 @@
       <c r="F84" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="G84" s="23"/>
-      <c r="H84" s="24"/>
-    </row>
-    <row r="85" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="G84" s="36"/>
+      <c r="H84" s="37"/>
+    </row>
+    <row r="85" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A85" s="3" t="s">
         <v>17</v>
       </c>
@@ -3137,7 +3204,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="86" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="86" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A86" s="3" t="s">
         <v>18</v>
       </c>
@@ -3163,7 +3230,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="87" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="87" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A87" s="3" t="s">
         <v>21</v>
       </c>
@@ -3189,7 +3256,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="88" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="88" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A88" s="3" t="s">
         <v>8</v>
       </c>
@@ -3215,7 +3282,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="89" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="89" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A89" s="3" t="s">
         <v>20</v>
       </c>
@@ -3241,7 +3308,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="90" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="90" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A90" s="3" t="s">
         <v>23</v>
       </c>
@@ -3267,8 +3334,8 @@
         <v>10</v>
       </c>
     </row>
-    <row r="92" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A92" s="22" t="s">
+    <row r="92" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A92" s="35" t="s">
         <v>0</v>
       </c>
       <c r="B92" s="1">
@@ -3293,8 +3360,8 @@
         <v>46187</v>
       </c>
     </row>
-    <row r="93" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A93" s="22"/>
+    <row r="93" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A93" s="35"/>
       <c r="B93" s="2" t="s">
         <v>1</v>
       </c>
@@ -3317,7 +3384,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="94" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="94" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A94" s="3" t="s">
         <v>22</v>
       </c>
@@ -3343,7 +3410,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="95" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="95" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A95" s="3" t="s">
         <v>21</v>
       </c>
@@ -3369,7 +3436,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="96" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="96" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A96" s="3" t="s">
         <v>8</v>
       </c>
@@ -3395,7 +3462,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="97" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="97" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A97" s="3" t="s">
         <v>23</v>
       </c>
@@ -3421,7 +3488,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="98" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="98" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A98" s="3" t="s">
         <v>18</v>
       </c>
@@ -3447,7 +3514,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="99" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="99" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A99" s="3" t="s">
         <v>14</v>
       </c>
@@ -3473,7 +3540,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="100" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="100" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A100" s="3" t="s">
         <v>12</v>
       </c>
@@ -3499,7 +3566,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="101" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="101" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A101" s="3" t="s">
         <v>20</v>
       </c>
@@ -3525,7 +3592,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="102" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="102" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A102" s="3" t="s">
         <v>17</v>
       </c>
@@ -3551,8 +3618,8 @@
         <v>10</v>
       </c>
     </row>
-    <row r="104" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A104" s="22" t="s">
+    <row r="104" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A104" s="35" t="s">
         <v>0</v>
       </c>
       <c r="B104" s="1">
@@ -3577,8 +3644,8 @@
         <v>46194</v>
       </c>
     </row>
-    <row r="105" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A105" s="22"/>
+    <row r="105" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A105" s="35"/>
       <c r="B105" s="2" t="s">
         <v>1</v>
       </c>
@@ -3601,7 +3668,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="106" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="106" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A106" s="3" t="s">
         <v>22</v>
       </c>
@@ -3627,7 +3694,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="107" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="107" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A107" s="3" t="s">
         <v>12</v>
       </c>
@@ -3653,7 +3720,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="108" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="108" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A108" s="3" t="s">
         <v>17</v>
       </c>
@@ -3679,7 +3746,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="109" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="109" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A109" s="3" t="s">
         <v>20</v>
       </c>
@@ -3705,7 +3772,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="110" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="110" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A110" s="3" t="s">
         <v>23</v>
       </c>
@@ -3731,7 +3798,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="111" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="111" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A111" s="3" t="s">
         <v>18</v>
       </c>
@@ -3757,7 +3824,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="112" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="112" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A112" s="3" t="s">
         <v>14</v>
       </c>
@@ -3783,7 +3850,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="113" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="113" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A113" s="3" t="s">
         <v>8</v>
       </c>
@@ -3809,7 +3876,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="114" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="114" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A114" s="3" t="s">
         <v>21</v>
       </c>
@@ -3835,8 +3902,8 @@
         <v>10</v>
       </c>
     </row>
-    <row r="116" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A116" s="22" t="s">
+    <row r="116" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A116" s="35" t="s">
         <v>0</v>
       </c>
       <c r="B116" s="1">
@@ -3861,8 +3928,8 @@
         <v>46201</v>
       </c>
     </row>
-    <row r="117" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A117" s="22"/>
+    <row r="117" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A117" s="35"/>
       <c r="B117" s="2" t="s">
         <v>1</v>
       </c>
@@ -3885,7 +3952,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="118" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="118" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A118" s="3" t="s">
         <v>8</v>
       </c>
@@ -3911,7 +3978,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="119" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="119" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A119" s="3" t="s">
         <v>22</v>
       </c>
@@ -3937,7 +4004,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="120" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="120" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A120" s="3" t="s">
         <v>18</v>
       </c>
@@ -3963,7 +4030,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="121" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="121" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A121" s="3" t="s">
         <v>23</v>
       </c>
@@ -3989,7 +4056,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="122" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="122" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A122" s="3" t="s">
         <v>21</v>
       </c>
@@ -4015,7 +4082,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="123" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="123" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A123" s="3" t="s">
         <v>12</v>
       </c>
@@ -4041,7 +4108,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="124" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="124" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A124" s="3" t="s">
         <v>17</v>
       </c>
@@ -4067,7 +4134,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="125" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="125" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A125" s="3" t="s">
         <v>20</v>
       </c>
@@ -4093,7 +4160,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="126" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="126" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A126" s="3" t="s">
         <v>14</v>
       </c>
@@ -4119,7 +4186,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="127" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="127" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A127" s="3" t="s">
         <v>27</v>
       </c>
@@ -4145,7 +4212,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="128" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="128" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A128" s="3" t="s">
         <v>28</v>
       </c>
@@ -4171,7 +4238,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="130" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="130" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A130" s="11" t="s">
         <v>0</v>
       </c>
@@ -4197,7 +4264,7 @@
         <v>46208</v>
       </c>
     </row>
-    <row r="131" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="131" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A131" s="11"/>
       <c r="B131" s="2" t="s">
         <v>1</v>
@@ -4221,7 +4288,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="132" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="132" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A132" s="3" t="s">
         <v>22</v>
       </c>
@@ -4247,7 +4314,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="133" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="133" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A133" s="3" t="s">
         <v>29</v>
       </c>
@@ -4273,7 +4340,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="134" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="134" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A134" s="3" t="s">
         <v>12</v>
       </c>
@@ -4299,7 +4366,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="135" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="135" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A135" s="3" t="s">
         <v>17</v>
       </c>
@@ -4325,7 +4392,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="136" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="136" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A136" s="3" t="s">
         <v>20</v>
       </c>
@@ -4351,7 +4418,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="137" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="137" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A137" s="3" t="s">
         <v>14</v>
       </c>
@@ -4377,7 +4444,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="138" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="138" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A138" s="3" t="s">
         <v>18</v>
       </c>
@@ -4403,7 +4470,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="139" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="139" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A139" s="3" t="s">
         <v>23</v>
       </c>
@@ -4429,7 +4496,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="140" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="140" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A140" s="3" t="s">
         <v>21</v>
       </c>
@@ -4455,7 +4522,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="141" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="141" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A141" s="3" t="s">
         <v>8</v>
       </c>
@@ -4481,7 +4548,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="142" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="142" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A142" s="3" t="s">
         <v>27</v>
       </c>
@@ -4507,7 +4574,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="143" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="143" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A143" s="3" t="s">
         <v>28</v>
       </c>
@@ -4533,8 +4600,8 @@
         <v>10</v>
       </c>
     </row>
-    <row r="145" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A145" s="22" t="s">
+    <row r="145" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A145" s="35" t="s">
         <v>0</v>
       </c>
       <c r="B145" s="1">
@@ -4559,8 +4626,8 @@
         <v>46215</v>
       </c>
     </row>
-    <row r="146" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A146" s="22"/>
+    <row r="146" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A146" s="35"/>
       <c r="B146" s="2" t="s">
         <v>1</v>
       </c>
@@ -4583,7 +4650,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="147" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="147" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A147" s="3" t="s">
         <v>22</v>
       </c>
@@ -4609,7 +4676,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="148" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="148" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A148" s="3" t="s">
         <v>29</v>
       </c>
@@ -4635,7 +4702,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="149" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="149" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A149" s="3" t="s">
         <v>14</v>
       </c>
@@ -4661,7 +4728,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="150" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="150" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A150" s="3" t="s">
         <v>18</v>
       </c>
@@ -4687,7 +4754,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="151" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="151" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A151" s="3" t="s">
         <v>20</v>
       </c>
@@ -4713,7 +4780,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="152" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="152" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A152" s="3" t="s">
         <v>21</v>
       </c>
@@ -4739,7 +4806,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="153" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="153" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A153" s="3" t="s">
         <v>12</v>
       </c>
@@ -4765,7 +4832,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="154" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="154" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A154" s="3" t="s">
         <v>8</v>
       </c>
@@ -4791,7 +4858,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="155" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="155" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A155" s="3" t="s">
         <v>17</v>
       </c>
@@ -4817,7 +4884,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="156" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="156" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A156" s="3" t="s">
         <v>23</v>
       </c>
@@ -4843,7 +4910,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="157" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="157" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A157" s="3" t="s">
         <v>27</v>
       </c>
@@ -4869,7 +4936,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="158" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="158" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A158" s="3" t="s">
         <v>28</v>
       </c>
@@ -4895,8 +4962,8 @@
         <v>11</v>
       </c>
     </row>
-    <row r="160" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A160" s="22" t="s">
+    <row r="160" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A160" s="35" t="s">
         <v>0</v>
       </c>
       <c r="B160" s="1">
@@ -4921,8 +4988,8 @@
         <v>46222</v>
       </c>
     </row>
-    <row r="161" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A161" s="22"/>
+    <row r="161" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A161" s="35"/>
       <c r="B161" s="2" t="s">
         <v>1</v>
       </c>
@@ -4945,7 +5012,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="162" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="162" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A162" s="3" t="s">
         <v>22</v>
       </c>
@@ -4971,7 +5038,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="163" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="163" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A163" s="3" t="s">
         <v>29</v>
       </c>
@@ -4997,7 +5064,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="164" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="164" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A164" s="3" t="s">
         <v>8</v>
       </c>
@@ -5023,7 +5090,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="165" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="165" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A165" s="3" t="s">
         <v>17</v>
       </c>
@@ -5049,7 +5116,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="166" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="166" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A166" s="3" t="s">
         <v>21</v>
       </c>
@@ -5075,7 +5142,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="167" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="167" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A167" s="3" t="s">
         <v>14</v>
       </c>
@@ -5101,7 +5168,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="168" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="168" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A168" s="3" t="s">
         <v>23</v>
       </c>
@@ -5127,7 +5194,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="169" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="169" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A169" s="3" t="s">
         <v>18</v>
       </c>
@@ -5153,7 +5220,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="170" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="170" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A170" s="3" t="s">
         <v>20</v>
       </c>
@@ -5179,7 +5246,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="171" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="171" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A171" s="3" t="s">
         <v>12</v>
       </c>
@@ -5205,7 +5272,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="172" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="172" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A172" s="3" t="s">
         <v>27</v>
       </c>
@@ -5231,7 +5298,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="173" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="173" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A173" s="3" t="s">
         <v>28</v>
       </c>
@@ -5257,8 +5324,8 @@
         <v>10</v>
       </c>
     </row>
-    <row r="175" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A175" s="22" t="s">
+    <row r="175" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A175" s="35" t="s">
         <v>0</v>
       </c>
       <c r="B175" s="1">
@@ -5283,8 +5350,8 @@
         <v>46229</v>
       </c>
     </row>
-    <row r="176" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A176" s="22"/>
+    <row r="176" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A176" s="35"/>
       <c r="B176" s="2" t="s">
         <v>1</v>
       </c>
@@ -5307,7 +5374,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="177" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="177" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A177" s="3" t="s">
         <v>22</v>
       </c>
@@ -5333,7 +5400,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="178" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="178" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A178" s="3" t="s">
         <v>29</v>
       </c>
@@ -5359,7 +5426,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="179" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="179" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A179" s="3" t="s">
         <v>12</v>
       </c>
@@ -5385,7 +5452,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="180" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="180" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A180" s="3" t="s">
         <v>21</v>
       </c>
@@ -5411,7 +5478,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="181" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="181" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A181" s="3" t="s">
         <v>23</v>
       </c>
@@ -5437,7 +5504,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="182" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="182" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A182" s="3" t="s">
         <v>18</v>
       </c>
@@ -5463,7 +5530,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="183" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="183" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A183" s="3" t="s">
         <v>17</v>
       </c>
@@ -5489,7 +5556,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="184" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="184" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A184" s="3" t="s">
         <v>14</v>
       </c>
@@ -5515,7 +5582,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="185" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="185" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A185" s="3" t="s">
         <v>8</v>
       </c>
@@ -5541,7 +5608,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="186" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="186" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A186" s="3" t="s">
         <v>20</v>
       </c>
@@ -5567,7 +5634,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="187" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="187" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A187" s="3" t="s">
         <v>28</v>
       </c>
@@ -5593,7 +5660,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="188" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="188" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A188" s="3" t="s">
         <v>27</v>
       </c>
@@ -5619,8 +5686,8 @@
         <v>34</v>
       </c>
     </row>
-    <row r="190" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A190" s="22" t="s">
+    <row r="190" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A190" s="35" t="s">
         <v>0</v>
       </c>
       <c r="B190" s="1">
@@ -5645,8 +5712,8 @@
         <v>46236</v>
       </c>
     </row>
-    <row r="191" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A191" s="22"/>
+    <row r="191" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A191" s="35"/>
       <c r="B191" s="2" t="s">
         <v>1</v>
       </c>
@@ -5669,7 +5736,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="192" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="192" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A192" s="3" t="s">
         <v>22</v>
       </c>
@@ -5695,7 +5762,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="193" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="193" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A193" s="16" t="s">
         <v>29</v>
       </c>
@@ -5721,7 +5788,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="194" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="194" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A194" s="16" t="s">
         <v>14</v>
       </c>
@@ -5747,7 +5814,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="195" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="195" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A195" s="16" t="s">
         <v>8</v>
       </c>
@@ -5773,7 +5840,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="196" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="196" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A196" s="17" t="s">
         <v>20</v>
       </c>
@@ -5799,7 +5866,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="197" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="197" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A197" s="18" t="s">
         <v>23</v>
       </c>
@@ -5825,7 +5892,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="198" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="198" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A198" s="17" t="s">
         <v>12</v>
       </c>
@@ -5851,7 +5918,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="199" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="199" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A199" s="16" t="s">
         <v>21</v>
       </c>
@@ -5877,7 +5944,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="200" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="200" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A200" s="16" t="s">
         <v>18</v>
       </c>
@@ -5903,7 +5970,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="201" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="201" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A201" s="3" t="s">
         <v>17</v>
       </c>
@@ -5929,7 +5996,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="202" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="202" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A202" s="16" t="s">
         <v>27</v>
       </c>
@@ -5955,7 +6022,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="203" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="203" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A203" s="3" t="s">
         <v>28</v>
       </c>
@@ -5981,13 +6048,707 @@
         <v>34</v>
       </c>
     </row>
+    <row r="205" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A205" s="33" t="s">
+        <v>0</v>
+      </c>
+      <c r="B205" s="22">
+        <v>46237</v>
+      </c>
+      <c r="C205" s="22">
+        <v>46238</v>
+      </c>
+      <c r="D205" s="22">
+        <v>46239</v>
+      </c>
+      <c r="E205" s="22">
+        <v>46240</v>
+      </c>
+      <c r="F205" s="22">
+        <v>46241</v>
+      </c>
+      <c r="G205" s="22">
+        <v>46242</v>
+      </c>
+      <c r="H205" s="22">
+        <v>46243</v>
+      </c>
+    </row>
+    <row r="206" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A206" s="34"/>
+      <c r="B206" s="23" t="s">
+        <v>1</v>
+      </c>
+      <c r="C206" s="23" t="s">
+        <v>2</v>
+      </c>
+      <c r="D206" s="23" t="s">
+        <v>3</v>
+      </c>
+      <c r="E206" s="23" t="s">
+        <v>4</v>
+      </c>
+      <c r="F206" s="23" t="s">
+        <v>5</v>
+      </c>
+      <c r="G206" s="23" t="s">
+        <v>6</v>
+      </c>
+      <c r="H206" s="23" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="207" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A207" s="23" t="s">
+        <v>22</v>
+      </c>
+      <c r="B207" s="24" t="s">
+        <v>9</v>
+      </c>
+      <c r="C207" s="24" t="s">
+        <v>9</v>
+      </c>
+      <c r="D207" s="24" t="s">
+        <v>9</v>
+      </c>
+      <c r="E207" s="24" t="s">
+        <v>9</v>
+      </c>
+      <c r="F207" s="24" t="s">
+        <v>9</v>
+      </c>
+      <c r="G207" s="25" t="s">
+        <v>10</v>
+      </c>
+      <c r="H207" s="24" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="208" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A208" s="23" t="s">
+        <v>29</v>
+      </c>
+      <c r="B208" s="24" t="s">
+        <v>9</v>
+      </c>
+      <c r="C208" s="24" t="s">
+        <v>9</v>
+      </c>
+      <c r="D208" s="24" t="s">
+        <v>9</v>
+      </c>
+      <c r="E208" s="24" t="s">
+        <v>9</v>
+      </c>
+      <c r="F208" s="24" t="s">
+        <v>9</v>
+      </c>
+      <c r="G208" s="24" t="s">
+        <v>9</v>
+      </c>
+      <c r="H208" s="25" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="209" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A209" s="23" t="s">
+        <v>18</v>
+      </c>
+      <c r="B209" s="24" t="s">
+        <v>9</v>
+      </c>
+      <c r="C209" s="24" t="s">
+        <v>9</v>
+      </c>
+      <c r="D209" s="24" t="s">
+        <v>9</v>
+      </c>
+      <c r="E209" s="26" t="s">
+        <v>19</v>
+      </c>
+      <c r="F209" s="26" t="s">
+        <v>19</v>
+      </c>
+      <c r="G209" s="26" t="s">
+        <v>19</v>
+      </c>
+      <c r="H209" s="26" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="210" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A210" s="23" t="s">
+        <v>20</v>
+      </c>
+      <c r="B210" s="24" t="s">
+        <v>9</v>
+      </c>
+      <c r="C210" s="24" t="s">
+        <v>9</v>
+      </c>
+      <c r="D210" s="24" t="s">
+        <v>9</v>
+      </c>
+      <c r="E210" s="24" t="s">
+        <v>9</v>
+      </c>
+      <c r="F210" s="24" t="s">
+        <v>9</v>
+      </c>
+      <c r="G210" s="24" t="s">
+        <v>9</v>
+      </c>
+      <c r="H210" s="25" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="211" spans="1:8" ht="47.25" x14ac:dyDescent="0.25">
+      <c r="A211" s="23" t="s">
+        <v>17</v>
+      </c>
+      <c r="B211" s="24" t="s">
+        <v>9</v>
+      </c>
+      <c r="C211" s="24" t="s">
+        <v>36</v>
+      </c>
+      <c r="D211" s="24" t="s">
+        <v>37</v>
+      </c>
+      <c r="E211" s="24" t="s">
+        <v>38</v>
+      </c>
+      <c r="F211" s="24" t="s">
+        <v>9</v>
+      </c>
+      <c r="G211" s="25" t="s">
+        <v>10</v>
+      </c>
+      <c r="H211" s="24" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="212" spans="1:8" ht="31.5" x14ac:dyDescent="0.25">
+      <c r="A212" s="23" t="s">
+        <v>12</v>
+      </c>
+      <c r="B212" s="24" t="s">
+        <v>39</v>
+      </c>
+      <c r="C212" s="24" t="s">
+        <v>42</v>
+      </c>
+      <c r="D212" s="24" t="s">
+        <v>41</v>
+      </c>
+      <c r="E212" s="24" t="s">
+        <v>41</v>
+      </c>
+      <c r="F212" s="24" t="s">
+        <v>9</v>
+      </c>
+      <c r="G212" s="25" t="s">
+        <v>10</v>
+      </c>
+      <c r="H212" s="24" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="213" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A213" s="23" t="s">
+        <v>14</v>
+      </c>
+      <c r="B213" s="24" t="s">
+        <v>11</v>
+      </c>
+      <c r="C213" s="24" t="s">
+        <v>11</v>
+      </c>
+      <c r="D213" s="24" t="s">
+        <v>11</v>
+      </c>
+      <c r="E213" s="24" t="s">
+        <v>11</v>
+      </c>
+      <c r="F213" s="24" t="s">
+        <v>11</v>
+      </c>
+      <c r="G213" s="24" t="s">
+        <v>11</v>
+      </c>
+      <c r="H213" s="25" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="214" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A214" s="23" t="s">
+        <v>8</v>
+      </c>
+      <c r="B214" s="24" t="s">
+        <v>11</v>
+      </c>
+      <c r="C214" s="24" t="s">
+        <v>11</v>
+      </c>
+      <c r="D214" s="24" t="s">
+        <v>11</v>
+      </c>
+      <c r="E214" s="24" t="s">
+        <v>11</v>
+      </c>
+      <c r="F214" s="24" t="s">
+        <v>11</v>
+      </c>
+      <c r="G214" s="24" t="s">
+        <v>11</v>
+      </c>
+      <c r="H214" s="25" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="215" spans="1:8" ht="31.5" x14ac:dyDescent="0.25">
+      <c r="A215" s="23" t="s">
+        <v>23</v>
+      </c>
+      <c r="B215" s="24" t="s">
+        <v>11</v>
+      </c>
+      <c r="C215" s="24" t="s">
+        <v>11</v>
+      </c>
+      <c r="D215" s="24" t="s">
+        <v>11</v>
+      </c>
+      <c r="E215" s="24" t="s">
+        <v>11</v>
+      </c>
+      <c r="F215" s="24" t="s">
+        <v>11</v>
+      </c>
+      <c r="G215" s="25" t="s">
+        <v>10</v>
+      </c>
+      <c r="H215" s="24" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="216" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A216" s="23" t="s">
+        <v>21</v>
+      </c>
+      <c r="B216" s="24" t="s">
+        <v>13</v>
+      </c>
+      <c r="C216" s="24" t="s">
+        <v>13</v>
+      </c>
+      <c r="D216" s="24" t="s">
+        <v>13</v>
+      </c>
+      <c r="E216" s="24" t="s">
+        <v>13</v>
+      </c>
+      <c r="F216" s="24" t="s">
+        <v>13</v>
+      </c>
+      <c r="G216" s="24" t="s">
+        <v>13</v>
+      </c>
+      <c r="H216" s="25" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="217" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A217" s="27" t="s">
+        <v>27</v>
+      </c>
+      <c r="B217" s="28" t="s">
+        <v>31</v>
+      </c>
+      <c r="C217" s="28" t="s">
+        <v>31</v>
+      </c>
+      <c r="D217" s="28" t="s">
+        <v>31</v>
+      </c>
+      <c r="E217" s="28" t="s">
+        <v>31</v>
+      </c>
+      <c r="F217" s="25" t="s">
+        <v>10</v>
+      </c>
+      <c r="G217" s="29" t="s">
+        <v>34</v>
+      </c>
+      <c r="H217" s="29" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="218" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A218" s="23" t="s">
+        <v>28</v>
+      </c>
+      <c r="B218" s="19" t="s">
+        <v>35</v>
+      </c>
+      <c r="C218" s="26" t="s">
+        <v>19</v>
+      </c>
+      <c r="D218" s="26" t="s">
+        <v>19</v>
+      </c>
+      <c r="E218" s="26" t="s">
+        <v>19</v>
+      </c>
+      <c r="F218" s="25" t="s">
+        <v>10</v>
+      </c>
+      <c r="G218" s="25" t="s">
+        <v>10</v>
+      </c>
+      <c r="H218" s="25" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="219" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A219" s="30"/>
+      <c r="B219" s="30"/>
+      <c r="C219" s="30"/>
+      <c r="D219" s="30"/>
+      <c r="E219" s="30"/>
+      <c r="F219" s="30"/>
+      <c r="G219" s="30"/>
+      <c r="H219" s="30"/>
+    </row>
+    <row r="220" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A220" s="33" t="s">
+        <v>0</v>
+      </c>
+      <c r="B220" s="22">
+        <v>46244</v>
+      </c>
+      <c r="C220" s="22">
+        <v>46245</v>
+      </c>
+      <c r="D220" s="22">
+        <v>46246</v>
+      </c>
+      <c r="E220" s="22">
+        <v>46247</v>
+      </c>
+      <c r="F220" s="22">
+        <v>46248</v>
+      </c>
+      <c r="G220" s="22">
+        <v>46249</v>
+      </c>
+      <c r="H220" s="22">
+        <v>46250</v>
+      </c>
+    </row>
+    <row r="221" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A221" s="34"/>
+      <c r="B221" s="23" t="s">
+        <v>1</v>
+      </c>
+      <c r="C221" s="23" t="s">
+        <v>2</v>
+      </c>
+      <c r="D221" s="23" t="s">
+        <v>3</v>
+      </c>
+      <c r="E221" s="23" t="s">
+        <v>4</v>
+      </c>
+      <c r="F221" s="23" t="s">
+        <v>5</v>
+      </c>
+      <c r="G221" s="23" t="s">
+        <v>6</v>
+      </c>
+      <c r="H221" s="23" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="222" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A222" s="23" t="s">
+        <v>22</v>
+      </c>
+      <c r="B222" s="24" t="s">
+        <v>9</v>
+      </c>
+      <c r="C222" s="24" t="s">
+        <v>9</v>
+      </c>
+      <c r="D222" s="24" t="s">
+        <v>9</v>
+      </c>
+      <c r="E222" s="24" t="s">
+        <v>9</v>
+      </c>
+      <c r="F222" s="24" t="s">
+        <v>9</v>
+      </c>
+      <c r="G222" s="24" t="s">
+        <v>9</v>
+      </c>
+      <c r="H222" s="25" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="223" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A223" s="23" t="s">
+        <v>29</v>
+      </c>
+      <c r="B223" s="24" t="s">
+        <v>9</v>
+      </c>
+      <c r="C223" s="24" t="s">
+        <v>9</v>
+      </c>
+      <c r="D223" s="24" t="s">
+        <v>9</v>
+      </c>
+      <c r="E223" s="24" t="s">
+        <v>9</v>
+      </c>
+      <c r="F223" s="24" t="s">
+        <v>9</v>
+      </c>
+      <c r="G223" s="25" t="s">
+        <v>10</v>
+      </c>
+      <c r="H223" s="24" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="224" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A224" s="23" t="s">
+        <v>14</v>
+      </c>
+      <c r="B224" s="24" t="s">
+        <v>9</v>
+      </c>
+      <c r="C224" s="24" t="s">
+        <v>9</v>
+      </c>
+      <c r="D224" s="24" t="s">
+        <v>9</v>
+      </c>
+      <c r="E224" s="24" t="s">
+        <v>9</v>
+      </c>
+      <c r="F224" s="24" t="s">
+        <v>9</v>
+      </c>
+      <c r="G224" s="25" t="s">
+        <v>10</v>
+      </c>
+      <c r="H224" s="24" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="225" spans="1:8" ht="31.5" x14ac:dyDescent="0.25">
+      <c r="A225" s="23" t="s">
+        <v>23</v>
+      </c>
+      <c r="B225" s="24" t="s">
+        <v>9</v>
+      </c>
+      <c r="C225" s="24" t="s">
+        <v>9</v>
+      </c>
+      <c r="D225" s="24" t="s">
+        <v>9</v>
+      </c>
+      <c r="E225" s="24" t="s">
+        <v>9</v>
+      </c>
+      <c r="F225" s="31" t="s">
+        <v>40</v>
+      </c>
+      <c r="G225" s="31" t="s">
+        <v>40</v>
+      </c>
+      <c r="H225" s="31" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="226" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A226" s="23" t="s">
+        <v>18</v>
+      </c>
+      <c r="B226" s="26" t="s">
+        <v>19</v>
+      </c>
+      <c r="C226" s="24" t="s">
+        <v>9</v>
+      </c>
+      <c r="D226" s="24" t="s">
+        <v>9</v>
+      </c>
+      <c r="E226" s="24" t="s">
+        <v>9</v>
+      </c>
+      <c r="F226" s="24" t="s">
+        <v>9</v>
+      </c>
+      <c r="G226" s="24" t="s">
+        <v>26</v>
+      </c>
+      <c r="H226" s="32" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="227" spans="1:8" ht="47.25" x14ac:dyDescent="0.25">
+      <c r="A227" s="23" t="s">
+        <v>17</v>
+      </c>
+      <c r="B227" s="24" t="s">
+        <v>9</v>
+      </c>
+      <c r="C227" s="24" t="s">
+        <v>36</v>
+      </c>
+      <c r="D227" s="24" t="s">
+        <v>37</v>
+      </c>
+      <c r="E227" s="24" t="s">
+        <v>38</v>
+      </c>
+      <c r="F227" s="24" t="s">
+        <v>9</v>
+      </c>
+      <c r="G227" s="24" t="s">
+        <v>11</v>
+      </c>
+      <c r="H227" s="25" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="228" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A228" s="23" t="s">
+        <v>8</v>
+      </c>
+      <c r="B228" s="24" t="s">
+        <v>11</v>
+      </c>
+      <c r="C228" s="24" t="s">
+        <v>11</v>
+      </c>
+      <c r="D228" s="24" t="s">
+        <v>11</v>
+      </c>
+      <c r="E228" s="24" t="s">
+        <v>11</v>
+      </c>
+      <c r="F228" s="24" t="s">
+        <v>11</v>
+      </c>
+      <c r="G228" s="26" t="s">
+        <v>19</v>
+      </c>
+      <c r="H228" s="26" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="229" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A229" s="23" t="s">
+        <v>21</v>
+      </c>
+      <c r="B229" s="24" t="s">
+        <v>11</v>
+      </c>
+      <c r="C229" s="24" t="s">
+        <v>11</v>
+      </c>
+      <c r="D229" s="24" t="s">
+        <v>11</v>
+      </c>
+      <c r="E229" s="24" t="s">
+        <v>11</v>
+      </c>
+      <c r="F229" s="24" t="s">
+        <v>11</v>
+      </c>
+      <c r="G229" s="25" t="s">
+        <v>10</v>
+      </c>
+      <c r="H229" s="24" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="230" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A230" s="23" t="s">
+        <v>20</v>
+      </c>
+      <c r="B230" s="24" t="s">
+        <v>11</v>
+      </c>
+      <c r="C230" s="24" t="s">
+        <v>11</v>
+      </c>
+      <c r="D230" s="24" t="s">
+        <v>11</v>
+      </c>
+      <c r="E230" s="24" t="s">
+        <v>11</v>
+      </c>
+      <c r="F230" s="24" t="s">
+        <v>11</v>
+      </c>
+      <c r="G230" s="25" t="s">
+        <v>10</v>
+      </c>
+      <c r="H230" s="24" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="231" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A231" s="23" t="s">
+        <v>12</v>
+      </c>
+      <c r="B231" s="24" t="s">
+        <v>13</v>
+      </c>
+      <c r="C231" s="24" t="s">
+        <v>13</v>
+      </c>
+      <c r="D231" s="24" t="s">
+        <v>13</v>
+      </c>
+      <c r="E231" s="24" t="s">
+        <v>13</v>
+      </c>
+      <c r="F231" s="24" t="s">
+        <v>13</v>
+      </c>
+      <c r="G231" s="24" t="s">
+        <v>13</v>
+      </c>
+      <c r="H231" s="25" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="232" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A232" s="30"/>
+      <c r="B232" s="30"/>
+      <c r="C232" s="30"/>
+      <c r="D232" s="30"/>
+      <c r="E232" s="30"/>
+      <c r="F232" s="30"/>
+      <c r="G232" s="30"/>
+      <c r="H232" s="30"/>
+    </row>
   </sheetData>
-  <mergeCells count="15">
+  <mergeCells count="17">
     <mergeCell ref="A1:A2"/>
     <mergeCell ref="A14:A15"/>
     <mergeCell ref="A27:A28"/>
     <mergeCell ref="A40:A41"/>
     <mergeCell ref="A53:A54"/>
+    <mergeCell ref="A205:A206"/>
+    <mergeCell ref="A220:A221"/>
     <mergeCell ref="A190:A191"/>
     <mergeCell ref="G84:H84"/>
     <mergeCell ref="A66:A67"/>

</xml_diff>

<commit_message>
Actualizacion automatica de datos - jue 06/08/2026 12:01:28,89
</commit_message>
<xml_diff>
--- a/Horario/Horario 2026.xlsx
+++ b/Horario/Horario 2026.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://virtualsoftserv-my.sharepoint.com/personal/maria_sanchez_virtualsoft_tech/Documents/Indicadores y Pagina WEB/Horario/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="8" documentId="6_{6E17BD36-3E42-42F2-8AFD-92DB165A9BC2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{8FE51109-7016-4FEF-BF2C-19B9330DBB34}"/>
+  <xr:revisionPtr revIDLastSave="10" documentId="6_{6E17BD36-3E42-42F2-8AFD-92DB165A9BC2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{97FBA5BF-47C2-406C-AC55-13C51F6A0428}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{9AAEFA76-0198-46F6-BBF5-EADAB38A6758}"/>
   </bookViews>
@@ -181,9 +181,9 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="1">
-    <numFmt numFmtId="167" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@_-"/>
+    <numFmt numFmtId="43" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@_-"/>
   </numFmts>
-  <fonts count="14" x14ac:knownFonts="1">
+  <fonts count="18" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -279,6 +279,29 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b/>
+      <sz val="12"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="12"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+    </font>
   </fonts>
   <fills count="13">
     <fill>
@@ -354,7 +377,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="6">
+  <borders count="7">
     <border>
       <left/>
       <right/>
@@ -429,15 +452,26 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="0"/>
-    <xf numFmtId="167" fontId="13" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="167" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="43" fontId="13" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="41">
+  <cellXfs count="53">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="16" fontId="2" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -485,31 +519,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="9" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="9" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -538,6 +548,66 @@
     </xf>
     <xf numFmtId="0" fontId="5" fillId="11" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="9" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="9" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="7" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="10" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="11" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="10" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="7" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="11" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="5">
@@ -611,6 +681,10 @@
     <xdr:clientData/>
   </xdr:twoCellAnchor>
 </xdr:wsDr>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -942,7 +1016,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:15" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A1" s="28" t="s">
+      <c r="A1" s="33" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="1">
@@ -989,7 +1063,7 @@
       </c>
     </row>
     <row r="2" spans="1:15" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A2" s="29"/>
+      <c r="A2" s="34"/>
       <c r="B2" s="2" t="s">
         <v>1</v>
       </c>
@@ -1504,7 +1578,7 @@
       </c>
     </row>
     <row r="14" spans="1:15" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A14" s="28" t="s">
+      <c r="A14" s="33" t="s">
         <v>0</v>
       </c>
       <c r="B14" s="1">
@@ -1530,7 +1604,7 @@
       </c>
     </row>
     <row r="15" spans="1:15" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A15" s="29"/>
+      <c r="A15" s="34"/>
       <c r="B15" s="2" t="s">
         <v>1</v>
       </c>
@@ -1814,7 +1888,7 @@
       </c>
     </row>
     <row r="27" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A27" s="28" t="s">
+      <c r="A27" s="33" t="s">
         <v>0</v>
       </c>
       <c r="B27" s="1">
@@ -1840,7 +1914,7 @@
       </c>
     </row>
     <row r="28" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A28" s="29"/>
+      <c r="A28" s="34"/>
       <c r="B28" s="2" t="s">
         <v>1</v>
       </c>
@@ -2124,7 +2198,7 @@
       </c>
     </row>
     <row r="40" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A40" s="25" t="s">
+      <c r="A40" s="35" t="s">
         <v>0</v>
       </c>
       <c r="B40" s="1">
@@ -2150,7 +2224,7 @@
       </c>
     </row>
     <row r="41" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A41" s="25"/>
+      <c r="A41" s="35"/>
       <c r="B41" s="2" t="s">
         <v>1</v>
       </c>
@@ -2434,7 +2508,7 @@
       </c>
     </row>
     <row r="53" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A53" s="25" t="s">
+      <c r="A53" s="35" t="s">
         <v>0</v>
       </c>
       <c r="B53" s="1">
@@ -2460,7 +2534,7 @@
       </c>
     </row>
     <row r="54" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A54" s="25"/>
+      <c r="A54" s="35"/>
       <c r="B54" s="2" t="s">
         <v>1</v>
       </c>
@@ -2744,7 +2818,7 @@
       </c>
     </row>
     <row r="66" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A66" s="25" t="s">
+      <c r="A66" s="35" t="s">
         <v>0</v>
       </c>
       <c r="B66" s="1">
@@ -2770,7 +2844,7 @@
       </c>
     </row>
     <row r="67" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A67" s="25"/>
+      <c r="A67" s="35"/>
       <c r="B67" s="2" t="s">
         <v>1</v>
       </c>
@@ -3054,7 +3128,7 @@
       </c>
     </row>
     <row r="79" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A79" s="25" t="s">
+      <c r="A79" s="35" t="s">
         <v>0</v>
       </c>
       <c r="B79" s="1">
@@ -3080,7 +3154,7 @@
       </c>
     </row>
     <row r="80" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A80" s="25"/>
+      <c r="A80" s="35"/>
       <c r="B80" s="2" t="s">
         <v>1</v>
       </c>
@@ -3200,8 +3274,8 @@
       <c r="F84" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="G84" s="26"/>
-      <c r="H84" s="27"/>
+      <c r="G84" s="36"/>
+      <c r="H84" s="37"/>
     </row>
     <row r="85" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A85" s="3" t="s">
@@ -3360,7 +3434,7 @@
       </c>
     </row>
     <row r="92" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A92" s="25" t="s">
+      <c r="A92" s="35" t="s">
         <v>0</v>
       </c>
       <c r="B92" s="1">
@@ -3386,7 +3460,7 @@
       </c>
     </row>
     <row r="93" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A93" s="25"/>
+      <c r="A93" s="35"/>
       <c r="B93" s="2" t="s">
         <v>1</v>
       </c>
@@ -3644,7 +3718,7 @@
       </c>
     </row>
     <row r="104" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A104" s="25" t="s">
+      <c r="A104" s="35" t="s">
         <v>0</v>
       </c>
       <c r="B104" s="1">
@@ -3670,7 +3744,7 @@
       </c>
     </row>
     <row r="105" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A105" s="25"/>
+      <c r="A105" s="35"/>
       <c r="B105" s="2" t="s">
         <v>1</v>
       </c>
@@ -3928,7 +4002,7 @@
       </c>
     </row>
     <row r="116" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A116" s="25" t="s">
+      <c r="A116" s="35" t="s">
         <v>0</v>
       </c>
       <c r="B116" s="1">
@@ -3954,7 +4028,7 @@
       </c>
     </row>
     <row r="117" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A117" s="25"/>
+      <c r="A117" s="35"/>
       <c r="B117" s="2" t="s">
         <v>1</v>
       </c>
@@ -4626,7 +4700,7 @@
       </c>
     </row>
     <row r="145" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A145" s="25" t="s">
+      <c r="A145" s="35" t="s">
         <v>0</v>
       </c>
       <c r="B145" s="1">
@@ -4652,7 +4726,7 @@
       </c>
     </row>
     <row r="146" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A146" s="25"/>
+      <c r="A146" s="35"/>
       <c r="B146" s="2" t="s">
         <v>1</v>
       </c>
@@ -4988,7 +5062,7 @@
       </c>
     </row>
     <row r="160" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A160" s="25" t="s">
+      <c r="A160" s="35" t="s">
         <v>0</v>
       </c>
       <c r="B160" s="1">
@@ -5014,7 +5088,7 @@
       </c>
     </row>
     <row r="161" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A161" s="25"/>
+      <c r="A161" s="35"/>
       <c r="B161" s="2" t="s">
         <v>1</v>
       </c>
@@ -5350,7 +5424,7 @@
       </c>
     </row>
     <row r="175" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A175" s="25" t="s">
+      <c r="A175" s="35" t="s">
         <v>0</v>
       </c>
       <c r="B175" s="1">
@@ -5376,7 +5450,7 @@
       </c>
     </row>
     <row r="176" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A176" s="25"/>
+      <c r="A176" s="35"/>
       <c r="B176" s="2" t="s">
         <v>1</v>
       </c>
@@ -5712,7 +5786,7 @@
       </c>
     </row>
     <row r="190" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A190" s="25" t="s">
+      <c r="A190" s="35" t="s">
         <v>0</v>
       </c>
       <c r="B190" s="1">
@@ -5738,7 +5812,7 @@
       </c>
     </row>
     <row r="191" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A191" s="25"/>
+      <c r="A191" s="35"/>
       <c r="B191" s="2" t="s">
         <v>1</v>
       </c>
@@ -6074,364 +6148,364 @@
       </c>
     </row>
     <row r="205" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A205" s="23" t="s">
+      <c r="A205" s="38" t="s">
         <v>0</v>
       </c>
-      <c r="B205" s="34">
+      <c r="B205" s="26">
         <v>46237</v>
       </c>
-      <c r="C205" s="34">
+      <c r="C205" s="26">
         <v>46238</v>
       </c>
-      <c r="D205" s="34">
+      <c r="D205" s="26">
         <v>46239</v>
       </c>
-      <c r="E205" s="34">
+      <c r="E205" s="26">
         <v>46240</v>
       </c>
-      <c r="F205" s="34">
+      <c r="F205" s="26">
         <v>46241</v>
       </c>
-      <c r="G205" s="34">
+      <c r="G205" s="26">
         <v>46242</v>
       </c>
-      <c r="H205" s="34">
+      <c r="H205" s="26">
         <v>46243</v>
       </c>
     </row>
     <row r="206" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A206" s="24"/>
-      <c r="B206" s="30" t="s">
+      <c r="A206" s="38"/>
+      <c r="B206" s="23" t="s">
         <v>1</v>
       </c>
-      <c r="C206" s="30" t="s">
+      <c r="C206" s="23" t="s">
         <v>2</v>
       </c>
-      <c r="D206" s="30" t="s">
+      <c r="D206" s="23" t="s">
         <v>3</v>
       </c>
-      <c r="E206" s="30" t="s">
+      <c r="E206" s="23" t="s">
         <v>4</v>
       </c>
-      <c r="F206" s="30" t="s">
+      <c r="F206" s="23" t="s">
         <v>5</v>
       </c>
-      <c r="G206" s="30" t="s">
+      <c r="G206" s="23" t="s">
         <v>6</v>
       </c>
-      <c r="H206" s="30" t="s">
+      <c r="H206" s="23" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="207" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A207" s="30" t="s">
+      <c r="A207" s="23" t="s">
         <v>22</v>
       </c>
-      <c r="B207" s="32" t="s">
-        <v>9</v>
-      </c>
-      <c r="C207" s="32" t="s">
-        <v>9</v>
-      </c>
-      <c r="D207" s="32" t="s">
-        <v>9</v>
-      </c>
-      <c r="E207" s="32" t="s">
-        <v>9</v>
-      </c>
-      <c r="F207" s="32" t="s">
-        <v>9</v>
-      </c>
-      <c r="G207" s="37" t="s">
-        <v>10</v>
-      </c>
-      <c r="H207" s="32" t="s">
+      <c r="B207" s="24" t="s">
+        <v>9</v>
+      </c>
+      <c r="C207" s="24" t="s">
+        <v>9</v>
+      </c>
+      <c r="D207" s="24" t="s">
+        <v>9</v>
+      </c>
+      <c r="E207" s="24" t="s">
+        <v>9</v>
+      </c>
+      <c r="F207" s="24" t="s">
+        <v>9</v>
+      </c>
+      <c r="G207" s="29" t="s">
+        <v>10</v>
+      </c>
+      <c r="H207" s="24" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="208" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A208" s="30" t="s">
+      <c r="A208" s="23" t="s">
         <v>29</v>
       </c>
-      <c r="B208" s="32" t="s">
-        <v>9</v>
-      </c>
-      <c r="C208" s="32" t="s">
-        <v>9</v>
-      </c>
-      <c r="D208" s="32" t="s">
-        <v>9</v>
-      </c>
-      <c r="E208" s="32" t="s">
-        <v>9</v>
-      </c>
-      <c r="F208" s="32" t="s">
-        <v>9</v>
-      </c>
-      <c r="G208" s="32" t="s">
-        <v>9</v>
-      </c>
-      <c r="H208" s="37" t="s">
+      <c r="B208" s="24" t="s">
+        <v>9</v>
+      </c>
+      <c r="C208" s="24" t="s">
+        <v>9</v>
+      </c>
+      <c r="D208" s="24" t="s">
+        <v>9</v>
+      </c>
+      <c r="E208" s="24" t="s">
+        <v>9</v>
+      </c>
+      <c r="F208" s="24" t="s">
+        <v>9</v>
+      </c>
+      <c r="G208" s="24" t="s">
+        <v>9</v>
+      </c>
+      <c r="H208" s="29" t="s">
         <v>10</v>
       </c>
     </row>
     <row r="209" spans="1:8" ht="46.8" x14ac:dyDescent="0.3">
-      <c r="A209" s="30" t="s">
+      <c r="A209" s="23" t="s">
         <v>18</v>
       </c>
-      <c r="B209" s="32" t="s">
-        <v>9</v>
-      </c>
-      <c r="C209" s="32" t="s">
-        <v>9</v>
-      </c>
-      <c r="D209" s="39" t="s">
+      <c r="B209" s="24" t="s">
+        <v>9</v>
+      </c>
+      <c r="C209" s="24" t="s">
+        <v>9</v>
+      </c>
+      <c r="D209" s="31" t="s">
         <v>43</v>
       </c>
-      <c r="E209" s="33" t="s">
+      <c r="E209" s="25" t="s">
         <v>19</v>
       </c>
-      <c r="F209" s="33" t="s">
+      <c r="F209" s="25" t="s">
         <v>19</v>
       </c>
-      <c r="G209" s="33" t="s">
+      <c r="G209" s="25" t="s">
         <v>19</v>
       </c>
-      <c r="H209" s="33" t="s">
+      <c r="H209" s="25" t="s">
         <v>19</v>
       </c>
     </row>
     <row r="210" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A210" s="30" t="s">
+      <c r="A210" s="23" t="s">
         <v>20</v>
       </c>
-      <c r="B210" s="32" t="s">
-        <v>9</v>
-      </c>
-      <c r="C210" s="32" t="s">
-        <v>9</v>
-      </c>
-      <c r="D210" s="32" t="s">
-        <v>9</v>
-      </c>
-      <c r="E210" s="32" t="s">
-        <v>9</v>
-      </c>
-      <c r="F210" s="32" t="s">
-        <v>9</v>
-      </c>
-      <c r="G210" s="32" t="s">
-        <v>9</v>
-      </c>
-      <c r="H210" s="37" t="s">
+      <c r="B210" s="24" t="s">
+        <v>9</v>
+      </c>
+      <c r="C210" s="24" t="s">
+        <v>9</v>
+      </c>
+      <c r="D210" s="24" t="s">
+        <v>9</v>
+      </c>
+      <c r="E210" s="24" t="s">
+        <v>9</v>
+      </c>
+      <c r="F210" s="24" t="s">
+        <v>13</v>
+      </c>
+      <c r="G210" s="24" t="s">
+        <v>13</v>
+      </c>
+      <c r="H210" s="29" t="s">
         <v>10</v>
       </c>
     </row>
     <row r="211" spans="1:8" ht="46.8" x14ac:dyDescent="0.3">
-      <c r="A211" s="30" t="s">
+      <c r="A211" s="23" t="s">
         <v>17</v>
       </c>
-      <c r="B211" s="32" t="s">
-        <v>9</v>
-      </c>
-      <c r="C211" s="32" t="s">
+      <c r="B211" s="24" t="s">
+        <v>9</v>
+      </c>
+      <c r="C211" s="24" t="s">
         <v>36</v>
       </c>
-      <c r="D211" s="32" t="s">
+      <c r="D211" s="24" t="s">
         <v>37</v>
       </c>
-      <c r="E211" s="32" t="s">
+      <c r="E211" s="24" t="s">
         <v>38</v>
       </c>
-      <c r="F211" s="32" t="s">
-        <v>9</v>
-      </c>
-      <c r="G211" s="37" t="s">
-        <v>10</v>
-      </c>
-      <c r="H211" s="32" t="s">
+      <c r="F211" s="24" t="s">
+        <v>9</v>
+      </c>
+      <c r="G211" s="29" t="s">
+        <v>10</v>
+      </c>
+      <c r="H211" s="24" t="s">
         <v>11</v>
       </c>
     </row>
     <row r="212" spans="1:8" ht="46.8" x14ac:dyDescent="0.3">
-      <c r="A212" s="30" t="s">
+      <c r="A212" s="23" t="s">
         <v>12</v>
       </c>
-      <c r="B212" s="32" t="s">
+      <c r="B212" s="24" t="s">
         <v>39</v>
       </c>
-      <c r="C212" s="32" t="s">
+      <c r="C212" s="24" t="s">
         <v>42</v>
       </c>
-      <c r="D212" s="32" t="s">
+      <c r="D212" s="24" t="s">
         <v>41</v>
       </c>
-      <c r="E212" s="39" t="s">
+      <c r="E212" s="31" t="s">
         <v>44</v>
       </c>
-      <c r="F212" s="32" t="s">
-        <v>13</v>
-      </c>
-      <c r="G212" s="32" t="s">
-        <v>13</v>
-      </c>
-      <c r="H212" s="37" t="s">
+      <c r="F212" s="24" t="s">
+        <v>9</v>
+      </c>
+      <c r="G212" s="24" t="s">
+        <v>11</v>
+      </c>
+      <c r="H212" s="29" t="s">
         <v>10</v>
       </c>
     </row>
     <row r="213" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A213" s="30" t="s">
+      <c r="A213" s="23" t="s">
         <v>14</v>
       </c>
-      <c r="B213" s="32" t="s">
-        <v>11</v>
-      </c>
-      <c r="C213" s="32" t="s">
-        <v>11</v>
-      </c>
-      <c r="D213" s="32" t="s">
-        <v>11</v>
-      </c>
-      <c r="E213" s="32" t="s">
-        <v>11</v>
-      </c>
-      <c r="F213" s="32" t="s">
-        <v>11</v>
-      </c>
-      <c r="G213" s="37" t="s">
-        <v>10</v>
-      </c>
-      <c r="H213" s="32" t="s">
+      <c r="B213" s="24" t="s">
+        <v>11</v>
+      </c>
+      <c r="C213" s="24" t="s">
+        <v>11</v>
+      </c>
+      <c r="D213" s="24" t="s">
+        <v>11</v>
+      </c>
+      <c r="E213" s="24" t="s">
+        <v>11</v>
+      </c>
+      <c r="F213" s="24" t="s">
+        <v>11</v>
+      </c>
+      <c r="G213" s="29" t="s">
+        <v>10</v>
+      </c>
+      <c r="H213" s="24" t="s">
         <v>13</v>
       </c>
     </row>
     <row r="214" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A214" s="30" t="s">
+      <c r="A214" s="23" t="s">
         <v>8</v>
       </c>
-      <c r="B214" s="32" t="s">
-        <v>11</v>
-      </c>
-      <c r="C214" s="32" t="s">
-        <v>11</v>
-      </c>
-      <c r="D214" s="32" t="s">
-        <v>11</v>
-      </c>
-      <c r="E214" s="32" t="s">
-        <v>11</v>
-      </c>
-      <c r="F214" s="32" t="s">
-        <v>11</v>
-      </c>
-      <c r="G214" s="32" t="s">
-        <v>11</v>
-      </c>
-      <c r="H214" s="37" t="s">
+      <c r="B214" s="24" t="s">
+        <v>11</v>
+      </c>
+      <c r="C214" s="24" t="s">
+        <v>11</v>
+      </c>
+      <c r="D214" s="24" t="s">
+        <v>11</v>
+      </c>
+      <c r="E214" s="24" t="s">
+        <v>11</v>
+      </c>
+      <c r="F214" s="24" t="s">
+        <v>11</v>
+      </c>
+      <c r="G214" s="24" t="s">
+        <v>9</v>
+      </c>
+      <c r="H214" s="29" t="s">
         <v>10</v>
       </c>
     </row>
     <row r="215" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A215" s="30" t="s">
+      <c r="A215" s="23" t="s">
         <v>23</v>
       </c>
-      <c r="B215" s="32" t="s">
-        <v>11</v>
-      </c>
-      <c r="C215" s="32" t="s">
-        <v>11</v>
-      </c>
-      <c r="D215" s="32" t="s">
-        <v>11</v>
-      </c>
-      <c r="E215" s="32" t="s">
-        <v>11</v>
-      </c>
-      <c r="F215" s="32" t="s">
-        <v>11</v>
-      </c>
-      <c r="G215" s="37" t="s">
-        <v>10</v>
-      </c>
-      <c r="H215" s="32" t="s">
+      <c r="B215" s="24" t="s">
+        <v>11</v>
+      </c>
+      <c r="C215" s="24" t="s">
+        <v>11</v>
+      </c>
+      <c r="D215" s="24" t="s">
+        <v>11</v>
+      </c>
+      <c r="E215" s="24" t="s">
+        <v>11</v>
+      </c>
+      <c r="F215" s="24" t="s">
+        <v>11</v>
+      </c>
+      <c r="G215" s="29" t="s">
+        <v>10</v>
+      </c>
+      <c r="H215" s="24" t="s">
         <v>26</v>
       </c>
     </row>
     <row r="216" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A216" s="30" t="s">
+      <c r="A216" s="23" t="s">
         <v>21</v>
       </c>
-      <c r="B216" s="32" t="s">
-        <v>13</v>
-      </c>
-      <c r="C216" s="32" t="s">
-        <v>13</v>
-      </c>
-      <c r="D216" s="32" t="s">
-        <v>13</v>
-      </c>
-      <c r="E216" s="32" t="s">
-        <v>13</v>
-      </c>
-      <c r="F216" s="32" t="s">
-        <v>9</v>
-      </c>
-      <c r="G216" s="32" t="s">
-        <v>11</v>
-      </c>
-      <c r="H216" s="37" t="s">
+      <c r="B216" s="24" t="s">
+        <v>13</v>
+      </c>
+      <c r="C216" s="24" t="s">
+        <v>13</v>
+      </c>
+      <c r="D216" s="24" t="s">
+        <v>13</v>
+      </c>
+      <c r="E216" s="24" t="s">
+        <v>13</v>
+      </c>
+      <c r="F216" s="45" t="s">
+        <v>9</v>
+      </c>
+      <c r="G216" s="45" t="s">
+        <v>11</v>
+      </c>
+      <c r="H216" s="29" t="s">
         <v>10</v>
       </c>
     </row>
     <row r="217" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A217" s="35" t="s">
+      <c r="A217" s="27" t="s">
         <v>27</v>
       </c>
-      <c r="B217" s="32" t="s">
+      <c r="B217" s="24" t="s">
         <v>31</v>
       </c>
-      <c r="C217" s="32" t="s">
+      <c r="C217" s="24" t="s">
         <v>31</v>
       </c>
-      <c r="D217" s="32" t="s">
+      <c r="D217" s="24" t="s">
         <v>31</v>
       </c>
-      <c r="E217" s="32" t="s">
+      <c r="E217" s="46" t="s">
         <v>31</v>
       </c>
-      <c r="F217" s="37" t="s">
-        <v>10</v>
-      </c>
-      <c r="G217" s="38" t="s">
+      <c r="F217" s="43" t="s">
         <v>34</v>
       </c>
-      <c r="H217" s="38" t="s">
+      <c r="G217" s="30" t="s">
         <v>34</v>
       </c>
+      <c r="H217" s="47" t="s">
+        <v>34</v>
+      </c>
     </row>
     <row r="218" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A218" s="30" t="s">
+      <c r="A218" s="23" t="s">
         <v>28</v>
       </c>
-      <c r="B218" s="40" t="s">
+      <c r="B218" s="32" t="s">
         <v>35</v>
       </c>
-      <c r="C218" s="33" t="s">
+      <c r="C218" s="25" t="s">
         <v>19</v>
       </c>
-      <c r="D218" s="33" t="s">
+      <c r="D218" s="25" t="s">
         <v>19</v>
       </c>
-      <c r="E218" s="33" t="s">
+      <c r="E218" s="48" t="s">
         <v>19</v>
       </c>
-      <c r="F218" s="37" t="s">
-        <v>10</v>
-      </c>
-      <c r="G218" s="37" t="s">
-        <v>10</v>
-      </c>
-      <c r="H218" s="37" t="s">
+      <c r="F218" s="29" t="s">
+        <v>10</v>
+      </c>
+      <c r="G218" s="29" t="s">
+        <v>10</v>
+      </c>
+      <c r="H218" s="49" t="s">
         <v>10</v>
       </c>
     </row>
@@ -6446,374 +6520,371 @@
       <c r="H219" s="22"/>
     </row>
     <row r="220" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A220" s="23" t="s">
+      <c r="A220" s="38" t="s">
         <v>0</v>
       </c>
-      <c r="B220" s="34">
+      <c r="B220" s="26">
         <v>46244</v>
       </c>
-      <c r="C220" s="34">
+      <c r="C220" s="26">
         <v>46245</v>
       </c>
-      <c r="D220" s="34">
+      <c r="D220" s="26">
         <v>46246</v>
       </c>
-      <c r="E220" s="34">
+      <c r="E220" s="26">
         <v>46247</v>
       </c>
-      <c r="F220" s="34">
+      <c r="F220" s="26">
         <v>46248</v>
       </c>
-      <c r="G220" s="34">
+      <c r="G220" s="26">
         <v>46249</v>
       </c>
-      <c r="H220" s="34">
+      <c r="H220" s="26">
         <v>46250</v>
       </c>
     </row>
     <row r="221" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A221" s="24"/>
-      <c r="B221" s="30" t="s">
+      <c r="A221" s="38"/>
+      <c r="B221" s="23" t="s">
         <v>1</v>
       </c>
-      <c r="C221" s="30" t="s">
+      <c r="C221" s="23" t="s">
         <v>2</v>
       </c>
-      <c r="D221" s="30" t="s">
+      <c r="D221" s="23" t="s">
         <v>3</v>
       </c>
-      <c r="E221" s="30" t="s">
+      <c r="E221" s="23" t="s">
         <v>4</v>
       </c>
-      <c r="F221" s="30" t="s">
+      <c r="F221" s="23" t="s">
         <v>5</v>
       </c>
-      <c r="G221" s="30" t="s">
+      <c r="G221" s="23" t="s">
         <v>6</v>
       </c>
-      <c r="H221" s="30" t="s">
+      <c r="H221" s="23" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="222" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A222" s="30" t="s">
+      <c r="A222" s="23" t="s">
         <v>22</v>
       </c>
-      <c r="B222" s="32" t="s">
-        <v>9</v>
-      </c>
-      <c r="C222" s="32" t="s">
-        <v>9</v>
-      </c>
-      <c r="D222" s="32" t="s">
-        <v>9</v>
-      </c>
-      <c r="E222" s="32" t="s">
-        <v>9</v>
-      </c>
-      <c r="F222" s="32" t="s">
-        <v>9</v>
-      </c>
-      <c r="G222" s="32" t="s">
-        <v>9</v>
-      </c>
-      <c r="H222" s="37" t="s">
+      <c r="B222" s="24" t="s">
+        <v>9</v>
+      </c>
+      <c r="C222" s="44" t="s">
+        <v>35</v>
+      </c>
+      <c r="D222" s="24" t="s">
+        <v>9</v>
+      </c>
+      <c r="E222" s="24" t="s">
+        <v>9</v>
+      </c>
+      <c r="F222" s="24" t="s">
+        <v>9</v>
+      </c>
+      <c r="G222" s="24" t="s">
+        <v>9</v>
+      </c>
+      <c r="H222" s="29" t="s">
         <v>10</v>
       </c>
     </row>
     <row r="223" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A223" s="30" t="s">
+      <c r="A223" s="23" t="s">
         <v>29</v>
       </c>
-      <c r="B223" s="32" t="s">
-        <v>9</v>
-      </c>
-      <c r="C223" s="32" t="s">
-        <v>9</v>
-      </c>
-      <c r="D223" s="32" t="s">
-        <v>9</v>
-      </c>
-      <c r="E223" s="32" t="s">
-        <v>9</v>
-      </c>
-      <c r="F223" s="32" t="s">
-        <v>9</v>
-      </c>
-      <c r="G223" s="37" t="s">
-        <v>10</v>
-      </c>
-      <c r="H223" s="32" t="s">
+      <c r="B223" s="24" t="s">
+        <v>9</v>
+      </c>
+      <c r="C223" s="24" t="s">
+        <v>9</v>
+      </c>
+      <c r="D223" s="24" t="s">
+        <v>9</v>
+      </c>
+      <c r="E223" s="24" t="s">
+        <v>9</v>
+      </c>
+      <c r="F223" s="24" t="s">
+        <v>9</v>
+      </c>
+      <c r="G223" s="29" t="s">
+        <v>10</v>
+      </c>
+      <c r="H223" s="24" t="s">
         <v>11</v>
       </c>
     </row>
     <row r="224" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A224" s="30" t="s">
+      <c r="A224" s="23" t="s">
         <v>21</v>
       </c>
-      <c r="B224" s="32" t="s">
-        <v>9</v>
-      </c>
-      <c r="C224" s="32" t="s">
-        <v>9</v>
-      </c>
-      <c r="D224" s="32" t="s">
-        <v>9</v>
-      </c>
-      <c r="E224" s="32" t="s">
-        <v>9</v>
-      </c>
-      <c r="F224" s="32" t="s">
-        <v>9</v>
-      </c>
-      <c r="G224" s="37" t="s">
-        <v>10</v>
-      </c>
-      <c r="H224" s="32" t="s">
+      <c r="B224" s="24" t="s">
+        <v>9</v>
+      </c>
+      <c r="C224" s="24" t="s">
+        <v>9</v>
+      </c>
+      <c r="D224" s="24" t="s">
+        <v>9</v>
+      </c>
+      <c r="E224" s="24" t="s">
+        <v>9</v>
+      </c>
+      <c r="F224" s="24" t="s">
+        <v>9</v>
+      </c>
+      <c r="G224" s="29" t="s">
+        <v>10</v>
+      </c>
+      <c r="H224" s="24" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="225" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A225" s="30" t="s">
+      <c r="A225" s="23" t="s">
         <v>23</v>
       </c>
-      <c r="B225" s="32" t="s">
-        <v>9</v>
-      </c>
-      <c r="C225" s="32" t="s">
-        <v>9</v>
-      </c>
-      <c r="D225" s="32" t="s">
-        <v>9</v>
-      </c>
-      <c r="E225" s="32" t="s">
-        <v>9</v>
-      </c>
-      <c r="F225" s="36" t="s">
+      <c r="B225" s="24" t="s">
+        <v>9</v>
+      </c>
+      <c r="C225" s="24" t="s">
+        <v>9</v>
+      </c>
+      <c r="D225" s="24" t="s">
+        <v>9</v>
+      </c>
+      <c r="E225" s="24" t="s">
+        <v>9</v>
+      </c>
+      <c r="F225" s="28" t="s">
         <v>40</v>
       </c>
-      <c r="G225" s="36" t="s">
+      <c r="G225" s="28" t="s">
         <v>40</v>
       </c>
-      <c r="H225" s="36" t="s">
+      <c r="H225" s="28" t="s">
         <v>40</v>
       </c>
     </row>
-    <row r="226" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A226" s="30" t="s">
+    <row r="226" spans="1:8" ht="46.8" x14ac:dyDescent="0.3">
+      <c r="A226" s="23" t="s">
+        <v>17</v>
+      </c>
+      <c r="B226" s="24" t="s">
+        <v>9</v>
+      </c>
+      <c r="C226" s="24" t="s">
+        <v>36</v>
+      </c>
+      <c r="D226" s="24" t="s">
+        <v>37</v>
+      </c>
+      <c r="E226" s="24" t="s">
+        <v>38</v>
+      </c>
+      <c r="F226" s="24" t="s">
+        <v>9</v>
+      </c>
+      <c r="G226" s="24" t="s">
+        <v>11</v>
+      </c>
+      <c r="H226" s="29" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="227" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A227" s="23" t="s">
+        <v>12</v>
+      </c>
+      <c r="B227" s="24" t="s">
+        <v>11</v>
+      </c>
+      <c r="C227" s="24" t="s">
+        <v>11</v>
+      </c>
+      <c r="D227" s="24" t="s">
+        <v>11</v>
+      </c>
+      <c r="E227" s="24" t="s">
+        <v>11</v>
+      </c>
+      <c r="F227" s="24" t="s">
+        <v>11</v>
+      </c>
+      <c r="G227" s="29" t="s">
+        <v>10</v>
+      </c>
+      <c r="H227" s="24" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="228" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A228" s="23" t="s">
+        <v>8</v>
+      </c>
+      <c r="B228" s="24" t="s">
+        <v>11</v>
+      </c>
+      <c r="C228" s="24" t="s">
+        <v>11</v>
+      </c>
+      <c r="D228" s="24" t="s">
+        <v>11</v>
+      </c>
+      <c r="E228" s="24" t="s">
+        <v>11</v>
+      </c>
+      <c r="F228" s="24" t="s">
+        <v>11</v>
+      </c>
+      <c r="G228" s="25" t="s">
+        <v>19</v>
+      </c>
+      <c r="H228" s="25" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="229" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A229" s="23" t="s">
+        <v>20</v>
+      </c>
+      <c r="B229" s="24" t="s">
+        <v>11</v>
+      </c>
+      <c r="C229" s="24" t="s">
+        <v>11</v>
+      </c>
+      <c r="D229" s="24" t="s">
+        <v>11</v>
+      </c>
+      <c r="E229" s="24" t="s">
+        <v>11</v>
+      </c>
+      <c r="F229" s="32" t="s">
+        <v>35</v>
+      </c>
+      <c r="G229" s="29" t="s">
+        <v>10</v>
+      </c>
+      <c r="H229" s="24" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="230" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A230" s="23" t="s">
+        <v>14</v>
+      </c>
+      <c r="B230" s="40" t="s">
+        <v>13</v>
+      </c>
+      <c r="C230" s="40" t="s">
+        <v>13</v>
+      </c>
+      <c r="D230" s="40" t="s">
+        <v>13</v>
+      </c>
+      <c r="E230" s="40" t="s">
+        <v>13</v>
+      </c>
+      <c r="F230" s="40" t="s">
+        <v>13</v>
+      </c>
+      <c r="G230" s="40" t="s">
+        <v>13</v>
+      </c>
+      <c r="H230" s="41" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="231" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A231" s="39" t="s">
         <v>18</v>
       </c>
-      <c r="B226" s="33" t="s">
+      <c r="B231" s="42" t="s">
         <v>19</v>
       </c>
-      <c r="C226" s="32" t="s">
-        <v>9</v>
-      </c>
-      <c r="D226" s="32" t="s">
-        <v>9</v>
-      </c>
-      <c r="E226" s="32" t="s">
-        <v>9</v>
-      </c>
-      <c r="F226" s="32" t="s">
-        <v>9</v>
-      </c>
-      <c r="G226" s="32" t="s">
+      <c r="C231" s="40" t="s">
+        <v>11</v>
+      </c>
+      <c r="D231" s="40" t="s">
+        <v>11</v>
+      </c>
+      <c r="E231" s="40" t="s">
+        <v>11</v>
+      </c>
+      <c r="F231" s="40" t="s">
+        <v>11</v>
+      </c>
+      <c r="G231" s="40" t="s">
         <v>26</v>
       </c>
-      <c r="H226" s="31" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="227" spans="1:8" ht="46.8" x14ac:dyDescent="0.3">
-      <c r="A227" s="30" t="s">
-        <v>17</v>
-      </c>
-      <c r="B227" s="32" t="s">
-        <v>9</v>
-      </c>
-      <c r="C227" s="32" t="s">
-        <v>36</v>
-      </c>
-      <c r="D227" s="32" t="s">
-        <v>37</v>
-      </c>
-      <c r="E227" s="32" t="s">
-        <v>38</v>
-      </c>
-      <c r="F227" s="32" t="s">
-        <v>9</v>
-      </c>
-      <c r="G227" s="32" t="s">
-        <v>11</v>
-      </c>
-      <c r="H227" s="37" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="228" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A228" s="30" t="s">
-        <v>12</v>
-      </c>
-      <c r="B228" s="32" t="s">
-        <v>11</v>
-      </c>
-      <c r="C228" s="32" t="s">
-        <v>11</v>
-      </c>
-      <c r="D228" s="32" t="s">
-        <v>11</v>
-      </c>
-      <c r="E228" s="32" t="s">
-        <v>11</v>
-      </c>
-      <c r="F228" s="32" t="s">
-        <v>11</v>
-      </c>
-      <c r="G228" s="37" t="s">
-        <v>10</v>
-      </c>
-      <c r="H228" s="32" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="229" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A229" s="30" t="s">
-        <v>8</v>
-      </c>
-      <c r="B229" s="32" t="s">
-        <v>11</v>
-      </c>
-      <c r="C229" s="32" t="s">
-        <v>11</v>
-      </c>
-      <c r="D229" s="32" t="s">
-        <v>11</v>
-      </c>
-      <c r="E229" s="32" t="s">
-        <v>11</v>
-      </c>
-      <c r="F229" s="32" t="s">
-        <v>11</v>
-      </c>
-      <c r="G229" s="33" t="s">
-        <v>19</v>
-      </c>
-      <c r="H229" s="33" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="230" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A230" s="30" t="s">
-        <v>20</v>
-      </c>
-      <c r="B230" s="32" t="s">
-        <v>11</v>
-      </c>
-      <c r="C230" s="32" t="s">
-        <v>11</v>
-      </c>
-      <c r="D230" s="32" t="s">
-        <v>11</v>
-      </c>
-      <c r="E230" s="32" t="s">
-        <v>11</v>
-      </c>
-      <c r="F230" s="40" t="s">
+      <c r="H231" s="41" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="232" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A232" s="50" t="s">
+        <v>27</v>
+      </c>
+      <c r="B232" s="45" t="s">
+        <v>31</v>
+      </c>
+      <c r="C232" s="45" t="s">
+        <v>31</v>
+      </c>
+      <c r="D232" s="45" t="s">
+        <v>31</v>
+      </c>
+      <c r="E232" s="45" t="s">
+        <v>31</v>
+      </c>
+      <c r="F232" s="51" t="s">
         <v>35</v>
       </c>
-      <c r="G230" s="37" t="s">
-        <v>10</v>
-      </c>
-      <c r="H230" s="32" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="231" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A231" s="30" t="s">
-        <v>14</v>
-      </c>
-      <c r="B231" s="32" t="s">
-        <v>13</v>
-      </c>
-      <c r="C231" s="32" t="s">
-        <v>13</v>
-      </c>
-      <c r="D231" s="32" t="s">
-        <v>13</v>
-      </c>
-      <c r="E231" s="32" t="s">
-        <v>13</v>
-      </c>
-      <c r="F231" s="32" t="s">
-        <v>13</v>
-      </c>
-      <c r="G231" s="32" t="s">
-        <v>13</v>
-      </c>
-      <c r="H231" s="37" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="232" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A232" s="35" t="s">
-        <v>27</v>
-      </c>
-      <c r="B232" s="32" t="s">
+      <c r="G232" s="52" t="s">
+        <v>10</v>
+      </c>
+      <c r="H232" s="29" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="233" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A233" s="23" t="s">
+        <v>28</v>
+      </c>
+      <c r="B233" s="24" t="s">
         <v>31</v>
       </c>
-      <c r="C232" s="32" t="s">
+      <c r="C233" s="24" t="s">
         <v>31</v>
       </c>
-      <c r="D232" s="32" t="s">
+      <c r="D233" s="24" t="s">
         <v>31</v>
       </c>
-      <c r="E232" s="32" t="s">
+      <c r="E233" s="24" t="s">
         <v>31</v>
       </c>
-      <c r="F232" s="40" t="s">
-        <v>35</v>
-      </c>
-      <c r="G232" s="37" t="s">
-        <v>10</v>
-      </c>
-      <c r="H232" s="37" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="233" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A233" s="30" t="s">
-        <v>28</v>
-      </c>
-      <c r="B233" s="32" t="s">
+      <c r="F233" s="24" t="s">
         <v>31</v>
       </c>
-      <c r="C233" s="32" t="s">
-        <v>31</v>
-      </c>
-      <c r="D233" s="32" t="s">
-        <v>31</v>
-      </c>
-      <c r="E233" s="32" t="s">
-        <v>31</v>
-      </c>
-      <c r="F233" s="32" t="s">
-        <v>31</v>
-      </c>
-      <c r="G233" s="38" t="s">
+      <c r="G233" s="30" t="s">
         <v>34</v>
       </c>
-      <c r="H233" s="38" t="s">
+      <c r="H233" s="47" t="s">
         <v>34</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="17">
-    <mergeCell ref="A1:A2"/>
-    <mergeCell ref="A14:A15"/>
-    <mergeCell ref="A27:A28"/>
-    <mergeCell ref="A40:A41"/>
-    <mergeCell ref="A53:A54"/>
+    <mergeCell ref="A220:A221"/>
+    <mergeCell ref="A205:A206"/>
     <mergeCell ref="A190:A191"/>
     <mergeCell ref="G84:H84"/>
     <mergeCell ref="A66:A67"/>
@@ -6824,8 +6895,11 @@
     <mergeCell ref="A175:A176"/>
     <mergeCell ref="A160:A161"/>
     <mergeCell ref="A145:A146"/>
-    <mergeCell ref="A220:A221"/>
-    <mergeCell ref="A205:A206"/>
+    <mergeCell ref="A1:A2"/>
+    <mergeCell ref="A14:A15"/>
+    <mergeCell ref="A27:A28"/>
+    <mergeCell ref="A40:A41"/>
+    <mergeCell ref="A53:A54"/>
   </mergeCells>
   <phoneticPr fontId="7" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -6834,6 +6908,26 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="9d4e7416-6feb-444a-9f0d-6e119e2a4ded">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="ab20b492-db1c-4b70-84db-283da62d5dcb" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100A49D20B196870C459C080BD3A88F41F5" ma:contentTypeVersion="12" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="c891d3af3c5d8789d4a1386f5525110a">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="9d4e7416-6feb-444a-9f0d-6e119e2a4ded" xmlns:ns3="ab20b492-db1c-4b70-84db-283da62d5dcb" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="a2d778173b158e0f4887e6c1a7be78b9" ns2:_="" ns3:_="">
     <xsd:import namespace="9d4e7416-6feb-444a-9f0d-6e119e2a4ded"/>
@@ -7034,27 +7128,26 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="9d4e7416-6feb-444a-9f0d-6e119e2a4ded">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="ab20b492-db1c-4b70-84db-283da62d5dcb" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{3E90FB8C-E259-434B-8A97-2530AD5FA4BD}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{3E7BE3CC-8834-4B2B-B0A5-EDC239DF005F}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="9d4e7416-6feb-444a-9f0d-6e119e2a4ded"/>
+    <ds:schemaRef ds:uri="ab20b492-db1c-4b70-84db-283da62d5dcb"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9D90F563-717D-4F15-9FD2-892B1218D415}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -7071,23 +7164,4 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{3E7BE3CC-8834-4B2B-B0A5-EDC239DF005F}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="9d4e7416-6feb-444a-9f0d-6e119e2a4ded"/>
-    <ds:schemaRef ds:uri="ab20b492-db1c-4b70-84db-283da62d5dcb"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{3E90FB8C-E259-434B-8A97-2530AD5FA4BD}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
Actualizacion automatica de datos - jue 06/08/2026 12:04:28,88
</commit_message>
<xml_diff>
--- a/Horario/Horario 2026.xlsx
+++ b/Horario/Horario 2026.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://virtualsoftserv-my.sharepoint.com/personal/maria_sanchez_virtualsoft_tech/Documents/Indicadores y Pagina WEB/Horario/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="10" documentId="6_{6E17BD36-3E42-42F2-8AFD-92DB165A9BC2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{97FBA5BF-47C2-406C-AC55-13C51F6A0428}"/>
+  <xr:revisionPtr revIDLastSave="12" documentId="6_{6E17BD36-3E42-42F2-8AFD-92DB165A9BC2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{8C241B4B-405A-4B29-A08D-1D78DC68F8ED}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{9AAEFA76-0198-46F6-BBF5-EADAB38A6758}"/>
   </bookViews>
@@ -471,7 +471,7 @@
     <xf numFmtId="43" fontId="13" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="53">
+  <cellXfs count="52">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="16" fontId="2" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -549,24 +549,6 @@
     <xf numFmtId="0" fontId="5" fillId="11" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="9" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="9" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="14" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
@@ -581,9 +563,6 @@
     </xf>
     <xf numFmtId="0" fontId="17" fillId="10" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="11" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -607,6 +586,24 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="9" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="9" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -681,10 +678,6 @@
     <xdr:clientData/>
   </xdr:twoCellAnchor>
 </xdr:wsDr>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1009,14 +1002,15 @@
   <cols>
     <col min="1" max="1" width="20.109375" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="17" bestFit="1" customWidth="1"/>
-    <col min="3" max="4" width="12.44140625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="15.88671875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="12.44140625" bestFit="1" customWidth="1"/>
     <col min="5" max="7" width="17" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="15.5546875" bestFit="1" customWidth="1"/>
     <col min="9" max="15" width="12.44140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:15" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A1" s="33" t="s">
+      <c r="A1" s="50" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="1">
@@ -1063,7 +1057,7 @@
       </c>
     </row>
     <row r="2" spans="1:15" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A2" s="34"/>
+      <c r="A2" s="51"/>
       <c r="B2" s="2" t="s">
         <v>1</v>
       </c>
@@ -1578,7 +1572,7 @@
       </c>
     </row>
     <row r="14" spans="1:15" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A14" s="33" t="s">
+      <c r="A14" s="50" t="s">
         <v>0</v>
       </c>
       <c r="B14" s="1">
@@ -1604,7 +1598,7 @@
       </c>
     </row>
     <row r="15" spans="1:15" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A15" s="34"/>
+      <c r="A15" s="51"/>
       <c r="B15" s="2" t="s">
         <v>1</v>
       </c>
@@ -1888,7 +1882,7 @@
       </c>
     </row>
     <row r="27" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A27" s="33" t="s">
+      <c r="A27" s="50" t="s">
         <v>0</v>
       </c>
       <c r="B27" s="1">
@@ -1914,7 +1908,7 @@
       </c>
     </row>
     <row r="28" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A28" s="34"/>
+      <c r="A28" s="51"/>
       <c r="B28" s="2" t="s">
         <v>1</v>
       </c>
@@ -2198,7 +2192,7 @@
       </c>
     </row>
     <row r="40" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A40" s="35" t="s">
+      <c r="A40" s="47" t="s">
         <v>0</v>
       </c>
       <c r="B40" s="1">
@@ -2224,7 +2218,7 @@
       </c>
     </row>
     <row r="41" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A41" s="35"/>
+      <c r="A41" s="47"/>
       <c r="B41" s="2" t="s">
         <v>1</v>
       </c>
@@ -2508,7 +2502,7 @@
       </c>
     </row>
     <row r="53" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A53" s="35" t="s">
+      <c r="A53" s="47" t="s">
         <v>0</v>
       </c>
       <c r="B53" s="1">
@@ -2534,7 +2528,7 @@
       </c>
     </row>
     <row r="54" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A54" s="35"/>
+      <c r="A54" s="47"/>
       <c r="B54" s="2" t="s">
         <v>1</v>
       </c>
@@ -2818,7 +2812,7 @@
       </c>
     </row>
     <row r="66" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A66" s="35" t="s">
+      <c r="A66" s="47" t="s">
         <v>0</v>
       </c>
       <c r="B66" s="1">
@@ -2844,7 +2838,7 @@
       </c>
     </row>
     <row r="67" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A67" s="35"/>
+      <c r="A67" s="47"/>
       <c r="B67" s="2" t="s">
         <v>1</v>
       </c>
@@ -3128,7 +3122,7 @@
       </c>
     </row>
     <row r="79" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A79" s="35" t="s">
+      <c r="A79" s="47" t="s">
         <v>0</v>
       </c>
       <c r="B79" s="1">
@@ -3154,7 +3148,7 @@
       </c>
     </row>
     <row r="80" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A80" s="35"/>
+      <c r="A80" s="47"/>
       <c r="B80" s="2" t="s">
         <v>1</v>
       </c>
@@ -3274,8 +3268,8 @@
       <c r="F84" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="G84" s="36"/>
-      <c r="H84" s="37"/>
+      <c r="G84" s="48"/>
+      <c r="H84" s="49"/>
     </row>
     <row r="85" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A85" s="3" t="s">
@@ -3434,7 +3428,7 @@
       </c>
     </row>
     <row r="92" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A92" s="35" t="s">
+      <c r="A92" s="47" t="s">
         <v>0</v>
       </c>
       <c r="B92" s="1">
@@ -3460,7 +3454,7 @@
       </c>
     </row>
     <row r="93" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A93" s="35"/>
+      <c r="A93" s="47"/>
       <c r="B93" s="2" t="s">
         <v>1</v>
       </c>
@@ -3718,7 +3712,7 @@
       </c>
     </row>
     <row r="104" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A104" s="35" t="s">
+      <c r="A104" s="47" t="s">
         <v>0</v>
       </c>
       <c r="B104" s="1">
@@ -3744,7 +3738,7 @@
       </c>
     </row>
     <row r="105" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A105" s="35"/>
+      <c r="A105" s="47"/>
       <c r="B105" s="2" t="s">
         <v>1</v>
       </c>
@@ -4002,7 +3996,7 @@
       </c>
     </row>
     <row r="116" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A116" s="35" t="s">
+      <c r="A116" s="47" t="s">
         <v>0</v>
       </c>
       <c r="B116" s="1">
@@ -4028,7 +4022,7 @@
       </c>
     </row>
     <row r="117" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A117" s="35"/>
+      <c r="A117" s="47"/>
       <c r="B117" s="2" t="s">
         <v>1</v>
       </c>
@@ -4700,7 +4694,7 @@
       </c>
     </row>
     <row r="145" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A145" s="35" t="s">
+      <c r="A145" s="47" t="s">
         <v>0</v>
       </c>
       <c r="B145" s="1">
@@ -4726,7 +4720,7 @@
       </c>
     </row>
     <row r="146" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A146" s="35"/>
+      <c r="A146" s="47"/>
       <c r="B146" s="2" t="s">
         <v>1</v>
       </c>
@@ -5062,7 +5056,7 @@
       </c>
     </row>
     <row r="160" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A160" s="35" t="s">
+      <c r="A160" s="47" t="s">
         <v>0</v>
       </c>
       <c r="B160" s="1">
@@ -5088,7 +5082,7 @@
       </c>
     </row>
     <row r="161" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A161" s="35"/>
+      <c r="A161" s="47"/>
       <c r="B161" s="2" t="s">
         <v>1</v>
       </c>
@@ -5424,7 +5418,7 @@
       </c>
     </row>
     <row r="175" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A175" s="35" t="s">
+      <c r="A175" s="47" t="s">
         <v>0</v>
       </c>
       <c r="B175" s="1">
@@ -5450,7 +5444,7 @@
       </c>
     </row>
     <row r="176" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A176" s="35"/>
+      <c r="A176" s="47"/>
       <c r="B176" s="2" t="s">
         <v>1</v>
       </c>
@@ -5786,7 +5780,7 @@
       </c>
     </row>
     <row r="190" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A190" s="35" t="s">
+      <c r="A190" s="47" t="s">
         <v>0</v>
       </c>
       <c r="B190" s="1">
@@ -5812,7 +5806,7 @@
       </c>
     </row>
     <row r="191" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A191" s="35"/>
+      <c r="A191" s="47"/>
       <c r="B191" s="2" t="s">
         <v>1</v>
       </c>
@@ -6148,7 +6142,7 @@
       </c>
     </row>
     <row r="205" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A205" s="38" t="s">
+      <c r="A205" s="46" t="s">
         <v>0</v>
       </c>
       <c r="B205" s="26">
@@ -6174,7 +6168,7 @@
       </c>
     </row>
     <row r="206" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A206" s="38"/>
+      <c r="A206" s="46"/>
       <c r="B206" s="23" t="s">
         <v>1</v>
       </c>
@@ -6447,10 +6441,10 @@
       <c r="E216" s="24" t="s">
         <v>13</v>
       </c>
-      <c r="F216" s="45" t="s">
-        <v>9</v>
-      </c>
-      <c r="G216" s="45" t="s">
+      <c r="F216" s="38" t="s">
+        <v>9</v>
+      </c>
+      <c r="G216" s="38" t="s">
         <v>11</v>
       </c>
       <c r="H216" s="29" t="s">
@@ -6470,16 +6464,16 @@
       <c r="D217" s="24" t="s">
         <v>31</v>
       </c>
-      <c r="E217" s="46" t="s">
+      <c r="E217" s="39" t="s">
         <v>31</v>
       </c>
-      <c r="F217" s="43" t="s">
+      <c r="F217" s="37" t="s">
         <v>34</v>
       </c>
       <c r="G217" s="30" t="s">
         <v>34</v>
       </c>
-      <c r="H217" s="47" t="s">
+      <c r="H217" s="40" t="s">
         <v>34</v>
       </c>
     </row>
@@ -6496,7 +6490,7 @@
       <c r="D218" s="25" t="s">
         <v>19</v>
       </c>
-      <c r="E218" s="48" t="s">
+      <c r="E218" s="41" t="s">
         <v>19</v>
       </c>
       <c r="F218" s="29" t="s">
@@ -6505,7 +6499,7 @@
       <c r="G218" s="29" t="s">
         <v>10</v>
       </c>
-      <c r="H218" s="49" t="s">
+      <c r="H218" s="42" t="s">
         <v>10</v>
       </c>
     </row>
@@ -6520,7 +6514,7 @@
       <c r="H219" s="22"/>
     </row>
     <row r="220" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A220" s="38" t="s">
+      <c r="A220" s="46" t="s">
         <v>0</v>
       </c>
       <c r="B220" s="26">
@@ -6546,7 +6540,7 @@
       </c>
     </row>
     <row r="221" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A221" s="38"/>
+      <c r="A221" s="46"/>
       <c r="B221" s="23" t="s">
         <v>1</v>
       </c>
@@ -6576,7 +6570,7 @@
       <c r="B222" s="24" t="s">
         <v>9</v>
       </c>
-      <c r="C222" s="44" t="s">
+      <c r="C222" s="32" t="s">
         <v>35</v>
       </c>
       <c r="D222" s="24" t="s">
@@ -6781,74 +6775,74 @@
       <c r="A230" s="23" t="s">
         <v>14</v>
       </c>
-      <c r="B230" s="40" t="s">
-        <v>13</v>
-      </c>
-      <c r="C230" s="40" t="s">
-        <v>13</v>
-      </c>
-      <c r="D230" s="40" t="s">
-        <v>13</v>
-      </c>
-      <c r="E230" s="40" t="s">
-        <v>13</v>
-      </c>
-      <c r="F230" s="40" t="s">
-        <v>13</v>
-      </c>
-      <c r="G230" s="40" t="s">
-        <v>13</v>
-      </c>
-      <c r="H230" s="41" t="s">
+      <c r="B230" s="34" t="s">
+        <v>13</v>
+      </c>
+      <c r="C230" s="34" t="s">
+        <v>13</v>
+      </c>
+      <c r="D230" s="34" t="s">
+        <v>13</v>
+      </c>
+      <c r="E230" s="34" t="s">
+        <v>13</v>
+      </c>
+      <c r="F230" s="34" t="s">
+        <v>13</v>
+      </c>
+      <c r="G230" s="34" t="s">
+        <v>13</v>
+      </c>
+      <c r="H230" s="35" t="s">
         <v>10</v>
       </c>
     </row>
     <row r="231" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A231" s="39" t="s">
+      <c r="A231" s="33" t="s">
         <v>18</v>
       </c>
-      <c r="B231" s="42" t="s">
+      <c r="B231" s="36" t="s">
         <v>19</v>
       </c>
-      <c r="C231" s="40" t="s">
-        <v>11</v>
-      </c>
-      <c r="D231" s="40" t="s">
-        <v>11</v>
-      </c>
-      <c r="E231" s="40" t="s">
-        <v>11</v>
-      </c>
-      <c r="F231" s="40" t="s">
-        <v>11</v>
-      </c>
-      <c r="G231" s="40" t="s">
+      <c r="C231" s="34" t="s">
+        <v>11</v>
+      </c>
+      <c r="D231" s="34" t="s">
+        <v>11</v>
+      </c>
+      <c r="E231" s="34" t="s">
+        <v>11</v>
+      </c>
+      <c r="F231" s="34" t="s">
+        <v>11</v>
+      </c>
+      <c r="G231" s="34" t="s">
         <v>26</v>
       </c>
-      <c r="H231" s="41" t="s">
+      <c r="H231" s="35" t="s">
         <v>10</v>
       </c>
     </row>
     <row r="232" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A232" s="50" t="s">
+      <c r="A232" s="43" t="s">
         <v>27</v>
       </c>
-      <c r="B232" s="45" t="s">
+      <c r="B232" s="38" t="s">
         <v>31</v>
       </c>
-      <c r="C232" s="45" t="s">
+      <c r="C232" s="38" t="s">
         <v>31</v>
       </c>
-      <c r="D232" s="45" t="s">
+      <c r="D232" s="38" t="s">
         <v>31</v>
       </c>
-      <c r="E232" s="45" t="s">
+      <c r="E232" s="38" t="s">
         <v>31</v>
       </c>
-      <c r="F232" s="51" t="s">
+      <c r="F232" s="44" t="s">
         <v>35</v>
       </c>
-      <c r="G232" s="52" t="s">
+      <c r="G232" s="45" t="s">
         <v>10</v>
       </c>
       <c r="H232" s="29" t="s">
@@ -6877,12 +6871,17 @@
       <c r="G233" s="30" t="s">
         <v>34</v>
       </c>
-      <c r="H233" s="47" t="s">
+      <c r="H233" s="40" t="s">
         <v>34</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="17">
+    <mergeCell ref="A1:A2"/>
+    <mergeCell ref="A14:A15"/>
+    <mergeCell ref="A27:A28"/>
+    <mergeCell ref="A40:A41"/>
+    <mergeCell ref="A53:A54"/>
     <mergeCell ref="A220:A221"/>
     <mergeCell ref="A205:A206"/>
     <mergeCell ref="A190:A191"/>
@@ -6895,11 +6894,6 @@
     <mergeCell ref="A175:A176"/>
     <mergeCell ref="A160:A161"/>
     <mergeCell ref="A145:A146"/>
-    <mergeCell ref="A1:A2"/>
-    <mergeCell ref="A14:A15"/>
-    <mergeCell ref="A27:A28"/>
-    <mergeCell ref="A40:A41"/>
-    <mergeCell ref="A53:A54"/>
   </mergeCells>
   <phoneticPr fontId="7" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -6908,26 +6902,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="9d4e7416-6feb-444a-9f0d-6e119e2a4ded">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="ab20b492-db1c-4b70-84db-283da62d5dcb" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100A49D20B196870C459C080BD3A88F41F5" ma:contentTypeVersion="12" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="c891d3af3c5d8789d4a1386f5525110a">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="9d4e7416-6feb-444a-9f0d-6e119e2a4ded" xmlns:ns3="ab20b492-db1c-4b70-84db-283da62d5dcb" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="a2d778173b158e0f4887e6c1a7be78b9" ns2:_="" ns3:_="">
     <xsd:import namespace="9d4e7416-6feb-444a-9f0d-6e119e2a4ded"/>
@@ -7128,10 +7102,41 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="9d4e7416-6feb-444a-9f0d-6e119e2a4ded">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="ab20b492-db1c-4b70-84db-283da62d5dcb" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{3E90FB8C-E259-434B-8A97-2530AD5FA4BD}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9D90F563-717D-4F15-9FD2-892B1218D415}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="9d4e7416-6feb-444a-9f0d-6e119e2a4ded"/>
+    <ds:schemaRef ds:uri="ab20b492-db1c-4b70-84db-283da62d5dcb"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -7148,20 +7153,9 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9D90F563-717D-4F15-9FD2-892B1218D415}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{3E90FB8C-E259-434B-8A97-2530AD5FA4BD}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="9d4e7416-6feb-444a-9f0d-6e119e2a4ded"/>
-    <ds:schemaRef ds:uri="ab20b492-db1c-4b70-84db-283da62d5dcb"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
Actualizacion de datos - mié 19/08/2026 14:13:28,67
</commit_message>
<xml_diff>
--- a/Horario/Horario 2026.xlsx
+++ b/Horario/Horario 2026.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://virtualsoftserv-my.sharepoint.com/personal/maria_sanchez_virtualsoft_tech/Documents/Indicadores y Pagina WEB/Horario/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="14" documentId="6_{6E17BD36-3E42-42F2-8AFD-92DB165A9BC2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{8523CC63-A23F-4D67-B0B7-88F4180EEA8F}"/>
+  <xr:revisionPtr revIDLastSave="15" documentId="6_{6E17BD36-3E42-42F2-8AFD-92DB165A9BC2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{951B51AD-FF0C-4423-AAA0-A9A149B6BDDE}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="5280" windowWidth="23280" windowHeight="12480" xr2:uid="{9AAEFA76-0198-46F6-BBF5-EADAB38A6758}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{9AAEFA76-0198-46F6-BBF5-EADAB38A6758}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1779" uniqueCount="45">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1883" uniqueCount="45">
   <si>
     <t>GESTOR</t>
   </si>
@@ -471,7 +471,7 @@
     <xf numFmtId="43" fontId="13" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="53">
+  <cellXfs count="55">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="16" fontId="2" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -607,6 +607,12 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="16" fontId="2" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1000,7 +1006,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4B1D5CB7-A214-4F9F-A075-10C6E5CC7E55}">
-  <dimension ref="A1:O248"/>
+  <dimension ref="A1:O263"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="20.140625" bestFit="1" customWidth="1"/>
@@ -7240,8 +7246,371 @@
         <v>10</v>
       </c>
     </row>
+    <row r="250" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A250" s="47" t="s">
+        <v>0</v>
+      </c>
+      <c r="B250" s="53">
+        <v>46258</v>
+      </c>
+      <c r="C250" s="53">
+        <v>46259</v>
+      </c>
+      <c r="D250" s="53">
+        <v>46260</v>
+      </c>
+      <c r="E250" s="53">
+        <v>46261</v>
+      </c>
+      <c r="F250" s="53">
+        <v>46262</v>
+      </c>
+      <c r="G250" s="53">
+        <v>46263</v>
+      </c>
+      <c r="H250" s="53">
+        <v>46264</v>
+      </c>
+    </row>
+    <row r="251" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A251" s="47"/>
+      <c r="B251" s="54" t="s">
+        <v>1</v>
+      </c>
+      <c r="C251" s="54" t="s">
+        <v>2</v>
+      </c>
+      <c r="D251" s="54" t="s">
+        <v>3</v>
+      </c>
+      <c r="E251" s="54" t="s">
+        <v>4</v>
+      </c>
+      <c r="F251" s="54" t="s">
+        <v>5</v>
+      </c>
+      <c r="G251" s="54" t="s">
+        <v>6</v>
+      </c>
+      <c r="H251" s="54" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="252" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A252" s="23" t="s">
+        <v>22</v>
+      </c>
+      <c r="B252" s="24" t="s">
+        <v>9</v>
+      </c>
+      <c r="C252" s="24" t="s">
+        <v>9</v>
+      </c>
+      <c r="D252" s="24" t="s">
+        <v>9</v>
+      </c>
+      <c r="E252" s="24" t="s">
+        <v>9</v>
+      </c>
+      <c r="F252" s="24" t="s">
+        <v>9</v>
+      </c>
+      <c r="G252" s="24" t="s">
+        <v>9</v>
+      </c>
+      <c r="H252" s="29" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="253" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A253" s="23" t="s">
+        <v>29</v>
+      </c>
+      <c r="B253" s="24" t="s">
+        <v>9</v>
+      </c>
+      <c r="C253" s="24" t="s">
+        <v>9</v>
+      </c>
+      <c r="D253" s="24" t="s">
+        <v>9</v>
+      </c>
+      <c r="E253" s="24" t="s">
+        <v>9</v>
+      </c>
+      <c r="F253" s="24" t="s">
+        <v>9</v>
+      </c>
+      <c r="G253" s="29" t="s">
+        <v>10</v>
+      </c>
+      <c r="H253" s="24" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="254" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A254" s="23" t="s">
+        <v>21</v>
+      </c>
+      <c r="B254" s="24" t="s">
+        <v>9</v>
+      </c>
+      <c r="C254" s="24" t="s">
+        <v>9</v>
+      </c>
+      <c r="D254" s="24" t="s">
+        <v>9</v>
+      </c>
+      <c r="E254" s="24" t="s">
+        <v>9</v>
+      </c>
+      <c r="F254" s="24" t="s">
+        <v>9</v>
+      </c>
+      <c r="G254" s="29" t="s">
+        <v>10</v>
+      </c>
+      <c r="H254" s="24" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="255" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A255" s="23" t="s">
+        <v>20</v>
+      </c>
+      <c r="B255" s="24" t="s">
+        <v>9</v>
+      </c>
+      <c r="C255" s="24" t="s">
+        <v>9</v>
+      </c>
+      <c r="D255" s="24" t="s">
+        <v>9</v>
+      </c>
+      <c r="E255" s="24" t="s">
+        <v>9</v>
+      </c>
+      <c r="F255" s="24" t="s">
+        <v>9</v>
+      </c>
+      <c r="G255" s="29" t="s">
+        <v>10</v>
+      </c>
+      <c r="H255" s="24" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="256" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A256" s="23" t="s">
+        <v>23</v>
+      </c>
+      <c r="B256" s="24" t="s">
+        <v>9</v>
+      </c>
+      <c r="C256" s="24" t="s">
+        <v>9</v>
+      </c>
+      <c r="D256" s="24" t="s">
+        <v>9</v>
+      </c>
+      <c r="E256" s="24" t="s">
+        <v>9</v>
+      </c>
+      <c r="F256" s="24" t="s">
+        <v>9</v>
+      </c>
+      <c r="G256" s="24" t="s">
+        <v>11</v>
+      </c>
+      <c r="H256" s="29" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="257" spans="1:8" ht="31.5" x14ac:dyDescent="0.25">
+      <c r="A257" s="23" t="s">
+        <v>12</v>
+      </c>
+      <c r="B257" s="24" t="s">
+        <v>39</v>
+      </c>
+      <c r="C257" s="24" t="s">
+        <v>42</v>
+      </c>
+      <c r="D257" s="24" t="s">
+        <v>41</v>
+      </c>
+      <c r="E257" s="24" t="s">
+        <v>41</v>
+      </c>
+      <c r="F257" s="24" t="s">
+        <v>9</v>
+      </c>
+      <c r="G257" s="29" t="s">
+        <v>10</v>
+      </c>
+      <c r="H257" s="24" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="258" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A258" s="23" t="s">
+        <v>18</v>
+      </c>
+      <c r="B258" s="24" t="s">
+        <v>9</v>
+      </c>
+      <c r="C258" s="24" t="s">
+        <v>11</v>
+      </c>
+      <c r="D258" s="24" t="s">
+        <v>11</v>
+      </c>
+      <c r="E258" s="24" t="s">
+        <v>11</v>
+      </c>
+      <c r="F258" s="24" t="s">
+        <v>11</v>
+      </c>
+      <c r="G258" s="24" t="s">
+        <v>11</v>
+      </c>
+      <c r="H258" s="29" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="259" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A259" s="23" t="s">
+        <v>14</v>
+      </c>
+      <c r="B259" s="24" t="s">
+        <v>11</v>
+      </c>
+      <c r="C259" s="24" t="s">
+        <v>11</v>
+      </c>
+      <c r="D259" s="24" t="s">
+        <v>11</v>
+      </c>
+      <c r="E259" s="24" t="s">
+        <v>11</v>
+      </c>
+      <c r="F259" s="24" t="s">
+        <v>11</v>
+      </c>
+      <c r="G259" s="24" t="s">
+        <v>9</v>
+      </c>
+      <c r="H259" s="29" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="260" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A260" s="23" t="s">
+        <v>8</v>
+      </c>
+      <c r="B260" s="24" t="s">
+        <v>11</v>
+      </c>
+      <c r="C260" s="24" t="s">
+        <v>11</v>
+      </c>
+      <c r="D260" s="24" t="s">
+        <v>11</v>
+      </c>
+      <c r="E260" s="24" t="s">
+        <v>11</v>
+      </c>
+      <c r="F260" s="24" t="s">
+        <v>11</v>
+      </c>
+      <c r="G260" s="29" t="s">
+        <v>10</v>
+      </c>
+      <c r="H260" s="24" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="261" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A261" s="23" t="s">
+        <v>17</v>
+      </c>
+      <c r="B261" s="24" t="s">
+        <v>13</v>
+      </c>
+      <c r="C261" s="24" t="s">
+        <v>13</v>
+      </c>
+      <c r="D261" s="24" t="s">
+        <v>13</v>
+      </c>
+      <c r="E261" s="24" t="s">
+        <v>13</v>
+      </c>
+      <c r="F261" s="24" t="s">
+        <v>13</v>
+      </c>
+      <c r="G261" s="24" t="s">
+        <v>13</v>
+      </c>
+      <c r="H261" s="29" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="262" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A262" s="44" t="s">
+        <v>27</v>
+      </c>
+      <c r="B262" s="24" t="s">
+        <v>31</v>
+      </c>
+      <c r="C262" s="24" t="s">
+        <v>31</v>
+      </c>
+      <c r="D262" s="24" t="s">
+        <v>31</v>
+      </c>
+      <c r="E262" s="24" t="s">
+        <v>31</v>
+      </c>
+      <c r="F262" s="24" t="s">
+        <v>31</v>
+      </c>
+      <c r="G262" s="30" t="s">
+        <v>34</v>
+      </c>
+      <c r="H262" s="41" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="263" spans="1:8" ht="31.5" x14ac:dyDescent="0.25">
+      <c r="A263" s="23" t="s">
+        <v>28</v>
+      </c>
+      <c r="B263" s="28" t="s">
+        <v>40</v>
+      </c>
+      <c r="C263" s="28" t="s">
+        <v>40</v>
+      </c>
+      <c r="D263" s="28" t="s">
+        <v>40</v>
+      </c>
+      <c r="E263" s="28" t="s">
+        <v>40</v>
+      </c>
+      <c r="F263" s="28" t="s">
+        <v>40</v>
+      </c>
+      <c r="G263" s="28" t="s">
+        <v>40</v>
+      </c>
+      <c r="H263" s="28" t="s">
+        <v>40</v>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="18">
+  <mergeCells count="19">
+    <mergeCell ref="A250:A251"/>
     <mergeCell ref="A1:A2"/>
     <mergeCell ref="A14:A15"/>
     <mergeCell ref="A27:A28"/>

</xml_diff>